<commit_message>
chore: scrape update — 137 releases [2026-03-15 06:55 UTC]
</commit_message>
<xml_diff>
--- a/reports/sneaker_releases.xlsx
+++ b/reports/sneaker_releases.xlsx
@@ -1104,7 +1104,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  06:53 AM</t>
+          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  06:55 AM</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="53" t="inlineStr">
         <is>
-          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  06:53 AM</t>
+          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  06:55 AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: scrape update — 137 releases [2026-03-15 06:56 UTC]
</commit_message>
<xml_diff>
--- a/reports/sneaker_releases.xlsx
+++ b/reports/sneaker_releases.xlsx
@@ -569,7 +569,7 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1104,7 +1104,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  06:55 AM</t>
+          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  06:56 AM</t>
         </is>
       </c>
     </row>
@@ -1993,12 +1993,12 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>adidas Has More FIFA Footwear Coming - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Will Patta Release The Next Air Max 1 “Waves” Before March Ends? - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
@@ -2028,19 +2028,19 @@
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE9MVVR4Nk1tYWMtS0ZDMUd0MzhaU0hZU3NBR3dra3B6ZERxVWdscXEzeUhhdTh6dTY1NmU4SXo5R25nYjUtcklpbWo0NFJWUVpZYWZtMDhNTDNZYUd1NGM1cU1Fcm1YdEczMFE0VWNwTGNueGxSZEQ2etIBeEFVX3lxTE9MVVR4Nk1tYWMtS0ZDMUd0MzhaU0hZU3NBR3dra3B6ZERxVWdscXEzeUhhdTh6dTY1NmU4SXo5R25nYjUtcklpbWo0NFJWUVpZYWZtMDhNTDNZYUd1NGM1cU1Fcm1YdEczMFE0VWNwTGNueGxSZEQ2eg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQVFczeDhmeUxySXN3a3VkVE4zeXlnV2dHNXpBc0lWd2dNay00WU1ncHJqWUs3SE9YQ092Mzd3a19JekVCYmYzckhGYl9hU2tTai1CeFZQVU5Qb3JtVWpUNEVYNnJNWFFzZVZrZUZNVGdDZ3JLT0p6RDhmUm80Qi1OY3VhZEFNRGQxRnZKUXFOT2c5eUxLQjZpQdIBmAFBVV95cUxQVFczeDhmeUxySXN3a3VkVE4zeXlnV2dHNXpBc0lWd2dNay00WU1ncHJqWUs3SE9YQ092Mzd3a19JekVCYmYzckhGYl9hU2tTai1CeFZQVU5Qb3JtVWpUNEVYNnJNWFFzZVZrZUZNVGdDZ3JLT0p6RDhmUm80Qi1OY3VhZEFNRGQxRnZKUXFOT2c5eUxLQjZpQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Will Patta Release The Next Air Max 1 “Waves” Before March Ends? - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B24" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The Air Jordan 3 RM Prepares For Takeoff With “Old Royal” Accents - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C24" s="27" t="inlineStr">
@@ -2048,9 +2048,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D24" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E24" s="17" t="inlineStr">
@@ -2058,31 +2058,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F24" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G24" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQVFczeDhmeUxySXN3a3VkVE4zeXlnV2dHNXpBc0lWd2dNay00WU1ncHJqWUs3SE9YQ092Mzd3a19JekVCYmYzckhGYl9hU2tTai1CeFZQVU5Qb3JtVWpUNEVYNnJNWFFzZVZrZUZNVGdDZ3JLT0p6RDhmUm80Qi1OY3VhZEFNRGQxRnZKUXFOT2c5eUxLQjZpQdIBmAFBVV95cUxQVFczeDhmeUxySXN3a3VkVE4zeXlnV2dHNXpBc0lWd2dNay00WU1ncHJqWUs3SE9YQ092Mzd3a19JekVCYmYzckhGYl9hU2tTai1CeFZQVU5Qb3JtVWpUNEVYNnJNWFFzZVZrZUZNVGdDZ3JLT0p6RDhmUm80Qi1OY3VhZEFNRGQxRnZKUXFOT2c5eUxLQjZpQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNem5hM1J4ZXVPY2pnUnFIaDZ4cXQ0ZzRUcHNYZGNjNWh0OXJSenhSVlNjVk5nV0lUMDA2aWIzdFNsWFJHc0ZSX09CamRBNlA1aGxINFdOc2RIbDdfeEtHUzA5YVpGMjI3RWRpZTFhUkp6SjJYY2JCb29SNnhTd1NNcWhTMUZlUHRNUTFSV2pGUG9tWXFzb3hZUnc0Y3BVLVVEYU440gGjAUFVX3lxTE16bmEzUnhldU9jamdScUhoNnhxdDRnNFRwc1hkY2M1aHQ5clJ6eFJWU2NWTmdXSVQwMDZpYjN0U2xYUkdzRlJfT0JqZEE2UDVobEg0V05zZEhsN194S0dTMDlhWkYyMjdFZGllMWFSSnpKMlhjYkJvb1I2eFN3U01xaFMxRmVQdE1RMVJXakZQb21ZcXNveFlSdzRjcFUtVURhTjg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>The Air Jordan 3 RM Prepares For Takeoff With “Old Royal” Accents - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Goes Into Tuxedo Mode With The Air Force 1 Low “Black Patent” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C25" s="22" t="inlineStr">
@@ -2090,9 +2090,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -2100,26 +2100,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G25" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNem5hM1J4ZXVPY2pnUnFIaDZ4cXQ0ZzRUcHNYZGNjNWh0OXJSenhSVlNjVk5nV0lUMDA2aWIzdFNsWFJHc0ZSX09CamRBNlA1aGxINFdOc2RIbDdfeEtHUzA5YVpGMjI3RWRpZTFhUkp6SjJYY2JCb29SNnhTd1NNcWhTMUZlUHRNUTFSV2pGUG9tWXFzb3hZUnc0Y3BVLVVEYU440gGjAUFVX3lxTE16bmEzUnhldU9jamdScUhoNnhxdDRnNFRwc1hkY2M1aHQ5clJ6eFJWU2NWTmdXSVQwMDZpYjN0U2xYUkdzRlJfT0JqZEE2UDVobEg0V05zZEhsN194S0dTMDlhWkYyMjdFZGllMWFSSnpKMlhjYkJvb1I2eFN3U01xaFMxRmVQdE1RMVJXakZQb21ZcXNveFlSdzRjcFUtVURhTjg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQNTFabi11OXA3QVRDSGk4cXJEc3RneXZGc2NYSXNUUURRaXFteUNTRjc2Y0d2Wm9JajlJRTlldXgtcUpWZEdMbWV5ckhfWVc4UkFwYzYxdDI2WGZlRUpHQklUenU2SUJ5QzYxM1dhcU1JU1lGTXVfX3dmU3g3Um5va3ZzUWp6NVHSAYcBQVVfeXFMUDUxWm4tdTlwN0FUQ0hpOHFyRHN0Z3l2RnNjWElzVFFEUWlxbXlDU0Y3NmNHdlpvSWo5SUU5ZXV4LXFKVmRHTG1leXJIX1lXOFJBcGM2MXQyNlhmZUVKR0JJVHp1NklCeUM2MTNXYXFNSVNZRk11X193ZlN4N1Jub2t2c1FqejVR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Nike Goes Into Tuxedo Mode With The Air Force 1 Low “Black Patent” - Sneaker News</t>
+          <t>The Nike Mind 001 And 002 Restock On March 19th - Sneaker News</t>
         </is>
       </c>
       <c r="B26" s="35" t="inlineStr">
@@ -2154,14 +2154,14 @@
       </c>
       <c r="H26" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQNTFabi11OXA3QVRDSGk4cXJEc3RneXZGc2NYSXNUUURRaXFteUNTRjc2Y0d2Wm9JajlJRTlldXgtcUpWZEdMbWV5ckhfWVc4UkFwYzYxdDI2WGZlRUpHQklUenU2SUJ5QzYxM1dhcU1JU1lGTXVfX3dmU3g3Um5va3ZzUWp6NVHSAYcBQVVfeXFMUDUxWm4tdTlwN0FUQ0hpOHFyRHN0Z3l2RnNjWElzVFFEUWlxbXlDU0Y3NmNHdlpvSWo5SUU5ZXV4LXFKVmRHTG1leXJIX1lXOFJBcGM2MXQyNlhmZUVKR0JJVHp1NklCeUM2MTNXYXFNSVNZRk11X193ZlN4N1Jub2t2c1FqejVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBuOURoZ1ZOOU5tN0hSdnlLR2djdHVXY2R4eHdLV2Q1aS1LeXhHOS0wU1BkVDFYcmFhLVhGRk9ndDhvaXpZY1o1Y3pPQWVxbXBJYVJWZU1PM1kxd2FLU0Zma3hsbDRabENQ0gFoQVVfeXFMUG45RGhnVk45Tm03SFJ2eUtHZ2N0dVdjZHh4d0tXZDVpLUt5eEc5LTBTUGRUMVhyYWEtWEZGT2d0OG9pelljWjVjek9BZXFtcElhUlZlTU8zWTF3YUtTRmZreGxsNFpsQ1A?oc=5</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>The Nike Mind 001 And 002 Restock On March 19th - Sneaker News</t>
+          <t>The Nike Vomero Premium Gears Up For Spring In “Volt Tint” - Sneaker News</t>
         </is>
       </c>
       <c r="B27" s="30" t="inlineStr">
@@ -2184,31 +2184,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBuOURoZ1ZOOU5tN0hSdnlLR2djdHVXY2R4eHdLV2Q1aS1LeXhHOS0wU1BkVDFYcmFhLVhGRk9ndDhvaXpZY1o1Y3pPQWVxbXBJYVJWZU1PM1kxd2FLU0Zma3hsbDRabENQ0gFoQVVfeXFMUG45RGhnVk45Tm03SFJ2eUtHZ2N0dVdjZHh4d0tXZDVpLUt5eEc5LTBTUGRUMVhyYWEtWEZGT2d0OG9pelljWjVjek9BZXFtcElhUlZlTU8zWTF3YUtTRmZreGxsNFpsQ1A?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWERiSnZ3N1pzd0xpa2tuT0Z4NXhrQWFWbGYwQl94OUZhZUFLVGQwXzNNV0E3NGlsRDBKOVVLUmo2anl3NUZsYjdqRUdZQXJoUHFLNXdXNC0xYUZWMVJoc2pITk9SeGFJanVvZFF1aHZuSlNpcTFldzk1dnVtX1duOVJfTUEzVVZXdHBwaWQxUDZ6VzM4TFhjTHZyMXNjZTRMTHAyNXp30gGmAUFVX3lxTE1YRGJKdnc3WnN3TGlra25PRng1eGtBYVZsZjBCX3g5RmFlQUtUZDBfM01XQTc0aWxEMEo5VUtSajZqeXc1RmxiN2pFR1lBcmhQcUs1d1c0LTFhRlYxUmhzakhOT1J4YUlqdW9kUXVodm5KU2lxMWV3OTV2dW1fV245Ul9NQTNVVld0cHBpZDFQNnpXMzhMWGNMdnIxc2NlNExMcDI1enc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>The Nike Vomero Premium Gears Up For Spring In “Volt Tint” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The Air Jordan 11 Football Cleat Continues Its Market Rush With “Anthracite” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C28" s="27" t="inlineStr">
@@ -2216,9 +2216,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D28" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>$220</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -2238,14 +2238,14 @@
       </c>
       <c r="H28" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNWERiSnZ3N1pzd0xpa2tuT0Z4NXhrQWFWbGYwQl94OUZhZUFLVGQwXzNNV0E3NGlsRDBKOVVLUmo2anl3NUZsYjdqRUdZQXJoUHFLNXdXNC0xYUZWMVJoc2pITk9SeGFJanVvZFF1aHZuSlNpcTFldzk1dnVtX1duOVJfTUEzVVZXdHBwaWQxUDZ6VzM4TFhjTHZyMXNjZTRMTHAyNXp30gGmAUFVX3lxTE1YRGJKdnc3WnN3TGlra25PRng1eGtBYVZsZjBCX3g5RmFlQUtUZDBfM01XQTc0aWxEMEo5VUtSajZqeXc1RmxiN2pFR1lBcmhQcUs1d1c0LTFhRlYxUmhzakhOT1J4YUlqdW9kUXVodm5KU2lxMWV3OTV2dW1fV245Ul9NQTNVVld0cHBpZDFQNnpXMzhMWGNMdnIxc2NlNExMcDI1enc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNVE9IWE0xQVd6TlNBLXNQak1JQ19RTXY1QTFtQ2RpRXl6bE93cW1MVmhKVDdiTGtORXlTZXlfQTdUeG9jQ2FlUjVxWmtRU2J2blE5eHNDNHNmTmtESzFTMEhLUEU4OTl3S2FTXzQ1a2VtZEdIdUVidXEyLUlkb0N4VlJJcXd2dDk3Z1pLY0phelo2WENmblHSAZYBQVVfeXFMTVRPSFhNMUFXek5TQS1zUGpNSUNfUU12NUExbUNkaUV5emxPd3FtTFZoSlQ3YkxrTkV5U2V5X0E3VHhvY0NhZVI1cVprUVNidm5ROXhzQzRzZk5rREsxUzBIS1BFODk5d0thU180NWtlbWRHSHVFYnVxMi1JZG9DeFZSSXF3dnQ5N2daS2NKYXpaNlhDZm5R?oc=5</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>The Air Jordan 11 Football Cleat Continues Its Market Rush With “Anthracite” - Sneaker News</t>
+          <t>Jordan Brand Adds A Touch Of Class To The Women’s Air Jordan 6 “Sail” - Sneaker News</t>
         </is>
       </c>
       <c r="B29" s="21" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>$220</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -2280,19 +2280,19 @@
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNVE9IWE0xQVd6TlNBLXNQak1JQ19RTXY1QTFtQ2RpRXl6bE93cW1MVmhKVDdiTGtORXlTZXlfQTdUeG9jQ2FlUjVxWmtRU2J2blE5eHNDNHNmTmtESzFTMEhLUEU4OTl3S2FTXzQ1a2VtZEdIdUVidXEyLUlkb0N4VlJJcXd2dDk3Z1pLY0phelo2WENmblHSAZYBQVVfeXFMTVRPSFhNMUFXek5TQS1zUGpNSUNfUU12NUExbUNkaUV5emxPd3FtTFZoSlQ3YkxrTkV5U2V5X0E3VHhvY0NhZVI1cVprUVNidm5ROXhzQzRzZk5rREsxUzBIS1BFODk5d0thU180NWtlbWRHSHVFYnVxMi1JZG9DeFZSSXF3dnQ5N2daS2NKYXpaNlhDZm5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxObzJQTVU5UXgyRzVzWmNHazIwNDk1bm9hQVNXU2ZrRF9mN2RSYVp1WW1xM18taWRJVUVXRW1fTW5UenNpa0pKYzBjejVhN1lOVWswbHUwU2R5Zm0xRzZoVHVsT2NWWWxqVjBuRVVQMV80a0toQUtybFVtR3UtOUhsM0d3Qy1wa0ZJVkdpQklnbFZMRzJvMU55TTFn0gGaAUFVX3lxTE5vMlBNVTlReDJHNXNaY0drMjA0OTVub2FBU1dTZmtEX2Y3ZFJhWnVZbXEzXy1pZElVRVdFbV9NblR6c2lrSkpjMGN6NWE3WU5VazBsdTBTZHlmbTFHNmhUdWxPY1ZZbGpWMG5FVVAxXzRrS2hBS3JsVW1HdS05SGwzR3dDLXBrRklWR2lCSWdsVkxHMm8xTnlNMWc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Jordan Brand Adds A Touch Of Class To The Women’s Air Jordan 6 “Sail” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B30" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>KITH Officially Reveals Their New Balance 991 And 991v2 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C30" s="27" t="inlineStr">
@@ -2300,9 +2300,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
@@ -2310,26 +2310,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F30" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G30" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F30" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G30" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H30" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxObzJQTVU5UXgyRzVzWmNHazIwNDk1bm9hQVNXU2ZrRF9mN2RSYVp1WW1xM18taWRJVUVXRW1fTW5UenNpa0pKYzBjejVhN1lOVWswbHUwU2R5Zm0xRzZoVHVsT2NWWWxqVjBuRVVQMV80a0toQUtybFVtR3UtOUhsM0d3Qy1wa0ZJVkdpQklnbFZMRzJvMU55TTFn0gGaAUFVX3lxTE5vMlBNVTlReDJHNXNaY0drMjA0OTVub2FBU1dTZmtEX2Y3ZFJhWnVZbXEzXy1pZElVRVdFbV9NblR6c2lrSkpjMGN6NWE3WU5VazBsdTBTZHlmbTFHNmhUdWxPY1ZZbGpWMG5FVVAxXzRrS2hBS3JsVW1HdS05SGwzR3dDLXBrRklWR2lCSWdsVkxHMm8xTnlNMWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE91R2xYeTVtOFMwWGVxb2JxSkJxeDZVVkwtamhROHpxbEtlUFVOajlabnNpeW01OGhiMG5IQVVibllFZHFoakVlVUFaWE5GTFdNT1lNSDVlMFZXSUh1RDZYY2E2cFQ2UG03OV9DeFVMSnnSAXBBVV95cUxPdUdsWHk1bThTMFhlcW9icUpCcXg2VVZMLWpoUTh6cWxLZVBVTmo5Wm5zaXltNThoYjBuSEFVYm5ZRWRxaGpFZVVBWlhORkxXTU9ZTUg1ZTBWV0lIdUQ2WGNhNnBUNlBtNzlfQ3hVTEp5?oc=5</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>KITH Officially Reveals Their New Balance 991 And 991v2 - Sneaker News</t>
+          <t>“Neptune Grey” Washes Over The New Balance 2010 - Sneaker News</t>
         </is>
       </c>
       <c r="B31" s="38" t="inlineStr">
@@ -2364,19 +2364,19 @@
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE91R2xYeTVtOFMwWGVxb2JxSkJxeDZVVkwtamhROHpxbEtlUFVOajlabnNpeW01OGhiMG5IQVVibllFZHFoakVlVUFaWE5GTFdNT1lNSDVlMFZXSUh1RDZYY2E2cFQ2UG03OV9DeFVMSnnSAXBBVV95cUxPdUdsWHk1bThTMFhlcW9icUpCcXg2VVZMLWpoUTh6cWxLZVBVTmo5Wm5zaXltNThoYjBuSEFVYm5ZRWRxaGpFZVVBWlhORkxXTU9ZTUg1ZTBWV0lIdUQ2WGNhNnBUNlBtNzlfQ3hVTEp5?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNam1Td1prcTZ0aVRCTGxubERiczh6bEEwMG54cmJtZkxpMDVRM21kZTNCZzJfY3JhVm5FZmNyWTNLdFE4XzlqQmVreUZYd3FwcnhyVmFzcFE3QUpCVnB2c004bVZzNlpMamFaYVRHQVJ4YlFFRGRib1Vyd3BUd2t3OWFKZU4tejR6WDZZ0gGLAUFVX3lxTE1qbVN3WmtxNnRpVEJMbG5sRGJzOHpsQTAwbnhyYm1mTGkwNVEzbWRlM0JnMl9jcmFWbkVmY3JZM0t0UThfOWpCZWt5Rlh3cXByeHJWYXNwUTdBSkJWcHZzTThtVnM2WkxqYVphVEdBUnhiUUVEZGJvVXJ3cFR3a3c5YUplTi16NHpYNlk?oc=5</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>“Neptune Grey” Washes Over The New Balance 2010 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B32" s="31" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>The Nike Air Max 95 “Bright Violet” Steps Into Spring - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C32" s="27" t="inlineStr">
@@ -2384,9 +2384,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D32" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
         </is>
       </c>
       <c r="E32" s="17" t="inlineStr">
@@ -2394,26 +2394,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F32" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G32" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H32" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNam1Td1prcTZ0aVRCTGxubERiczh6bEEwMG54cmJtZkxpMDVRM21kZTNCZzJfY3JhVm5FZmNyWTNLdFE4XzlqQmVreUZYd3FwcnhyVmFzcFE3QUpCVnB2c004bVZzNlpMamFaYVRHQVJ4YlFFRGRib1Vyd3BUd2t3OWFKZU4tejR6WDZZ0gGLAUFVX3lxTE1qbVN3WmtxNnRpVEJMbG5sRGJzOHpsQTAwbnhyYm1mTGkwNVEzbWRlM0JnMl9jcmFWbkVmY3JZM0t0UThfOWpCZWt5Rlh3cXByeHJWYXNwUTdBSkJWcHZzTThtVnM2WkxqYVphVEdBUnhiUUVEZGJvVXJ3cFR3a3c5YUplTi16NHpYNlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPT2NaUGJDY0p0amRJbGdyMHJmUlpfVjdIVU4zZzA0R3VjakZNdTd4V29acXpYX3dQY0NQbEQ1ZnBhMVE0and2SnBOSndOWlNVQTdxY3lCQzd2UmpqUFhhYjJSOEh5NkFuOE9oZG1YcVdhTTE2VDR0UHlsa05ScnduRjMzZnBOODVhaXJVSFNiOXZ4S1dKSWJzeVJzVEtaX03SAZ8BQVVfeXFMT09jWlBiQ2NKdGpkSWxncjByZlJaX1Y3SFVOM2cwNEd1Y2pGTXU3eFdvWnF6WF93UGNDUGxENWZwYTFRNGp3dkpwTkp3TlpTVUE3cWN5QkM3dlJqalBYYWIyUjhIeTZBbjhPaGRtWHFXYU0xNlQ0dFB5bGtOUnJ3bkYzM2ZwTjg1YWlyVUhTYjl2eEtXSklic3lSc1RLWl9N?oc=5</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>The Nike Air Max 95 “Bright Violet” Steps Into Spring - Sneaker News</t>
+          <t>Dylan Harper Coats His Nike GT Cut 4 PE In Bronze - Sneaker News</t>
         </is>
       </c>
       <c r="B33" s="30" t="inlineStr">
@@ -2426,9 +2426,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>$160</t>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
@@ -2448,19 +2448,19 @@
       </c>
       <c r="H33" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPT2NaUGJDY0p0amRJbGdyMHJmUlpfVjdIVU4zZzA0R3VjakZNdTd4V29acXpYX3dQY0NQbEQ1ZnBhMVE0and2SnBOSndOWlNVQTdxY3lCQzd2UmpqUFhhYjJSOEh5NkFuOE9oZG1YcVdhTTE2VDR0UHlsa05ScnduRjMzZnBOODVhaXJVSFNiOXZ4S1dKSWJzeVJzVEtaX03SAZ8BQVVfeXFMT09jWlBiQ2NKdGpkSWxncjByZlJaX1Y3SFVOM2cwNEd1Y2pGTXU3eFdvWnF6WF93UGNDUGxENWZwYTFRNGp3dkpwTkp3TlpTVUE3cWN5QkM3dlJqalBYYWIyUjhIeTZBbjhPaGRtWHFXYU0xNlQ0dFB5bGtOUnJ3bkYzM2ZwTjg1YWlyVUhTYjl2eEtXSklic3lSc1RLWl9N?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNNW9rMnNkdUdzVHdadWxRVXJqUlY3ZWdyQnV1bEpfaU5rRWE1aUZGRW5CaC14Tl9zLXdIM3lSTWVrUVdEcUQ3YWNzRlhuanRORWNVd1ZEZGZlMXdXNU13cGNaVkx2bU1XZm5HY3VlaGtpUkxZRWFfWWVlWlp4amdhVkVxT0VvaVRZWXhRQWdRREkyYnRrZE9LNWlmb3E5Z9IBngFBVV95cUxNNW9rMnNkdUdzVHdadWxRVXJqUlY3ZWdyQnV1bEpfaU5rRWE1aUZGRW5CaC14Tl9zLXdIM3lSTWVrUVdEcUQ3YWNzRlhuanRORWNVd1ZEZGZlMXdXNU13cGNaVkx2bU1XZm5HY3VlaGtpUkxZRWFfWWVlWlp4amdhVkVxT0VvaVRZWXhRQWdRREkyYnRrZE9LNWlmb3E5Zw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Dylan Harper Coats His Nike GT Cut 4 PE In Bronze - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B34" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Sneaker News - Air Jordans, Sneaker Release Dates, News and More - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C34" s="27" t="inlineStr">
@@ -2478,31 +2478,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G34" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F34" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G34" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H34" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNNW9rMnNkdUdzVHdadWxRVXJqUlY3ZWdyQnV1bEpfaU5rRWE1aUZGRW5CaC14Tl9zLXdIM3lSTWVrUVdEcUQ3YWNzRlhuanRORWNVd1ZEZGZlMXdXNU13cGNaVkx2bU1XZm5HY3VlaGtpUkxZRWFfWWVlWlp4amdhVkVxT0VvaVRZWXhRQWdRREkyYnRrZE9LNWlmb3E5Z9IBngFBVV95cUxNNW9rMnNkdUdzVHdadWxRVXJqUlY3ZWdyQnV1bEpfaU5rRWE1aUZGRW5CaC14Tl9zLXdIM3lSTWVrUVdEcUQ3YWNzRlhuanRORWNVd1ZEZGZlMXdXNU13cGNaVkx2bU1XZm5HY3VlaGtpUkxZRWFfWWVlWlp4amdhVkVxT0VvaVRZWXhRQWdRREkyYnRrZE9LNWlmb3E5Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiPEFVX3lxTE1KS2VObTBlWlJ5ZlZUd01pbzB0QV9NaUN5VDFGTTdHSGhSTko2UnpiSzJSa0NXZFo5Y1J3UA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Sneaker News - Air Jordans, Sneaker Release Dates, News and More - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The First-Ever Mamba Day Sneaker Returns: Nike Kobe 11 Protro Arrives April 13th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C35" s="22" t="inlineStr">
@@ -2520,31 +2520,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F35" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G35" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiPEFVX3lxTE1KS2VObTBlWlJ5ZlZUd01pbzB0QV9NaUN5VDFGTTdHSGhSTko2UnpiSzJSa0NXZFo5Y1J3UA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5JR0hlZjNqSVM4bnVGbkZsSmxjMmthQm9iY3NzT0ZMcm9ld3ZjN0dkaUdsU3YwbkRyOFpGcHZmT0t5dWF3NFNEX2tOd3l1YzZKcVJmN3V5OURZOGl4QzNBeUlsT0dTZzUzLUROVUtSejFaYnJ2eTNDNW90T2TSAXxBVV95cUxOSUdIZWYzaklTOG51Rm5GbEpsYzJrYUJvYmNzc09GTHJvZXd2YzdHZGlHbFN2MG5EcjhaRnB2Zk9LeXVhdzRTRF9rTnd5dWM2SnFSZjd1eTlEWThpeEMzQXlJbE9HU2c1My1ETlVLUnoxWmJydnkzQzVvdE9k?oc=5</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>The First-Ever Mamba Day Sneaker Returns: Nike Kobe 11 Protro Arrives April 13th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B36" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Vans Rides The Patent Leather Craze With The Old Skool “Harajuku” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Vans</t>
         </is>
       </c>
       <c r="C36" s="27" t="inlineStr">
@@ -2562,19 +2562,19 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F36" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G36" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H36" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5JR0hlZjNqSVM4bnVGbkZsSmxjMmthQm9iY3NzT0ZMcm9ld3ZjN0dkaUdsU3YwbkRyOFpGcHZmT0t5dWF3NFNEX2tOd3l1YzZKcVJmN3V5OURZOGl4QzNBeUlsT0dTZzUzLUROVUtSejFaYnJ2eTNDNW90T2TSAXxBVV95cUxOSUdIZWYzaklTOG51Rm5GbEpsYzJrYUJvYmNzc09GTHJvZXd2YzdHZGlHbFN2MG5EcjhaRnB2Zk9LeXVhdzRTRF9rTnd5dWM2SnFSZjd1eTlEWThpeEMzQXlJbE9HU2c1My1ETlVLUnoxWmJydnkzQzVvdE9k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5wd3ZSdVhEZnl4cllMVEhnZHVsRlZVUXRJQ3R3RWVTQThKekdiZjVOU3JZd0FIQlA5RE9TXzI4UlNoMHU3ekRybUJneEs1U3BldUJ6WnZDbVYyUjMtLWVVczRkMFBRdG1pZzlRejRFTFhJQ29LTDRSeWx2RlFCYVnSAX9BVV95cUxOcHd2UnVYRGZ5eHJZTFRIZ2R1bEZWVVF0SUN0d0VlU0E4SnpHYmY1TlNyWXdBSEJQOURPU18yOFJTaDB1N3pEcm1CZ3hLNVNwZXVCelp2Q21WMlIzLS1lVXM0ZDBQUXRtaWc5UXo0RUxYSUNvS0w0UnlsdkZRQmFZ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3673,12 +3673,12 @@
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Detailed Look At The Air Jordan 5 “Wolf Grey” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B63" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Satoshi Nakamoto Influence Continues On The Vans Slip-On For Spring - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>Vans</t>
         </is>
       </c>
       <c r="C63" s="22" t="inlineStr">
@@ -3686,9 +3686,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D63" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D63" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
@@ -3696,31 +3696,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F63" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G63" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F63" s="39" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G63" s="40" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H63" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFAwQUZiQktBRDlWQmJSVlRpYjdVSVRZZUYycVFjZ053cG0tM2stODZRX0UtRHdnVW1EbHg1Z3lXejZfWU1RODkza190cGJLQmxtandjdFlBc2xZSGVpa3dIcjFoVUNLRTNWcHfSAWpBVV95cUxQMEFGYkJLQUQ5VkJiUlZUaWI3VUlUWWVGMnFRY2dOd3BtLTNrLTg2UV9FLUR3Z1VtRGx4NWd5V3o2X1lNUTg5M2tfdHBiS0JsbWp3Y3RZQXNsWUhlaWt3SHIxaFVDS0UzVnB3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOV9IBeEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOVw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>Quavo Spotted In The Upcoming Sinclair x PUMA Suede - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B64" s="41" t="inlineStr">
-        <is>
-          <t>Puma</t>
+          <t>Detailed Look At The Air Jordan 5 “Wolf Grey” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C64" s="27" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>$75</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="E64" s="17" t="inlineStr">
@@ -3738,31 +3738,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F64" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G64" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F64" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G64" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H64" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE13eWlSUXpENWV1UWhPdkY2SDVtVGhINXBNSUNRdDMzMDdtWVR3S1RwSndiLS1XVGxuZkJxV3FLQzRuZy1sSFNYZkx0M2g4Z04zTGNwZFQwQmphQ0VlaEdzVGdEcExKY2xocVY2R0xR0gFuQVVfeXFMTXd5aVJRekQ1ZXVRaE92RjZINW1UaEg1cE1JQ1F0MzMwN21ZVHdLVHBKd2ItLVdUbG5mQnFXcUtDNG5nLWxIU1hmTHQzaDhnTjNMY3BkVDBCamFDRWVoR3NUZ0RwTEpjbGhxVjZHTFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFAwQUZiQktBRDlWQmJSVlRpYjdVSVRZZUYycVFjZ053cG0tM2stODZRX0UtRHdnVW1EbHg1Z3lXejZfWU1RODkza190cGJLQmxtandjdFlBc2xZSGVpa3dIcjFoVUNLRTNWcHfSAWpBVV95cUxQMEFGYkJLQUQ5VkJiUlZUaWI3VUlUWWVGMnFRY2dOd3BtLTNrLTg2UV9FLUR3Z1VtRGx4NWd5V3o2X1lNUTg5M2tfdHBiS0JsbWp3Y3RZQXNsWUhlaWt3SHIxaFVDS0UzVnB3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>The Nike ACG LDV Tells The Origin Story Of All-Conditions Gear - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B65" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Quavo Spotted In The Upcoming Sinclair x PUMA Suede - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B65" s="41" t="inlineStr">
+        <is>
+          <t>Puma</t>
         </is>
       </c>
       <c r="C65" s="22" t="inlineStr">
@@ -3770,9 +3770,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D65" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>$75</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -3780,31 +3780,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G65" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F65" s="39" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G65" s="40" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H65" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE5IdXF1aDZ3Q3gyOUJVb2FVeVZHWG4wcTVwYUk5cGU0cUFMZjhWeFBnZzhkR0ZXaVNhOXEzTU41cUx5VDcwTFB3T0o3a0ZqTzNmSXFxTERwS2YzZG81cEVyR3JXUl9BRUVza2tHRHFn0gFuQVVfeXFMTkh1cXVoNndDeDI5QlVvYVV5VkdYbjBxNXBhSTlwZTRxQUxmOFZ4UGdnOGRHRldpU2E5cTNNTjVxTHlUNzBMUHdPSjdrRmpPM2ZJcXFMRHBLZjNkbzVwRXJHcldSX0FFRXNra0dEcWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE13eWlSUXpENWV1UWhPdkY2SDVtVGhINXBNSUNRdDMzMDdtWVR3S1RwSndiLS1XVGxuZkJxV3FLQzRuZy1sSFNYZkx0M2g4Z04zTGNwZFQwQmphQ0VlaEdzVGdEcExKY2xocVY2R0xR0gFuQVVfeXFMTXd5aVJRekQ1ZXVRaE92RjZINW1UaEg1cE1JQ1F0MzMwN21ZVHdLVHBKd2ItLVdUbG5mQnFXcUtDNG5nLWxIU1hmTHQzaDhnTjNMY3BkVDBCamFDRWVoR3NUZ0RwTEpjbGhxVjZHTFE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>Elephant Print Finally Arrives On This Jordan Dad Shoe - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B66" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike ACG LDV Tells The Origin Story Of All-Conditions Gear - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B66" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C66" s="27" t="inlineStr">
@@ -3822,31 +3822,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F66" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G66" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H66" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZ9IBhgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE5IdXF1aDZ3Q3gyOUJVb2FVeVZHWG4wcTVwYUk5cGU0cUFMZjhWeFBnZzhkR0ZXaVNhOXEzTU41cUx5VDcwTFB3T0o3a0ZqTzNmSXFxTERwS2YzZG81cEVyR3JXUl9BRUVza2tHRHFn0gFuQVVfeXFMTkh1cXVoNndDeDI5QlVvYVV5VkdYbjBxNXBhSTlwZTRxQUxmOFZ4UGdnOGRHRldpU2E5cTNNTjVxTHlUNzBMUHdPSjdrRmpPM2ZJcXFMRHBLZjNkbzVwRXJHcldSX0FFRXNra0dEcWc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>adidas Delivers A Late “Chinese New Year” Tribute On The EVO SL Trainer - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Elephant Print Finally Arrives On This Jordan Dad Shoe - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C67" s="22" t="inlineStr">
@@ -3864,31 +3864,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F67" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G67" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F67" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G67" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H67" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQdIBfkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZ9IBhgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>Kim Kardashian And NikeSkims Debut The Rift Mesh “Light Bone” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B68" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>adidas Delivers A Late “Chinese New Year” Tribute On The EVO SL Trainer - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C68" s="27" t="inlineStr">
@@ -3918,19 +3918,19 @@
       </c>
       <c r="H68" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPWVh4LUNfVjg0bFllenoxZFp1M1BxM1NQdDZCTmotbmt0MFRuVzUtanlJN1BiSkk1V240U2szLVlMVE1rZlBxbVhHRmV2MGcta0JBUnVSY3AwR0cyN05LWjVxYW9NNVUzUlZaR0V5cF9QWlBnTHVsTEg2THdka3NKTG82NkLSAYQBQVVfeXFMT1lYeC1DX1Y4NGxZZXp6MWRadTNQcTNTUHQ2Qk5qLW5rdDBUblc1LWp5STdQYkpJNVduNFNrMy1ZTFRNa2ZQcW1YR0ZldjBnLWtCQVJ1UmNwMEdHMjdOS1o1cWFvTTVVM1JWWkdFeXBfUFpQZ0x1bExINkx3ZGtzSkxvNjZC?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQdIBfkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Reebok Is Restocking The Angel Reese 1 “Receipts Ready” On February 6th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B69" s="23" t="inlineStr">
-        <is>
-          <t>Reebok</t>
+          <t>Kim Kardashian And NikeSkims Debut The Rift Mesh “Light Bone” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B69" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C69" s="22" t="inlineStr">
@@ -3948,31 +3948,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F69" s="39" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G69" s="40" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F69" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G69" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QdIBeEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPWVh4LUNfVjg0bFllenoxZFp1M1BxM1NQdDZCTmotbmt0MFRuVzUtanlJN1BiSkk1V240U2szLVlMVE1rZlBxbVhHRmV2MGcta0JBUnVSY3AwR0cyN05LWjVxYW9NNVUzUlZaR0V5cF9QWlBnTHVsTEg2THdka3NKTG82NkLSAYQBQVVfeXFMT1lYeC1DX1Y4NGxZZXp6MWRadTNQcTNTUHQ2Qk5qLW5rdDBUblc1LWp5STdQYkpJNVduNFNrMy1ZTFRNa2ZQcW1YR0ZldjBnLWtCQVJ1UmNwMEdHMjdOS1o1cWFvTTVVM1JWWkdFeXBfUFpQZ0x1bExINkx3ZGtzSkxvNjZC?oc=5</t>
         </is>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>The Nike Air Max Plus Carries “Pink Foam” Echoes - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B70" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Reebok Is Restocking The Angel Reese 1 “Receipts Ready” On February 6th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="inlineStr">
+        <is>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="C70" s="27" t="inlineStr">
@@ -3980,9 +3980,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D70" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
+      <c r="D70" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E70" s="17" t="inlineStr">
@@ -3990,26 +3990,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F70" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G70" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F70" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G70" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H70" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNRU1pWDF4alUtNjJGUVFLR0hya1h1Vm5RVFJnM1BvNGh1azNHdUFld19kZS15LUZIRXZ3aUFtbnlnYlpQWTZCTHAzd1FmZi1XY3A5OUFEZ3ZXRmR0MFpNU3BFX2ZDYUYzZG10Sl96OVlBd094OUVtQ1FiR0RrbTkyc2hBQzZlVml2MWdLQ0FUakpPY0pLRXfSAZYBQVVfeXFMTUVNaVgxeGpVLTYyRlFRS0dIcmtYdVZuUVRSZzNQbzRodWszR3VBZXdfZGUteS1GSEV2d2lBbW55Z2JaUFk2QkxwM3dRZmYtV2NwOTlBRGd2V0ZkdDBaTVNwRV9mQ2FGM2RtdEpfejlZQXdPeDlFbUNRYkdEa205MnNoQUM2ZVZpdjFnS0NBVGpKT2NKS0V3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QdIBeEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Where To Buy The Nike Ja 3 “Light Show” - Sneaker News</t>
+          <t>The Nike Air Max Plus Carries “Pink Foam” Echoes - Sneaker News</t>
         </is>
       </c>
       <c r="B71" s="30" t="inlineStr">
@@ -4022,9 +4022,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D71" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>$160</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
@@ -4044,14 +4044,14 @@
       </c>
       <c r="H71" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE13M1JfZjJrYmwzdUs0N0FiS1Q2NEJQbS01TnJLbEVpNzUwMUt1NFphVmtoWTBFeU90NmNqbVNwNnNlay1HZXBHcGtRTk1wRFR5WV92MnpxSTlQUmpmUGFkNXN5QnJJaUxfOFZLVmNaMnRnUWp3TGfSAXZBVV95cUxNdzNSX2Yya2JsM3VLNDdBYktUNjRCUG0tNU5yS2xFaTc1MDFLdTRaYVZraFkwRXlPdDZjam1TcDZzZWstR2VwR3BrUU5NcERUeVlfdjJ6cUk5UFJqZlBhZDVzeUJySWlMXzhWS1ZjWjJ0Z1Fqd0xn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNRU1pWDF4alUtNjJGUVFLR0hya1h1Vm5RVFJnM1BvNGh1azNHdUFld19kZS15LUZIRXZ3aUFtbnlnYlpQWTZCTHAzd1FmZi1XY3A5OUFEZ3ZXRmR0MFpNU3BFX2ZDYUYzZG10Sl96OVlBd094OUVtQ1FiR0RrbTkyc2hBQzZlVml2MWdLQ0FUakpPY0pLRXfSAZYBQVVfeXFMTUVNaVgxeGpVLTYyRlFRS0dIcmtYdVZuUVRSZzNQbzRodWszR3VBZXdfZGUteS1GSEV2d2lBbW55Z2JaUFk2QkxwM3dRZmYtV2NwOTlBRGd2V0ZkdDBaTVNwRV9mQ2FGM2RtdEpfejlZQXdPeDlFbUNRYkdEa205MnNoQUM2ZVZpdjFnS0NBVGpKT2NKS0V3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>The Nike Mind 001 Dons “Team Red” - Sneaker News</t>
+          <t>Where To Buy The Nike Ja 3 “Light Show” - Sneaker News</t>
         </is>
       </c>
       <c r="B72" s="35" t="inlineStr">
@@ -4086,14 +4086,14 @@
       </c>
       <c r="H72" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPdUhnbEZUUWhwTFVvR213Z3NsazZoT190ajJkNnRDOWxuUzJsLWY0UjFfUk5jSlV6OEVUOWl1ZmZGRmxmemlHMWI2NEotdnFPTmV1UUpCTUNwcGR0NXdDZll4Vks2aWhzSHI1T0I1clAtYzN5UlFFWm5ycHlXa2hiQVVVQkcxaUtUd25Gb2VSbkx1b2dKbWhOOXlQUFBmQnfSAZ8BQVVfeXFMT3VIZ2xGVFFocExVb0dtd2dzbGs2aE9fdGoyZDZ0QzlsblMybC1mNFIxX1JOY0pVejhFVDlpdWZmRkZsZnppRzFiNjRKLXZxT05ldVFKQk1DcHBkdDV3Q2ZZeFZLNmloc0hyNU9CNXJQLWMzeVJRRVpucnB5V2toYkFVVUJHMWlLVHduRm9lUm5MdW9nSm1oTjl5UFBQZkJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE13M1JfZjJrYmwzdUs0N0FiS1Q2NEJQbS01TnJLbEVpNzUwMUt1NFphVmtoWTBFeU90NmNqbVNwNnNlay1HZXBHcGtRTk1wRFR5WV92MnpxSTlQUmpmUGFkNXN5QnJJaUxfOFZLVmNaMnRnUWp3TGfSAXZBVV95cUxNdzNSX2Yya2JsM3VLNDdBYktUNjRCUG0tNU5yS2xFaTc1MDFLdTRaYVZraFkwRXlPdDZjam1TcDZzZWstR2VwR3BrUU5NcERUeVlfdjJ6cUk5UFJqZlBhZDVzeUJySWlMXzhWS1ZjWjJ0Z1Fqd0xn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Fragment Design Gives A Peek Into The Future Of The Nike Mind Series - Sneaker News</t>
+          <t>The Nike Mind 001 Dons “Team Red” - Sneaker News</t>
         </is>
       </c>
       <c r="B73" s="30" t="inlineStr">
@@ -4116,26 +4116,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F73" s="42" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G73" s="43" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H73" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQajFRX3BidzVza3RsNEpsYkF0UzlCVFJGbXZXNUsySGxWd3c2MUlHRmhhNDVybmgzYld3M202aWI0dEFhOXp2NXVMVk9TRWkzQ1l3SG9vYVZYNG9tcmQyRXFmQzMyVy1idkQ0MmhPZ01ST251SlZ0TF9fWktLaXY4NDNR0gGCAUFVX3lxTFBqMVFfcGJ3NXNrdGw0SmxiQXRTOUJUUkZtdlc1SzJIbFZ3dzYxSUdGaGE0NXJuaDNiV3czbTZpYjR0QWE5enY1dUxWT1NFaTNDWXdIb29hVlg0b21yZDJFcWZDMzJXLWJ2RDQyaE9nTVJPbnVKVnRMX19aS0tpdjg0M1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPdUhnbEZUUWhwTFVvR213Z3NsazZoT190ajJkNnRDOWxuUzJsLWY0UjFfUk5jSlV6OEVUOWl1ZmZGRmxmemlHMWI2NEotdnFPTmV1UUpCTUNwcGR0NXdDZll4Vks2aWhzSHI1T0I1clAtYzN5UlFFWm5ycHlXa2hiQVVVQkcxaUtUd25Gb2VSbkx1b2dKbWhOOXlQUFBmQnfSAZ8BQVVfeXFMT3VIZ2xGVFFocExVb0dtd2dzbGs2aE9fdGoyZDZ0QzlsblMybC1mNFIxX1JOY0pVejhFVDlpdWZmRkZsZnppRzFiNjRKLXZxT05ldVFKQk1DcHBkdDV3Q2ZZeFZLNmloc0hyNU9CNXJQLWMzeVJRRVpucnB5V2toYkFVVUJHMWlLVHduRm9lUm5MdW9nSm1oTjl5UFBQZkJ3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>Nike Almost Put adidas And Reebok Logos On This LeBron Shirt - Sneaker News</t>
+          <t>Fragment Design Gives A Peek Into The Future Of The Nike Mind Series - Sneaker News</t>
         </is>
       </c>
       <c r="B74" s="35" t="inlineStr">
@@ -4158,31 +4158,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F74" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G74" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F74" s="36" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G74" s="37" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H74" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRd9IBckFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQajFRX3BidzVza3RsNEpsYkF0UzlCVFJGbXZXNUsySGxWd3c2MUlHRmhhNDVybmgzYld3M202aWI0dEFhOXp2NXVMVk9TRWkzQ1l3SG9vYVZYNG9tcmQyRXFmQzMyVy1idkQ0MmhPZ01ST251SlZ0TF9fWktLaXY4NDNR0gGCAUFVX3lxTFBqMVFfcGJ3NXNrdGw0SmxiQXRTOUJUUkZtdlc1SzJIbFZ3dzYxSUdGaGE0NXJuaDNiV3czbTZpYjR0QWE5enY1dUxWT1NFaTNDWXdIb29hVlg0b21yZDJFcWZDMzJXLWJ2RDQyaE9nTVJPbnVKVnRMX19aS0tpdjg0M1E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>The Jordan MVP 92 Approaches A “Tour” Colorway - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B75" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Almost Put adidas And Reebok Logos On This LeBron Shirt - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B75" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C75" s="22" t="inlineStr">
@@ -4200,31 +4200,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F75" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G75" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H75" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPOXZZY2ozRUpkRVpXSzl6YWsxZ2hPaWlQajVWSUZPajVSVjRmX00wOXdlNEE2amtpcmtiRVZPQl9MTnQ4eWc3TXptakxKQmw3WVBuemVCQTdoTC1sSHZCT0VmYVlDWDA1dlAwRWVwNTBLQkxBeG1XZ0plNlllNzItX0lBMnN4Y1lGeWtXaTc5WkxzZzVIME930gGXAUFVX3lxTE85dlljajNFSmRFWldLOXphazFnaE9paVBqNVZJRk9qNVJWNGZfTTA5d2U0QTZqa2lya2JFVk9CX0xOdDh5ZzdNem1qTEpCbDdZUG56ZUJBN2hMLWxIdkJPRWZhWUNYMDV2UDBFZXA1MEtCTEF4bVdnSmU2WWU3Mi1fSUEyc3hjWUZ5a1dpNzlaTHNnNUgwT3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRd9IBckFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRdw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>The Nike Air Max Plus Gathers A “Pencil Point” Gradient - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B76" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The Jordan MVP 92 Approaches A “Tour” Colorway - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B76" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C76" s="27" t="inlineStr">
@@ -4232,9 +4232,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D76" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
+      <c r="D76" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E76" s="17" t="inlineStr">
@@ -4242,31 +4242,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F76" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G76" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F76" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G76" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H76" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOenBOTEVoZjlEY0lFejN2bGFSaVpHekxuMWkzU1VUNHNHTmpvSjVMMDdFV3ltTlEyUjhvRURDNGlDMGVFUXYwVXhvNTE1M3VoeDdaQzgyTzMtR18tY2hrMS1JZlpLNlNhVHdVOE56eDJLZ0UtLU90SFFIWGxoQXhDVlkxcEdRR01JYW53OEkzSmcyTnl4Slg5Z2RlUlnSAZwBQVVfeXFMTnpwTkxFaGY5RGNJRXozdmxhUmlaR3pMbjFpM1NVVDRzR05qb0o1TDA3RVd5bU5RMlI4b0VEQzRpQzBlRVF2MFV4bzUxNTN1aHg3WkM4Mk8zLUdfLWNoazEtSWZaSzZTYVR3VThOengyS2dFLS1PdEhRSFhsaEF4Q1ZZMXBHUUdNSWFudzhJM0pnMk55eEpYOWdkZVJZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPOXZZY2ozRUpkRVpXSzl6YWsxZ2hPaWlQajVWSUZPajVSVjRmX00wOXdlNEE2amtpcmtiRVZPQl9MTnQ4eWc3TXptakxKQmw3WVBuemVCQTdoTC1sSHZCT0VmYVlDWDA1dlAwRWVwNTBLQkxBeG1XZ0plNlllNzItX0lBMnN4Y1lGeWtXaTc5WkxzZzVIME930gGXAUFVX3lxTE85dlljajNFSmRFWldLOXphazFnaE9paVBqNVZJRk9qNVJWNGZfTTA5d2U0QTZqa2lya2JFVk9CX0xOdDh5ZzdNem1qTEpCbDdZUG56ZUJBN2hMLWxIdkJPRWZhWUNYMDV2UDBFZXA1MEtCTEF4bVdnSmU2WWU3Mi1fSUEyc3hjWUZ5a1dpNzlaTHNnNUgwT3c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Official Images Of The Air Jordan 3 “El Vuelo” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B77" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike Air Max Plus Gathers A “Pencil Point” Gradient - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C77" s="22" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t>$160</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
@@ -4284,31 +4284,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F77" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G77" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H77" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNMkxLNHFJenQ5VUc0OXg1M2hKWGwyeUpjN25QZHRKYllRSE5TU2xvcXBNSjNqQ0RzLXF4OVVfWDdaLTkweXZQZkZlWEplQmVqbm5BZlZibXBuWWgxeTFwSlZsVkpfSXlmaTM3Y0xTOFI3ZmFBLVRyRHpCUFc3WkRaVmJKeVFhSTNz0gGIAUFVX3lxTE0yTEs0cUl6dDlVRzQ5eDUzaEpYbDJ5SmM3blBkdEpiWVFITlNTbG9xcE1KM2pDRHMtcXg5VV9YN1otOTB5dlBmRmVYSmVCZWpubkFmVmJtcG5ZaDF5MXBKVmxWSl9JeWZpMzdjTFM4UjdmYUEtVHJEekJQVzdaRFpWYkp5UWFJM3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOenBOTEVoZjlEY0lFejN2bGFSaVpHekxuMWkzU1VUNHNHTmpvSjVMMDdFV3ltTlEyUjhvRURDNGlDMGVFUXYwVXhvNTE1M3VoeDdaQzgyTzMtR18tY2hrMS1JZlpLNlNhVHdVOE56eDJLZ0UtLU90SFFIWGxoQXhDVlkxcEdRR01JYW53OEkzSmcyTnl4Slg5Z2RlUlnSAZwBQVVfeXFMTnpwTkxFaGY5RGNJRXozdmxhUmlaR3pMbjFpM1NVVDRzR05qb0o1TDA3RVd5bU5RMlI4b0VEQzRpQzBlRVF2MFV4bzUxNTN1aHg3WkM4Mk8zLUdfLWNoazEtSWZaSzZTYVR3VThOengyS2dFLS1PdEhRSFhsaEF4Q1ZZMXBHUUdNSWFudzhJM0pnMk55eEpYOWdkZVJZ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>Dylan Harper’s Nike GT Cut 1 “Tri-State” Drops March 19th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B78" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Official Images Of The Air Jordan 3 “El Vuelo” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B78" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C78" s="27" t="inlineStr">
@@ -4316,9 +4316,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D78" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E78" s="17" t="inlineStr">
@@ -4326,26 +4326,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F78" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G78" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F78" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G78" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H78" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOb0ROYk0wWW5EMUNqbmNuVmFvdmtRTXVkQVNrVFJmVDB6RUttdWk0cUw5Y0NlbnNmSHhDZWMydXdnWndoWjNlQURkMlRFWHBCVXpOZVlXdzZ4RmRtSDJRcW10S0wxTVRTd1VyeVhYVEpMMTQzbmo1QzNEWjdfRm1aN9IBgAFBVV95cUxOb0ROYk0wWW5EMUNqbmNuVmFvdmtRTXVkQVNrVFJmVDB6RUttdWk0cUw5Y0NlbnNmSHhDZWMydXdnWndoWjNlQURkMlRFWHBCVXpOZVlXdzZ4RmRtSDJRcW10S0wxTVRTd1VyeVhYVEpMMTQzbmo1QzNEWjdfRm1aNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNMkxLNHFJenQ5VUc0OXg1M2hKWGwyeUpjN25QZHRKYllRSE5TU2xvcXBNSjNqQ0RzLXF4OVVfWDdaLTkweXZQZkZlWEplQmVqbm5BZlZibXBuWWgxeTFwSlZsVkpfSXlmaTM3Y0xTOFI3ZmFBLVRyRHpCUFc3WkRaVmJKeVFhSTNz0gGIAUFVX3lxTE0yTEs0cUl6dDlVRzQ5eDUzaEpYbDJ5SmM3blBkdEpiWVFITlNTbG9xcE1KM2pDRHMtcXg5VV9YN1otOTB5dlBmRmVYSmVCZWpubkFmVmJtcG5ZaDF5MXBKVmxWSl9JeWZpMzdjTFM4UjdmYUEtVHJEekJQVzdaRFpWYkp5UWFJM3M?oc=5</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>The Nike KD 4 Retro “Easter” Releases On April 18th - Sneaker News</t>
+          <t>Dylan Harper’s Nike GT Cut 1 “Tri-State” Drops March 19th - Sneaker News</t>
         </is>
       </c>
       <c r="B79" s="30" t="inlineStr">
@@ -4380,14 +4380,14 @@
       </c>
       <c r="H79" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOMnBtTnMtOFdWZ3p3Q1lSVG9jNG94VFZvWndfb3k4SUg2MVdsZV9ZS3RhZHpfVmNsQzYwUW80VUNqdlE1UUU0a1doaEJqT0V5UXNkQXI0ZU93RU5ZVjg4YTNLcEZKMlhUQ044aFpFR2hYc2FmSXFENFFsYzFvZlRHVmFR0gGCAUFVX3lxTE4ycG1Ocy04V1ZnendDWVJUb2M0b3hUVm9ad19veThJSDYxV2xlX1lLdGFkel9WY2xDNjBRbzRVQ2p2UTVRRTRrV2hoQmpPRXlRc2RBcjRlT3dFTllWODhhM0twRkoyWFRDTjhoWkVHaFhzYWZJcUQ0UWxjMW9mVEdWYVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOb0ROYk0wWW5EMUNqbmNuVmFvdmtRTXVkQVNrVFJmVDB6RUttdWk0cUw5Y0NlbnNmSHhDZWMydXdnWndoWjNlQURkMlRFWHBCVXpOZVlXdzZ4RmRtSDJRcW10S0wxTVRTd1VyeVhYVEpMMTQzbmo1QzNEWjdfRm1aN9IBgAFBVV95cUxOb0ROYk0wWW5EMUNqbmNuVmFvdmtRTXVkQVNrVFJmVDB6RUttdWk0cUw5Y0NlbnNmSHhDZWMydXdnWndoWjNlQURkMlRFWHBCVXpOZVlXdzZ4RmRtSDJRcW10S0wxTVRTd1VyeVhYVEpMMTQzbmo1QzNEWjdfRm1aNw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>Nike Basketball’s Unseen Hours Collection Inspired By Hustle And Grind - Sneaker News</t>
+          <t>The Nike KD 4 Retro “Easter” Releases On April 18th - Sneaker News</t>
         </is>
       </c>
       <c r="B80" s="35" t="inlineStr">
@@ -4422,19 +4422,19 @@
       </c>
       <c r="H80" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6b9IBgAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOMnBtTnMtOFdWZ3p3Q1lSVG9jNG94VFZvWndfb3k4SUg2MVdsZV9ZS3RhZHpfVmNsQzYwUW80VUNqdlE1UUU0a1doaEJqT0V5UXNkQXI0ZU93RU5ZVjg4YTNLcEZKMlhUQ044aFpFR2hYc2FmSXFENFFsYzFvZlRHVmFR0gGCAUFVX3lxTE4ycG1Ocy04V1ZnendDWVJUb2M0b3hUVm9ad19veThJSDYxV2xlX1lLdGFkel9WY2xDNjBRbzRVQ2p2UTVRRTRrV2hoQmpPRXlRc2RBcjRlT3dFTllWODhhM0twRkoyWFRDTjhoWkVHaFhzYWZJcUQ0UWxjMW9mVEdWYVE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>Meet The Newest New Balance Basketball Shoe, The P400 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B81" s="38" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>Nike Basketball’s Unseen Hours Collection Inspired By Hustle And Grind - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B81" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C81" s="22" t="inlineStr">
@@ -4452,31 +4452,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F81" s="39" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G81" s="40" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G81" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H81" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE13Q0d5X0VaTDlsSndTUDhUYUxLTjJMX1ZnQWFiRktEN1I4S3lEazc5R1BXYXJnSUd3QUpZeWpzMW5UQS1vWHNuQ2VFM19SWEhRVDhNSmRWWC1pVENGa0N3RkptRnhZVTN3bElHQkFoS3lPV3PSAXNBVV95cUxNd0NHeV9FWkw5bEp3U1A4VGFMS04yTF9WZ0FhYkZLRDdSOEt5RGs3OUdQV2FyZ0lHd0FKWXlqczFuVEEtb1hzbkNlRTNfUlhIUVQ4TUpkVlgtaVRDRmtDd0ZKbUZ4WVUzd2xJR0JBaEt5T1dz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6b9IBgAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6bw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Jordan Brand Officially Unveils The Jordan Heir Series 2 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B82" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Meet The Newest New Balance Basketball Shoe, The P400 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B82" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C82" s="27" t="inlineStr">
@@ -4494,31 +4494,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F82" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G82" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F82" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G82" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H82" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSdIBeEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE13Q0d5X0VaTDlsSndTUDhUYUxLTjJMX1ZnQWFiRktEN1I4S3lEazc5R1BXYXJnSUd3QUpZeWpzMW5UQS1vWHNuQ2VFM19SWEhRVDhNSmRWWC1pVENGa0N3RkptRnhZVTN3bElHQkFoS3lPV3PSAXNBVV95cUxNd0NHeV9FWkw5bEp3U1A4VGFMS04yTF9WZ0FhYkZLRDdSOEt5RGs3OUdQV2FyZ0lHd0FKWXlqczFuVEEtb1hzbkNlRTNfUlhIUVQ4TUpkVlgtaVRDRmtDd0ZKbUZ4WVUzd2xJR0JBaEt5T1dz?oc=5</t>
         </is>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Giannis Antetokounmpo’s Nike Giannis Freak 7 Launches On July 29th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B83" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Jordan Brand Officially Unveils The Jordan Heir Series 2 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B83" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C83" s="22" t="inlineStr">
@@ -4536,26 +4536,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F83" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G83" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G83" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbtIBeEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSdIBeEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>Official Images Of The Nike Sabrina 3 “Blueprint” - Sneaker News</t>
+          <t>Giannis Antetokounmpo’s Nike Giannis Freak 7 Launches On July 29th - Sneaker News</t>
         </is>
       </c>
       <c r="B84" s="35" t="inlineStr">
@@ -4590,19 +4590,19 @@
       </c>
       <c r="H84" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOYXRTM3V2MWdaYmp3M2FITldSbG8yRWhLdGhscE9wcGs3dEpVY21XVVRGRTllNEVIRlI0Ukwzb05FcmsxQnJMSHZsZGcwSVE5bGZTVDdmbHFNcmk3LUxnTG5kRVR4X1Vna25WYzVLZEp3OHE1bEdnUmRoX3NPQTRmMUZRYXJzV0MyUWJRMdIBjAFBVV95cUxOYXRTM3V2MWdaYmp3M2FITldSbG8yRWhLdGhscE9wcGs3dEpVY21XVVRGRTllNEVIRlI0Ukwzb05FcmsxQnJMSHZsZGcwSVE5bGZTVDdmbHFNcmk3LUxnTG5kRVR4X1Vna25WYzVLZEp3OHE1bEdnUmRoX3NPQTRmMUZRYXJzV0MyUWJRMQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbtIBeEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>Crocheted Swooshes Appear On This Air Jordan 1 Mid - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B85" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Official Images Of The Nike Sabrina 3 “Blueprint” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B85" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C85" s="22" t="inlineStr">
@@ -4610,9 +4610,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D85" s="8" t="inlineStr">
-        <is>
-          <t>$115</t>
+      <c r="D85" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -4620,26 +4620,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F85" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G85" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNTkIyV2h4TlA5eTFFY1hCMmYtU1ctR2tSUVBsbkpsU3F2RHRDSEtpdlJOOVgwdjJzVzF3YllrUmxrY2hpN19BVXczVDRMeXNjQTI5ZXNKS1M2MVVmTnpkUzZxUWdEOHZLVmdoSVllZzlsdXp1SVFDM0hHOVAzNWRVbExhUExtQXJ4WnBtWEIxX0h2dXdJWkk4akxJa2FETml3VFFPeEk5UDFtRDZlVTVZ0gGvAUFVX3lxTE1OQjJXaHhOUDl5MUVjWEIyZi1TVy1Ha1JRUGxuSmxTcXZEdENIS2l2Uk45WDB2MnNXMXdiWWtSbGtjaGk3X0FVdzNUNEx5c2NBMjllc0pLUzYxVWZOemRTNnFRZ0Q4dktWZ2hJWWVnOWx1enVJUUMzSEc5UDM1ZFVsTGFQTG1BcnhacG1YQjFfSHZ1d0laSThqTElrYUROaXdUUU94STlQMW1ENmVVNVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOYXRTM3V2MWdaYmp3M2FITldSbG8yRWhLdGhscE9wcGs3dEpVY21XVVRGRTllNEVIRlI0Ukwzb05FcmsxQnJMSHZsZGcwSVE5bGZTVDdmbHFNcmk3LUxnTG5kRVR4X1Vna25WYzVLZEp3OHE1bEdnUmRoX3NPQTRmMUZRYXJzV0MyUWJRMdIBjAFBVV95cUxOYXRTM3V2MWdaYmp3M2FITldSbG8yRWhLdGhscE9wcGs3dEpVY21XVVRGRTllNEVIRlI0Ukwzb05FcmsxQnJMSHZsZGcwSVE5bGZTVDdmbHFNcmk3LUxnTG5kRVR4X1Vna25WYzVLZEp3OHE1bEdnUmRoX3NPQTRmMUZRYXJzV0MyUWJRMQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>The Travis Scott Fragment Air Jordan 1 Is The Most Wanted Sneaker Release Of All Time - Sneaker News</t>
+          <t>Crocheted Swooshes Appear On This Air Jordan 1 Mid - Sneaker News</t>
         </is>
       </c>
       <c r="B86" s="26" t="inlineStr">
@@ -4652,9 +4652,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D86" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>$115</t>
         </is>
       </c>
       <c r="E86" s="17" t="inlineStr">
@@ -4662,31 +4662,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F86" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G86" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F86" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G86" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H86" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNdktzbHl1SlhFUndNYzV6ZDY5WEJiYmdHb0FkTmNXMU9mSVo5Q0dPcGFmS1RFS3h3amlWZFplUy1qb2tBUl9ISWgtQXdPVGsxMVN0MC1BMFVMalhTZmh0UDNsem93bjJ3VkdfSUt6R2tidzBja3NaNGRHRlpZN3pYSzJmcFB3MW01UTZQMEtTdFPSAZABQVVfeXFMTXZLc2x5dUpYRVJ3TWM1emQ2OVhCYmJnR29BZE5jVzFPZklaOUNHT3BhZktURUt4d2ppVmRaZVMtam9rQVJfSEloLUF3T1RrMTFTdDAtQTBVTGpYU2ZodFAzbHpvd24yd1ZHX0lLekdrYncwY2tzWjRkR0ZaWTd6WEsyZnBQdzFtNVE2UDBLU3RT?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNTkIyV2h4TlA5eTFFY1hCMmYtU1ctR2tSUVBsbkpsU3F2RHRDSEtpdlJOOVgwdjJzVzF3YllrUmxrY2hpN19BVXczVDRMeXNjQTI5ZXNKS1M2MVVmTnpkUzZxUWdEOHZLVmdoSVllZzlsdXp1SVFDM0hHOVAzNWRVbExhUExtQXJ4WnBtWEIxX0h2dXdJWkk4akxJa2FETml3VFFPeEk5UDFtRDZlVTVZ0gGvAUFVX3lxTE1OQjJXaHhOUDl5MUVjWEIyZi1TVy1Ha1JRUGxuSmxTcXZEdENIS2l2Uk45WDB2MnNXMXdiWWtSbGtjaGk3X0FVdzNUNEx5c2NBMjllc0pLUzYxVWZOemRTNnFRZ0Q4dktWZ2hJWWVnOWx1enVJUUMzSEc5UDM1ZFVsTGFQTG1BcnhacG1YQjFfSHZ1d0laSThqTElrYUROaXdUUU94STlQMW1ENmVVNVk?oc=5</t>
         </is>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>adidas Celebrates Atlanta’s 404 Day With The Superstar - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>The Travis Scott Fragment Air Jordan 1 Is The Most Wanted Sneaker Release Of All Time - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B87" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C87" s="22" t="inlineStr">
@@ -4704,31 +4704,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F87" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G87" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F87" s="42" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G87" s="43" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H87" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZ9IBfkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNdktzbHl1SlhFUndNYzV6ZDY5WEJiYmdHb0FkTmNXMU9mSVo5Q0dPcGFmS1RFS3h3amlWZFplUy1qb2tBUl9ISWgtQXdPVGsxMVN0MC1BMFVMalhTZmh0UDNsem93bjJ3VkdfSUt6R2tidzBja3NaNGRHRlpZN3pYSzJmcFB3MW01UTZQMEtTdFPSAZABQVVfeXFMTXZLc2x5dUpYRVJ3TWM1emQ2OVhCYmJnR29BZE5jVzFPZklaOUNHT3BhZktURUt4d2ppVmRaZVMtam9rQVJfSEloLUF3T1RrMTFTdDAtQTBVTGpYU2ZodFAzbHpvd24yd1ZHX0lLekdrYncwY2tzWjRkR0ZaWTd6WEsyZnBQdzFtNVE2UDBLU3RT?oc=5</t>
         </is>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>The New Balance P350 Basketball Shoe Debuts On February 11th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B88" s="31" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>adidas Celebrates Atlanta’s 404 Day With The Superstar - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C88" s="27" t="inlineStr">
@@ -4746,31 +4746,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F88" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G88" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G88" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H88" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBPckdQYi1najdwS0ozUmVvZHJDajdRQTRzN2RsT09zbi1pZmtWWm9MRDNDUDlnblAzblNSemlsMlUtNVFOejdxYzZBdkdJWVBpUTVZZTFRSHJ4UVVSMHE0UFdQWm5wYmhMRUQ5YWY1RnJTYVHSAXNBVV95cUxQT3JHUGItZ2o3cEtKM1Jlb2RyQ2o3UUE0czdkbE9Pc24taWZrVlpvTEQzQ1A5Z25QM25TUnppbDJVLTVRTno3cWM2QXZHSVlQaVE1WWUxUUhyeFFVUjBxNFBXUFpucGJoTEVEOWFmNUZyU2FR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZ9IBfkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>The Nike Structure Plus Launches February 5th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B89" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The New Balance P350 Basketball Shoe Debuts On February 11th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B89" s="38" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C89" s="22" t="inlineStr">
@@ -4788,26 +4788,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F89" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G89" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F89" s="39" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G89" s="40" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H89" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUdIBZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBPckdQYi1najdwS0ozUmVvZHJDajdRQTRzN2RsT09zbi1pZmtWWm9MRDNDUDlnblAzblNSemlsMlUtNVFOejdxYzZBdkdJWVBpUTVZZTFRSHJ4UVVSMHE0UFdQWm5wYmhMRUQ5YWY1RnJTYVHSAXNBVV95cUxQT3JHUGItZ2o3cEtKM1Jlb2RyQ2o3UUE0czdkbE9Pc24taWZrVlpvTEQzQ1A5Z25QM25TUnppbDJVLTVRTno3cWM2QXZHSVlQaVE1WWUxUUhyeFFVUjBxNFBXUFpucGJoTEVEOWFmNUZyU2FR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>The Nike First Sight Shadow Channels The Alpha Project Basketball Era - Sneaker News</t>
+          <t>The Nike Structure Plus Launches February 5th - Sneaker News</t>
         </is>
       </c>
       <c r="B90" s="35" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="H90" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUdIBckFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUdIBZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>Caitlin Clark’s Nike Kobe 5 Protro “Indiana Fever” Dropping In June - Sneaker News</t>
+          <t>The Nike First Sight Shadow Channels The Alpha Project Basketball Era - Sneaker News</t>
         </is>
       </c>
       <c r="B91" s="30" t="inlineStr">
@@ -4884,19 +4884,19 @@
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQQlhMZ0g0WWNOcFVQc2Y2NDdXUzZfVTVCQW1tY3ZhSHhXdGV1QmxiWEo1ZXN3YmJsN2d2QVhpbkE1QXpaUGVvendzYzBHVmREX1RoMFFEc25naEV1aFdWcFVIMkxHeWVqR2NBY0FOY0xDVk1TSVdKVDVVcVpGVTdkZ0VFQmFlVVNJMDRETTdlVzNFNkxsSGNNU9IBmAFBVV95cUxQQlhMZ0g0WWNOcFVQc2Y2NDdXUzZfVTVCQW1tY3ZhSHhXdGV1QmxiWEo1ZXN3YmJsN2d2QVhpbkE1QXpaUGVvendzYzBHVmREX1RoMFFEc25naEV1aFdWcFVIMkxHeWVqR2NBY0FOY0xDVk1TSVdKVDVVcVpGVTdkZ0VFQmFlVVNJMDRETTdlVzNFNkxsSGNNUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUdIBckFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>Bad Bunny Is Dropping His Own adidas Clothing Line - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B92" s="14" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Caitlin Clark’s Nike Kobe 5 Protro “Indiana Fever” Dropping In June - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B92" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C92" s="27" t="inlineStr">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="H92" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBibmZGRldoVjVka21ONWNCUktDajBteGNKa3kzcGltZ0pFNjFzSEI2d0paNTlzM1NkeXBzamFKay1LNTAtbEMxU09PRW9wWnVPbzFZZmtHWDhYalB0WjVoOVpTNlNZbTk0aFVWREpRM2tIMjVFbVlqZ2Z30gF6QVVfeXFMUGJuZkZGV2hWNWRrbU41Y0JSS0NqMG14Y0preTNwaW1nSkU2MXNIQjZ3Slo1OXMzU2R5cHNqYUprLUs1MC1sQzFTT09Fb3BadU9vMVlma0dYOFhqUHRaNWg5WlM2U1ltOTRoVVZESlEza0gyNUVtWWpnZnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQQlhMZ0g0WWNOcFVQc2Y2NDdXUzZfVTVCQW1tY3ZhSHhXdGV1QmxiWEo1ZXN3YmJsN2d2QVhpbkE1QXpaUGVvendzYzBHVmREX1RoMFFEc25naEV1aFdWcFVIMkxHeWVqR2NBY0FOY0xDVk1TSVdKVDVVcVpGVTdkZ0VFQmFlVVNJMDRETTdlVzNFNkxsSGNNU9IBmAFBVV95cUxQQlhMZ0g0WWNOcFVQc2Y2NDdXUzZfVTVCQW1tY3ZhSHhXdGV1QmxiWEo1ZXN3YmJsN2d2QVhpbkE1QXpaUGVvendzYzBHVmREX1RoMFFEc25naEV1aFdWcFVIMkxHeWVqR2NBY0FOY0xDVk1TSVdKVDVVcVpGVTdkZ0VFQmFlVVNJMDRETTdlVzNFNkxsSGNNUw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>The adidas Anthony Edwards 2 “Bulldawgs” Releases Ahead Of March Madness - Sneaker News</t>
+          <t>Bad Bunny Is Dropping His Own adidas Clothing Line - Sneaker News</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
@@ -4968,19 +4968,19 @@
       </c>
       <c r="H93" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCONIBgwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBibmZGRldoVjVka21ONWNCUktDajBteGNKa3kzcGltZ0pFNjFzSEI2d0paNTlzM1NkeXBzamFKay1LNTAtbEMxU09PRW9wWnVPbzFZZmtHWDhYalB0WjVoOVpTNlNZbTk0aFVWREpRM2tIMjVFbVlqZ2Z30gF6QVVfeXFMUGJuZkZGV2hWNWRrbU41Y0JSS0NqMG14Y0preTNwaW1nSkU2MXNIQjZ3Slo1OXMzU2R5cHNqYUprLUs1MC1sQzFTT09Fb3BadU9vMVlma0dYOFhqUHRaNWg5WlM2U1ltOTRoVVZESlEza0gyNUVtWWpnZnc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>Cooper Flagg Is Finally Dropping His First New Balance Shoe - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B94" s="31" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>The adidas Anthony Edwards 2 “Bulldawgs” Releases Ahead Of March Madness - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C94" s="27" t="inlineStr">
@@ -4998,26 +4998,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F94" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G94" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G94" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H94" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTzNpWjVHV2JLVHhnQllSeDZwbjYtZVU2c2dHVURTUWdCSVdyQU05Nzh2N0RfaDdKY1BqWW9fSVZ1US12OFI1YzNWemUwMDZEMVlRdlhfV2RuZEtmZDYwOC1sblhqSDFUdGRTZy1temN2QnA2SkdkWWpfQmNhblllN2FIZVFCcG1T0gGIAUFVX3lxTE5PM2laNUdXYktUeGdCWVJ4NnBuNi1lVTZzZ0dVRFNRZ0JJV3JBTTk3OHY3RF9oN0pjUGpZb19JVnVRLXY4UjVjM1Z6ZTAwNkQxWVF2WF9XZG5kS2ZkNjA4LWxuWGpIMVR0ZFNnLW16Y3ZCcDZKR2RZal9CY2FuWWU3YUhlUUJwbVM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCONIBgwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCOA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Easter Comes Early On The New Balance 2000 - Sneaker News</t>
+          <t>Cooper Flagg Is Finally Dropping His First New Balance Shoe - Sneaker News</t>
         </is>
       </c>
       <c r="B95" s="38" t="inlineStr">
@@ -5052,19 +5052,19 @@
       </c>
       <c r="H95" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1EQTk4ZjFuSF8yUndRR3g4SnRBeDd1V2V0eEs5MGZ6VGhtVEhkSVBQMDdoZXZ5dlNob1V4aUZucUVUcmRtdTZGeTdwV1FBR2VwZFZKelNlY2M2MVlQU2NpUmZtSTh3RHZoMmYyVzdUSFZpMTJEMkZV0gF3QVVfeXFMTURBOThmMW5IXzJSd1FHeDhKdEF4N3VXZXR4SzkwZnpUaG1USGRJUFAwN2hldnl2U2hvVXhpRm5xRVRyZG11NkZ5N3BXUUFHZXBkVkp6U2VjYzYxWVBTY2lSZm1JOHdEdmgyZjJXN1RIVmkxMkQyRlU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTzNpWjVHV2JLVHhnQllSeDZwbjYtZVU2c2dHVURTUWdCSVdyQU05Nzh2N0RfaDdKY1BqWW9fSVZ1US12OFI1YzNWemUwMDZEMVlRdlhfV2RuZEtmZDYwOC1sblhqSDFUdGRTZy1temN2QnA2SkdkWWpfQmNhblllN2FIZVFCcG1T0gGIAUFVX3lxTE5PM2laNUdXYktUeGdCWVJ4NnBuNi1lVTZzZ0dVRFNRZ0JJV3JBTTk3OHY3RF9oN0pjUGpZb19JVnVRLXY4UjVjM1Z6ZTAwNkQxWVF2WF9XZG5kS2ZkNjA4LWxuWGpIMVR0ZFNnLW16Y3ZCcDZKR2RZal9CY2FuWWU3YUhlUUJwbVM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Unveiled - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B96" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Easter Comes Early On The New Balance 2000 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B96" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C96" s="27" t="inlineStr">
@@ -5082,31 +5082,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F96" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G96" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F96" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G96" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H96" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE9iaUkzUDRSbVRzUE5sTlczbGNtbEZjRVFwb0JsTkRjMW9lQXRnZ2FjVlZUOWhFeFZsSUxnLW1URnl1S0tTdldXYnVfNlVBOUNlWkpoVHItaUFLcnhiellj0gFfQVVfeXFMT2JpSTNQNFJtVHNQTmxOVzNsY21sRmNFUXBvQmxORGMxb2VBdGdnYWNWVlQ5aEV4VmxJTGctbVRGeXVLS1N2V1didV82VUE5Q2VaSmhUci1pQUtyeGJ6WWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1EQTk4ZjFuSF8yUndRR3g4SnRBeDd1V2V0eEs5MGZ6VGhtVEhkSVBQMDdoZXZ5dlNob1V4aUZucUVUcmRtdTZGeTdwV1FBR2VwZFZKelNlY2M2MVlQU2NpUmZtSTh3RHZoMmYyVzdUSFZpMTJEMkZV0gF3QVVfeXFMTURBOThmMW5IXzJSd1FHeDhKdEF4N3VXZXR4SzkwZnpUaG1USGRJUFAwN2hldnl2U2hvVXhpRm5xRVRyZG11NkZ5N3BXUUFHZXBkVkp6U2VjYzYxWVBTY2lSZm1JOHdEdmgyZjJXN1RIVmkxMkQyRlU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2k4 “All-Star” Returning In 2026 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B97" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>It’s “Melo World” And The PUMA MB.05 Is Just Living In it - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B97" s="41" t="inlineStr">
+        <is>
+          <t>Puma</t>
         </is>
       </c>
       <c r="C97" s="22" t="inlineStr">
@@ -5124,31 +5124,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G97" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F97" s="39" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G97" s="40" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H97" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNMF9pQmlnZ0swQ2hxVk5NeXlfOUFnTGVwZllMWTZGQUw3TWE4TkR3c1VFc3A0R2NWdmMwNEVIUl9uLXd0SlNWbDVJOGlla1c2TXAwRmpQeVdVdGZvdTFTTHlnVjM1RGJhOE4tTFB3cHgyRE5naklVZmtwR09MQUZ3V05CbVrSAYQBQVVfeXFMTTBfaUJpZ2dLMENocVZOTXl5XzlBZ0xlcGZZTFk2RkFMN01hOE5Ed3NVRXNwNEdjVnZjMDRFSFJfbi13dEpTVmw1SThpZWtXNk1wMEZqUHlXVXRmb3UxU0x5Z1YzNURiYThOLUxQd3B4MkROZ2pJVWZrcEdPTEFGd1dOQm1a?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9VdmVOd0FPN3hQNXh5NEN5dGpBektnbS1vSlJFS2lBNVJKMHQxYy0wT0JRTDZ6YS02eXNWV2RaSlNDN095b0JyTnFLdlRIeDZxY295R2JDa1Buc0tUSktleUFSd05jaTFJWG0yOGxDeFlzLVJReWfSAXZBVV95cUxPVXZlTndBTzd4UDV4eTRDeXRqQXpLZ20tb0pSRUtpQTVSSjB0MWMtME9CUUw2emEtNnlzVldkWkpTQzdPeW9Cck5xS3ZUSHg2cWNveUdiQ2tQbnNLVEpLZXlBUndOY2kxSVhtMjhsQ3hZcy1SUXln?oc=5</t>
         </is>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>The New Balance 9060Z Puts On Two Night Vision Colorways - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B98" s="31" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>Nike LeBron 23 Unveiled - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B98" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C98" s="27" t="inlineStr">
@@ -5166,26 +5166,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F98" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G98" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G98" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H98" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5uWGpZMVVSN3ZiTVVSbzdMWXF6am5EVEdZckUxSmtBeFhZY0daQXNrMjRvMjA1WGNWWEVZc1hlel9ZOG5PRUY0TWpFUXctVTNpS3lpaGJ4dWYwQXlHVTBPZ0NiZ0c0Q2FUS2RWX1lEemJrZVHSAXNBVV95cUxOblhqWTFVUjd2Yk1VUm83TFlxempuRFRHWXJFMUprQXhYWWNHWkFzazI0bzIwNVhjVlhFWXNYZXpfWThuT0VGNE1qRVF3LVUzaUt5aWhieHVmMEF5R1UwT2dDYmdHNENhVEtkVl9ZRHpia2VR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE9iaUkzUDRSbVRzUE5sTlczbGNtbEZjRVFwb0JsTkRjMW9lQXRnZ2FjVlZUOWhFeFZsSUxnLW1URnl1S0tTdldXYnVfNlVBOUNlWkpoVHItaUFLcnhiellj0gFfQVVfeXFMT2JpSTNQNFJtVHNQTmxOVzNsY21sRmNFUXBvQmxORGMxb2VBdGdnYWNWVlQ5aEV4VmxJTGctbVRGeXVLS1N2V1didV82VUE5Q2VaSmhUci1pQUtyeGJ6WWM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>Official Images Of The Nike A’One “Indigo Girl” - Sneaker News</t>
+          <t>Nike Zoom Huarache 2k4 “All-Star” Returning In 2026 - Sneaker News</t>
         </is>
       </c>
       <c r="B99" s="30" t="inlineStr">
@@ -5220,19 +5220,19 @@
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1obUpQQWoxMExaOUl1N20tZllnMVdLbVJwX1FXcGprMmg1TjE1d2NkMzV3NW1wOHc4UWU1eHZtUDF2Z1V4MGFxUXF0WTJTZ0NoUnk1TW1sYmc1TElYSlJLcHNXcjZOWjVUMnFqZExGeHNNTlZ5c0HSAXZBVV95cUxNaG1KUEFqMTBMWjlJdTdtLWZZZzFXS21ScF9RV3BqazJoNU4xNXdjZDM1dzVtcDh3OFFlNXh2bVAxdmdVeDBhcVFxdFkyU2dDaFJ5NU1tbGJnNUxJWEpSS3BzV3I2Tlo1VDJxamRMRnhzTU5WeXNB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNMF9pQmlnZ0swQ2hxVk5NeXlfOUFnTGVwZllMWTZGQUw3TWE4TkR3c1VFc3A0R2NWdmMwNEVIUl9uLXd0SlNWbDVJOGlla1c2TXAwRmpQeVdVdGZvdTFTTHlnVjM1RGJhOE4tTFB3cHgyRE5naklVZmtwR09MQUZ3V05CbVrSAYQBQVVfeXFMTTBfaUJpZ2dLMENocVZOTXl5XzlBZ0xlcGZZTFk2RkFMN01hOE5Ed3NVRXNwNEdjVnZjMDRFSFJfbi13dEpTVmw1SThpZWtXNk1wMEZqUHlXVXRmb3UxU0x5Z1YzNURiYThOLUxQd3B4MkROZ2pJVWZrcEdPTEFGd1dOQm1a?oc=5</t>
         </is>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>YOASOBI’s “Just A Little Step” Turns Into An ASICS Sneaker Collaboration - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B100" s="32" t="inlineStr">
-        <is>
-          <t>ASICS</t>
+          <t>The New Balance 9060Z Puts On Two Night Vision Colorways - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B100" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C100" s="27" t="inlineStr">
@@ -5250,31 +5250,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F100" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G100" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F100" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G100" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H100" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB4Sm1iZVVLNE9LS1VTSkMwLWViNkE2R3gzZXhyWlVOeGFxdVhMY3pyZXl6enZjb0xYbk9nWkt5SXlKNGlNSVlubjB3NmwtU1h2M3gwZlN5dk42UVhPaDNXcmNJZVBoN3FzYUdlWmNZNlgzVTNiN2lz0gF3QVVfeXFMUHhKbWJlVUs0T0tLVVNKQzAtZWI2QTZHeDNleHJaVU54YXF1WExjenJleXp6dmNvTFhuT2daS3lJeUo0aU1JWW5uMHc2bC1TWHYzeDBmU3l2TjZRWE9oM1dyY0llUGg3cXNhR2VaY1k2WDNVM2I3aXM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5uWGpZMVVSN3ZiTVVSbzdMWXF6am5EVEdZckUxSmtBeFhZY0daQXNrMjRvMjA1WGNWWEVZc1hlel9ZOG5PRUY0TWpFUXctVTNpS3lpaGJ4dWYwQXlHVTBPZ0NiZ0c0Q2FUS2RWX1lEemJrZVHSAXNBVV95cUxOblhqWTFVUjd2Yk1VUm83TFlxempuRFRHWXJFMUprQXhYWWNHWkFzazI0bzIwNVhjVlhFWXNYZXpfWThuT0VGNE1qRVF3LVUzaUt5aWhieHVmMEF5R1UwT2dDYmdHNENhVEtkVl9ZRHpia2VR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Nike Mind 001 / 002, Jordan Luka 5, And This Week’s Best Releases - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B101" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Official Images Of The Nike A’One “Indigo Girl” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B101" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C101" s="22" t="inlineStr">
@@ -5292,31 +5292,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F101" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G101" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F101" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G101" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOdnkwZWZXT0REVVhjQnBXZzBVaGFPT3JDZGxCck12dHhwbXE2aDFUWDNfTWdyTTJpNnJwMzFqR2w1RkNrbFpkZExyQXRWMDU2UGpiSnA5T0V2MVNBcDRuVFcxeFNEd2U4eC1mLVNreHh6ZWlPVHE0cGJGYlF5SDV0amRnSkvSAYQBQVVfeXFMTnZ5MGVmV09ERFVYY0JwV2cwVWhhT09yQ2RsQnJNdnR4cG1xNmgxVFgzX01nck0yaTZycDMxakdsNUZDa2xaZGRMckF0VjA1NlBqYkpwOU9FdjFTQXA0blRXMXhTRHdlOHgtZi1Ta3h4emVpT1RxNHBiRmJReUg1dGpkZ0pL?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1obUpQQWoxMExaOUl1N20tZllnMVdLbVJwX1FXcGprMmg1TjE1d2NkMzV3NW1wOHc4UWU1eHZtUDF2Z1V4MGFxUXF0WTJTZ0NoUnk1TW1sYmc1TElYSlJLcHNXcjZOWjVUMnFqZExGeHNNTlZ5c0HSAXZBVV95cUxNaG1KUEFqMTBMWjlJdTdtLWZZZzFXS21ScF9RV3BqazJoNU4xNXdjZDM1dzVtcDh3OFFlNXh2bVAxdmdVeDBhcVFxdFkyU2dDaFJ5NU1tbGJnNUxJWEpSS3BzV3I2Tlo1VDJxamRMRnhzTU5WeXNB?oc=5</t>
         </is>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>Nike Ja 3 “Murray State” Launches On March 5th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B102" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>YOASOBI’s “Just A Little Step” Turns Into An ASICS Sneaker Collaboration - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B102" s="32" t="inlineStr">
+        <is>
+          <t>ASICS</t>
         </is>
       </c>
       <c r="C102" s="27" t="inlineStr">
@@ -5334,26 +5334,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F102" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G102" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F102" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G102" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H102" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOekNBTnN0OEJSY0ZWWXd5T3hDeVA0ZHlhWHJmWWRlUm5RU3VmSVg3UFM2blFpQm1Ic3VseGY2RC1QdEZEVXEzZml1WmFjVC00Q1FJYVpORjdVZjREMjNIalN2R25SbVVXNFhQbm04c25SSjNfYXVpTG02dmxaUGNCMHJzakthTGZ4RXfSAYoBQVVfeXFMTnpDQU5zdDhCUmNGVll3eU94Q3lQNGR5YVhyZllkZVJuUVN1ZklYN1BTNm5RaUJtSHN1bHhmNkQtUHRGRFVxM2ZpdVphY1QtNENRSWFaTkY3VWY0RDIzSGpTdkduUm1VVzRYUG5tOHNuUkozX2F1aUxtNnZsWlBjQjByc2pLYUxmeEV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB4Sm1iZVVLNE9LS1VTSkMwLWViNkE2R3gzZXhyWlVOeGFxdVhMY3pyZXl6enZjb0xYbk9nWkt5SXlKNGlNSVlubjB3NmwtU1h2M3gwZlN5dk42UVhPaDNXcmNJZVBoN3FzYUdlWmNZNlgzVTNiN2lz0gF3QVVfeXFMUHhKbWJlVUs0T0tLVVNKQzAtZWI2QTZHeDNleHJaVU54YXF1WExjenJleXp6dmNvTFhuT2daS3lJeUo0aU1JWW5uMHc2bC1TWHYzeDBmU3l2TjZRWE9oM1dyY0llUGg3cXNhR2VaY1k2WDNVM2I3aXM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Wolf Grey” Postponed To February 28th - Sneaker News</t>
+          <t>Nike Mind 001 / 002, Jordan Luka 5, And This Week’s Best Releases - Sneaker News</t>
         </is>
       </c>
       <c r="B103" s="21" t="inlineStr">
@@ -5366,9 +5366,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D103" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D103" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
@@ -5388,14 +5388,14 @@
       </c>
       <c r="H103" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1xZHFjb1Q4RmZpbXB4cTFoblVaZmJOUUFVZEtWWWttelpYSGN4czg2bGx4WVN2Z1hWTkQ2bnNvbVhHbFcybmdDLXlCd29fNVNRYU9GVXItdnc0MjV2TFhwamY1MWpFQlJTSmNlNmN0d1VzSUNEc0V2dFFYUnI3RTjSAX9BVV95cUxNcWRxY29UOEZmaW1weHExaG5VWmZiTlFBVWRLVllrbXpaWEhjeHM4NmxseFlTdmdYVk5ENm5zb21YR2xXMm5nQy15QndvXzVTUWFPRlVyLXZ3NDI1dkxYcGpmNTFqRUJSU0pjZTZjdHdVc0lDRHNFdnRRWFJyN0U4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOdnkwZWZXT0REVVhjQnBXZzBVaGFPT3JDZGxCck12dHhwbXE2aDFUWDNfTWdyTTJpNnJwMzFqR2w1RkNrbFpkZExyQXRWMDU2UGpiSnA5T0V2MVNBcDRuVFcxeFNEd2U4eC1mLVNreHh6ZWlPVHE0cGJGYlF5SDV0amRnSkvSAYQBQVVfeXFMTnZ5MGVmV09ERFVYY0JwV2cwVWhhT09yQ2RsQnJNdnR4cG1xNmgxVFgzX01nck0yaTZycDMxakdsNUZDa2xaZGRMckF0VjA1NlBqYkpwOU9FdjFTQXA0blRXMXhTRHdlOHgtZi1Ta3h4emVpT1RxNHBiRmJReUg1dGpkZ0pL?oc=5</t>
         </is>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>The Nike Mind 002 “Black/Hyper Crimson” Releases On February 5th - Sneaker News</t>
+          <t>Nike Ja 3 “Murray State” Launches On March 5th - Sneaker News</t>
         </is>
       </c>
       <c r="B104" s="35" t="inlineStr">
@@ -5430,19 +5430,19 @@
       </c>
       <c r="H104" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOcTYtWWhHTGk4T09CbElTMFpzT3J3dUF0OGxrNEVtY3AxeHRYRjc2WDVfQXlxQllnQzM4UXlGVHd5Y3d0NHdCTHZHS2kzSHZ1VEFGWi03UFJEUS01cG5ySGl2UGVjWlZ0OGpwSE5rdHgzZ3B0TW5kZ3p2Z3piV3ltOHdPczVyZ3NneFduWm1nMnDSAZABQVVfeXFMTnE2LVloR0xpOE9PQmxJUzBac09yd3VBdDhsazRFbWNwMXh0WEY3Nlg1X0F5cUJZZ0MzOFF5RlR3eWN3dDR3Qkx2R0tpM0h2dVRBRlotN1BSRFEtNXBuckhpdlBlY1pWdDhqcEhOa3R4M2dwdE1uZGd6dmd6Yld5bTh3T3M1cmdzZ3hXblptZzJw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxOekNBTnN0OEJSY0ZWWXd5T3hDeVA0ZHlhWHJmWWRlUm5RU3VmSVg3UFM2blFpQm1Ic3VseGY2RC1QdEZEVXEzZml1WmFjVC00Q1FJYVpORjdVZjREMjNIalN2R25SbVVXNFhQbm04c25SSjNfYXVpTG02dmxaUGNCMHJzakthTGZ4RXfSAYoBQVVfeXFMTnpDQU5zdDhCUmNGVll3eU94Q3lQNGR5YVhyZllkZVJuUVN1ZklYN1BTNm5RaUJtSHN1bHhmNkQtUHRGRFVxM2ZpdVphY1QtNENRSWFaTkY3VWY0RDIzSGpTdkduUm1VVzRYUG5tOHNuUkozX2F1aUxtNnZsWlBjQjByc2pLYUxmeEV3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 “Hyper Crimson” Is Available Now - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B105" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Air Jordan 5 “Wolf Grey” Postponed To February 28th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B105" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C105" s="22" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>$110</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
@@ -5460,26 +5460,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F105" s="42" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G105" s="43" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F105" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G105" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H105" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQb2RIdkRFNmlXWWIybWQxWTRjOVdhUlVFUTJ2TXpyNHR4RlhyZ3FTQnQtS3FkekhwdGYwZ1RzLU1qcHV0V0thSDRJbVgtR3M1ZFJsb0p6Ny1Cbi1fZDRXajhldGZtN2xqNjhTazNORkpIYkhkZFdMVTk1U2FnUFNxMklyNWMxcnB4VVlB0gGLAUFVX3lxTFBvZEh2REU2aVdZYjJtZDFZNGM5V2FSVUVRMnZNenI0dHhGWHJncVNCdC1LcWR6SHB0ZjBnVHMtTWpwdXRXS2FINEltWC1HczVkUmxvSno3LUJuLV9kNFdqOGV0Zm03bGo2OFNrM05GSkhiSGRkV0xVOTVTYWdQU3EySXI1YzFycHhVWUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1xZHFjb1Q4RmZpbXB4cTFoblVaZmJOUUFVZEtWWWttelpYSGN4czg2bGx4WVN2Z1hWTkQ2bnNvbVhHbFcybmdDLXlCd29fNVNRYU9GVXItdnc0MjV2TFhwamY1MWpFQlJTSmNlNmN0d1VzSUNEc0V2dFFYUnI3RTjSAX9BVV95cUxNcWRxY29UOEZmaW1weHExaG5VWmZiTlFBVWRLVllrbXpaWEhjeHM4NmxseFlTdmdYVk5ENm5zb21YR2xXMm5nQy15QndvXzVTUWFPRlVyLXZ3NDI1dkxYcGpmNTFqRUJSU0pjZTZjdHdVc0lDRHNFdnRRWFJyN0U4?oc=5</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>Nike Is Releasing A Triple White Ja 2 - Sneaker News</t>
+          <t>The Nike Mind 002 “Black/Hyper Crimson” Releases On February 5th - Sneaker News</t>
         </is>
       </c>
       <c r="B106" s="35" t="inlineStr">
@@ -5514,19 +5514,19 @@
       </c>
       <c r="H106" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBmUWxueWp2bV81VFRzTDd6SkpnNE4xbGx1RmRuNFF1blNWYlRWMDNYR1BtbU9WcEpzd3JnMEw2aWhTRk9zWWktOXJ0YnBiMEFudjR4MFVMdkhhb2FUdEJ1ZWVBbTFDQjFsZ0hpSG9tOEJNLU1Zc09R0gF3QVVfeXFMUGZRbG55anZtXzVUVHNMN3pKSmc0TjFsbHVGZG40UXVuU1ZiVFYwM1hHUG1tT1ZwSnN3cmcwTDZpaFNGT3NZaS05cnRicGIwQW52NHgwVUx2SGFvYVR0QnVlZUFtMUNCMWxnSGlIb204Qk0tTVlzT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOcTYtWWhHTGk4T09CbElTMFpzT3J3dUF0OGxrNEVtY3AxeHRYRjc2WDVfQXlxQllnQzM4UXlGVHd5Y3d0NHdCTHZHS2kzSHZ1VEFGWi03UFJEUS01cG5ySGl2UGVjWlZ0OGpwSE5rdHgzZ3B0TW5kZ3p2Z3piV3ltOHdPczVyZ3NneFduWm1nMnDSAZABQVVfeXFMTnE2LVloR0xpOE9PQmxJUzBac09yd3VBdDhsazRFbWNwMXh0WEY3Nlg1X0F5cUJZZ0MzOFF5RlR3eWN3dDR3Qkx2R0tpM0h2dVRBRlotN1BSRFEtNXBuckhpdlBlY1pWdDhqcEhOa3R4M2dwdE1uZGd6dmd6Yld5bTh3T3M1cmdzZ3hXblptZzJw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>Travis Scott Shoes, “Valentine” Jordan 3, And This Week’s Best Releases - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B107" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Patta x Nike Air Max 1 “Hyper Crimson” Is Available Now - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B107" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C107" s="22" t="inlineStr">
@@ -5534,9 +5534,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D107" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D107" s="8" t="inlineStr">
+        <is>
+          <t>$110</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
@@ -5556,14 +5556,14 @@
       </c>
       <c r="H107" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUdIBhgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQb2RIdkRFNmlXWWIybWQxWTRjOVdhUlVFUTJ2TXpyNHR4RlhyZ3FTQnQtS3FkekhwdGYwZ1RzLU1qcHV0V0thSDRJbVgtR3M1ZFJsb0p6Ny1Cbi1fZDRXajhldGZtN2xqNjhTazNORkpIYkhkZFdMVTk1U2FnUFNxMklyNWMxcnB4VVlB0gGLAUFVX3lxTFBvZEh2REU2aVdZYjJtZDFZNGM5V2FSVUVRMnZNenI0dHhGWHJncVNCdC1LcWR6SHB0ZjBnVHMtTWpwdXRXS2FINEltWC1HczVkUmxvSno3LUJuLV9kNFdqOGV0Zm03bGo2OFNrM05GSkhiSGRkV0xVOTVTYWdQU3EySXI1YzFycHhVWUE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>Nike Prepares For April Showers With A New Batch Of Air Force 1 Vibram Options - Sneaker News</t>
+          <t>Nike Is Releasing A Triple White Ja 2 - Sneaker News</t>
         </is>
       </c>
       <c r="B108" s="35" t="inlineStr">
@@ -5598,14 +5598,14 @@
       </c>
       <c r="H108" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CN9IBgAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBmUWxueWp2bV81VFRzTDd6SkpnNE4xbGx1RmRuNFF1blNWYlRWMDNYR1BtbU9WcEpzd3JnMEw2aWhTRk9zWWktOXJ0YnBiMEFudjR4MFVMdkhhb2FUdEJ1ZWVBbTFDQjFsZ0hpSG9tOEJNLU1Zc09R0gF3QVVfeXFMUGZRbG55anZtXzVUVHNMN3pKSmc0TjFsbHVGZG40UXVuU1ZiVFYwM1hHUG1tT1ZwSnN3cmcwTDZpaFNGT3NZaS05cnRicGIwQW52NHgwVUx2SGFvYVR0QnVlZUFtMUNCMWxnSGlIb204Qk0tTVlzT1E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>Detailed Look At The Paris Saint-Germain x Air Jordan 6 - Sneaker News</t>
+          <t>Travis Scott Shoes, “Valentine” Jordan 3, And This Week’s Best Releases - Sneaker News</t>
         </is>
       </c>
       <c r="B109" s="21" t="inlineStr">
@@ -5618,9 +5618,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D109" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D109" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
@@ -5628,31 +5628,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F109" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G109" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F109" s="42" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G109" s="43" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H109" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE44ZFVoWFRjQTREMXVva2o4S1lQX004N09PbFZNN0RmSkhiRUNxQkJGYldTVEJuSEdLX1g2dHJidmNOV1hNNVQzVEFDUDBZYy0wTXU1dzd2dzN1Wm5LMVhIU0FUUnp5emlsa0FxYjhyZGfSAXBBVV95cUxOOGRVaFhUY0E0RDF1b2tqOEtZUF9NODdPT2xWTTdEZkpIYkVDcUJCRmJXU1RCbkhHS19YNnRyYnZjTldYTTVUM1RBQ1AwWWMtME11NXc3dnczdVpuSzFYSFNBVFJ6eXppbGtBcWI4cmRn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUdIBhgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>Where To Buy The Air Jordan 1 “All-Star” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B110" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Prepares For April Showers With A New Batch Of Air Force 1 Vibram Options - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B110" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C110" s="27" t="inlineStr">
@@ -5670,31 +5670,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F110" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G110" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G110" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H110" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1FLW1lUEs3dWMxX0MzZFJaMUF2Wmp1clV3bk92VDNqbDN4LXFHOE0xZkRJYl9VVlRiSzJKZE5RVnlYWVZZaU1xR2IzSDAtR3NycHI3VE02UmJGcHNDWWFkem1nSkRqSTlZQVpFQnZ6czQ0aFdOeG930gF3QVVfeXFMTUUtbWVQSzd1YzFfQzNkUloxQXZaanVyVXduT3ZUM2psM3gtcUc4TTFmREliX1VWVGJLMkpkTlFWeVhZVllpTXFHYjNIMC1Hc3JwcjdUTTZSYkZwc0NZYWR6bWdKRGpJOVlBWkVCdnpzNDRoV054b3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CN9IBgAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CNw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>Paul Rodriguez Previews Upcoming Nike SB P-Rod 1 Drops For 2026 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B111" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Detailed Look At The Paris Saint-Germain x Air Jordan 6 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B111" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C111" s="22" t="inlineStr">
@@ -5702,9 +5702,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D111" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D111" s="8" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
@@ -5712,19 +5712,19 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F111" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G111" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F111" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G111" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H111" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBPVHg0cElyWDdpZmZveXFOUzl6cHNLUVFmaHNuQ0g5X0NjY2F3M3c0OXBiYjJETGZtbG9QQldUS09BUThaOHk3ZFZ4cVhyNkZjNDFFT3NraGNFbUlwMWFWQS05dXEyZWvSAWdBVV95cUxQT1R4NHBJclg3aWZmb3lxTlM5enBzS1FRZmhzbkNIOV9DY2NhdzN3NDlwYmIyRExmbWxvUEJXVEtPQVE4Wjh5N2RWeHFYcjZGYzQxRU9za2hjRW1JcDFhVkEtOXVxMmVr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE44ZFVoWFRjQTREMXVva2o4S1lQX004N09PbFZNN0RmSkhiRUNxQkJGYldTVEJuSEdLX1g2dHJidmNOV1hNNVQzVEFDUDBZYy0wTXU1dzd2dzN1Wm5LMVhIU0FUUnp5emlsa0FxYjhyZGfSAXBBVV95cUxOOGRVaFhUY0E0RDF1b2tqOEtZUF9NODdPT2xWTTdEZkpIYkVDcUJCRmJXU1RCbkhHS19YNnRyYnZjTldYTTVUM1RBQ1AwWWMtME11NXc3dnczdVpuSzFYSFNBVFJ6eXppbGtBcWI4cmRn?oc=5</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="53" t="inlineStr">
         <is>
-          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  06:55 AM</t>
+          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  06:56 AM</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7155,7 @@
         </is>
       </c>
       <c r="B9" s="62" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
@@ -7175,7 +7175,7 @@
         </is>
       </c>
       <c r="B10" s="64" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
@@ -7215,7 +7215,7 @@
         </is>
       </c>
       <c r="B12" s="64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
@@ -7255,11 +7255,11 @@
         </is>
       </c>
       <c r="B14" s="64" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>4.0 / 5</t>
+        <v>4</v>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>3.0 / 5</t>
         </is>
       </c>
       <c r="D14" s="70" t="inlineStr">
@@ -7295,7 +7295,7 @@
         </is>
       </c>
       <c r="B16" s="64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
@@ -7389,11 +7389,11 @@
         </is>
       </c>
       <c r="C22" s="64" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D22" s="70" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>10%</t>
         </is>
       </c>
     </row>
@@ -7409,11 +7409,11 @@
         </is>
       </c>
       <c r="C23" s="62" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D23" s="66" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>47%</t>
         </is>
       </c>
     </row>
@@ -7429,11 +7429,11 @@
         </is>
       </c>
       <c r="C24" s="64" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D24" s="70" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: scrape update — 137 releases [2026-03-15 07:12 UTC]
</commit_message>
<xml_diff>
--- a/reports/sneaker_releases.xlsx
+++ b/reports/sneaker_releases.xlsx
@@ -1107,7 +1107,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  07:09 AM</t>
+          <t>🔥  SNEAKER RELEASE TRACKER   ·   March 15, 2026  07:12 AM</t>
         </is>
       </c>
     </row>
@@ -2584,12 +2584,12 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Behold The Nike Air Max 1000, A 3D-Printed Re-imagination Of The Air Max 1 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>BOTTER And Reebok Join Forces For A Wild 3D-Printed Shoe - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="C37" s="22" t="inlineStr">
@@ -2597,9 +2597,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>$110</t>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -2607,26 +2607,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G37" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F37" s="41" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G37" s="42" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1wcERqSnJvZlV0U3B0YXBuSWJvRm8xWDJuZVFXMnBKdVZyblRXZzktbW5KYkM2MVBVV3R0ZDBJNVVfLWhpTUh3UmgySTd5RGNFWTFaVDFvSHNOMTltSnBmZzlvb9IBY0FVX3lxTE1wcERqSnJvZlV0U3B0YXBuSWJvRm8xWDJuZVFXMnBKdVZyblRXZzktbW5KYkM2MVBVV3R0ZDBJNVVfLWhpTUh3UmgySTd5RGNFWTFaVDFvSHNOMTltSnBmZzlvbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBHZGJjbTVIVHc5YU9jLUxHSDIxVlpxOUhmdW5FbmFzTTd5V0p6OVJVdEdVNmdJXy10ckdpYUFFdkZKQTZZNXJhZzVEMUZCWUFYXzhEZDg0RGdWbGJ2VUItSXlHdU8zMnN4OFY1Z21LZ3J1Wl9f0gF0QVVfeXFMUEdkYmNtNUhUdzlhT2MtTEdIMjFWWnE5SGZ1bkVuYXNNN3lXSno5UlV0R1U2Z0lfLXRyR2lhQUV2RkpBNlk1cmFnNUQxRkJZQVhfOERkODREZ1ZsYnZVQi1JeUd1TzMyc3g4VjVnbUtncnVaX18?oc=5</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Nike Already Has Liquid Max Collaborations Ready, And It’s With Fragment Design - Sneaker News</t>
+          <t>Behold The Nike Air Max 1000, A 3D-Printed Re-imagination Of The Air Max 1 - Sneaker News</t>
         </is>
       </c>
       <c r="B38" s="35" t="inlineStr">
@@ -2639,9 +2639,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D38" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>$110</t>
         </is>
       </c>
       <c r="E38" s="17" t="inlineStr">
@@ -2649,26 +2649,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F38" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G38" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H38" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOODNETVAwMVo1S2NrMmxSbng4MFFtVDRva2JIcm0yOTRPZDB1Rnp3bVEwT0Vrb1QtWWgyaEpJVjBxdEJRamJWT1dWODBDMjJOaTFIMmFxeDU5NVBWUl81ZnFVbXV5RHlMQlZhYW9DYU9TSFFNLU5QOF91TE5QQ0hRcWh4aHPSAYQBQVVfeXFMTjgzRE1QMDFaNUtjazJsUm54ODBRbVQ0b2tiSHJtMjk0T2QwdUZ6d21RME9Fa29ULVloMmhKSVYwcXRCUWpiVk9XVjgwQzIyTmkxSDJhcXg1OTVQVlJfNWZxVW11eUR5TEJWYWFvQ2FPU0hRTS1OUDhfdUxOUENIUXFoeGhz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE1wcERqSnJvZlV0U3B0YXBuSWJvRm8xWDJuZVFXMnBKdVZyblRXZzktbW5KYkM2MVBVV3R0ZDBJNVVfLWhpTUh3UmgySTd5RGNFWTFaVDFvSHNOMTltSnBmZzlvb9IBY0FVX3lxTE1wcERqSnJvZlV0U3B0YXBuSWJvRm8xWDJuZVFXMnBKdVZyblRXZzktbW5KYkM2MVBVV3R0ZDBJNVVfLWhpTUh3UmgySTd5RGNFWTFaVDFvSHNOMTltSnBmZzlvbw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Exclusive Look At The Upcoming Nike Air Max 1000 - Sneaker News</t>
+          <t>Nike Already Has Liquid Max Collaborations Ready, And It’s With Fragment Design - Sneaker News</t>
         </is>
       </c>
       <c r="B39" s="30" t="inlineStr">
@@ -2681,9 +2681,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>$110</t>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -2691,26 +2691,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G39" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F39" s="38" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G39" s="39" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9reWhTdEdNdEVKZ09OcWRialplYVdMWTgzcXdVNzU4UEJKUkl6MndQZGxTNWhudXhWdFBuNUFIdlhCWHpjRlBvYmQzWXZpN1FCU2pwa1l6MDhtczBrRmtuc0ozRHFTbWhmYVhydlViRnhvMVh3V2wxY1h3RVXSAXxBVV95cUxPa3loU3RHTXRFSmdPTnFkYmpaZWFXTFk4M3F3VTc1OFBCSlJJejJ3UGRsUzVobnV4VnRQbjVBSHZYQlh6Y0ZQb2JkM1l2aTdRQlNqcGtZejA4bXMwa0ZrbnNKM0RxU21oZmFYcnZVYkZ4bzFYd1dsMWNYd0VV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOODNETVAwMVo1S2NrMmxSbng4MFFtVDRva2JIcm0yOTRPZDB1Rnp3bVEwT0Vrb1QtWWgyaEpJVjBxdEJRamJWT1dWODBDMjJOaTFIMmFxeDU5NVBWUl81ZnFVbXV5RHlMQlZhYW9DYU9TSFFNLU5QOF91TE5QQ0hRcWh4aHPSAYQBQVVfeXFMTjgzRE1QMDFaNUtjazJsUm54ODBRbVQ0b2tiSHJtMjk0T2QwdUZ6d21RME9Fa29ULVloMmhKSVYwcXRCUWpiVk9XVjgwQzIyTmkxSDJhcXg1OTVQVlJfNWZxVW11eUR5TEJWYWFvQ2FPU0hRTS1OUDhfdUxOUENIUXFoeGhz?oc=5</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Of Course England Gets An Nike Air Max 95 For The World Cup - Sneaker News</t>
+          <t>Exclusive Look At The Upcoming Nike Air Max 1000 - Sneaker News</t>
         </is>
       </c>
       <c r="B40" s="35" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$110</t>
         </is>
       </c>
       <c r="E40" s="17" t="inlineStr">
@@ -2733,31 +2733,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F40" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G40" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F40" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G40" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H40" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQT0JBU2tTSmdEc0NoZWxmaUNrOVR5dm93LUpOQXBCakwzdTJPNzQ4M0NNWnU2b1VZc19FZldFSDRqY3VOQUNVV0RJRlRPYktBU2F6QnhMNHVlY2xrSFEtLVZ4U2V2SU1Bc0JwcWlvUjdXUnlXWmNfUEpySGFqdFBtT2psNmt5ZmvSAYcBQVVfeXFMUE9CQVNrU0pnRHNDaGVsZmlDazlUeXZvdy1KTkFwQmpMM3UyTzc0ODNDTVp1Nm9VWXNfRWZXRUg0amN1TkFDVVdESUZUT2JLQVNhekJ4TDR1ZWNsa0hRLS1WeFNldklNQXNCcHFpb1I3V1J5V1pjX1BKckhhanRQbU9qbDZreWZr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9reWhTdEdNdEVKZ09OcWRialplYVdMWTgzcXdVNzU4UEJKUkl6MndQZGxTNWhudXhWdFBuNUFIdlhCWHpjRlBvYmQzWXZpN1FCU2pwa1l6MDhtczBrRmtuc0ozRHFTbWhmYVhydlViRnhvMVh3V2wxY1h3RVXSAXxBVV95cUxPa3loU3RHTXRFSmdPTnFkYmpaZWFXTFk4M3F3VTc1OFBCSlJJejJ3UGRsUzVobnV4VnRQbjVBSHZYQlh6Y0ZQb2JkM1l2aTdRQlNqcGtZejA4bXMwa0ZrbnNKM0RxU21oZmFYcnZVYkZ4bzFYd1dsMWNYd0VV?oc=5</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>No, These Jordan Trunners Aren’t Action Bronson Collabs - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B41" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Of Course England Gets An Nike Air Max 95 For The World Cup - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C41" s="22" t="inlineStr">
@@ -2765,9 +2765,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D41" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>$160</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -2775,31 +2775,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F41" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G41" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9ENUxlRXd3bkJKeTBveTlSUnFfUDNEbTZ2WkxFdjJ1NnloRDRIZUNHaTY3R0l5dFNPUWRDckNyQ0FJOU5WWU5sRmUzZHBHR1U2aEVzYVNwRGlIYzZGVEh1NEtBVzdBelpVRkl6Ynk5MHozdjJjT1hz0gF3QVVfeXFMT0Q1TGVFd3duQkp5MG95OVJScV9QM0RtNnZaTEV2MnU2eWhENEhlQ0dpNjdHSXl0U09RZENyQ3JDQUk5TlZZTmxGZTNkcEdHVTZoRXNhU3BEaUhjNkZUSHU0S0FXN0F6WlVGSXpieTkwejN2MmNPWHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQT0JBU2tTSmdEc0NoZWxmaUNrOVR5dm93LUpOQXBCakwzdTJPNzQ4M0NNWnU2b1VZc19FZldFSDRqY3VOQUNVV0RJRlRPYktBU2F6QnhMNHVlY2xrSFEtLVZ4U2V2SU1Bc0JwcWlvUjdXUnlXWmNfUEpySGFqdFBtT2psNmt5ZmvSAYcBQVVfeXFMUE9CQVNrU0pnRHNDaGVsZmlDazlUeXZvdy1KTkFwQmpMM3UyTzc0ODNDTVp1Nm9VWXNfRWZXRUg0amN1TkFDVVdESUZUT2JLQVNhekJ4TDR1ZWNsa0hRLS1WeFNldklNQXNCcHFpb1I3V1J5V1pjX1BKckhhanRQbU9qbDZreWZr?oc=5</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>First Look At The Nike Kobe 8 Protro “Mambacurial” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B42" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Salehe Bembury – Collaborations &amp; 2025 Releases - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
       <c r="C42" s="27" t="inlineStr">
@@ -2817,26 +2817,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F42" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G42" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>★☆☆☆☆  1/5</t>
+        </is>
+      </c>
+      <c r="G42" s="43" t="inlineStr">
+        <is>
+          <t>⚪ General Release</t>
         </is>
       </c>
       <c r="H42" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNeXlHVUdiNHhkRmVpZ1VscjREV0NoY2hwX2pScG0tSnJIWHZmWWtGQXctUUFVTVVrX29OanZIeHB6eHVjYldENk9nNVJQTHQySlQ2ZkRGSmNqQ0RKaXlPeFdvRXBwZWFJZnVOZndMV3pqS01YQkVHTDFnOExvYjJERkJtUjhrb0wzeG5OUnU4WDNlMllU0gGUAUFVX3lxTE15eUdVR2I0eGRGZWlnVWxyNERXQ2hjaHBfalJwbS1KckhYdmZZa0ZBdy1RQVVNVWtfb05qdkh4cHp4dWNiV0Q2T2c1UlBMdDJKVDZmREZKY2pDREppeU94V29FcHBlYUlmdU5md0xXempLTVhCRUdMMWc4TG9iMkRGQm1SOGtvTDN4bk5SdThYM2UyWVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9qWjA2bFFkcnhsUHhLQ3gyemp0cFhHaTFOb2t1NDZuOVFyTHVLdUZzWnU5UklTY0IyUE85aWRQcVlhaVpRRlVZUVdNRmIwQ1JLSWRqemVn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Jordan Brand Preps For Graduation Season With The Air Jordan 6 “Cap And Gown” - Sneaker News</t>
+          <t>No, These Jordan Trunners Aren’t Action Bronson Collabs - Sneaker News</t>
         </is>
       </c>
       <c r="B43" s="21" t="inlineStr">
@@ -2849,9 +2849,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -2871,19 +2871,19 @@
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBVbFZaUlNQWFcyemItamVtR0hsd2R4UHZreVFhOGV5T1JRanctZ0RRQ0J5dGNjOFlXUldRYWFGXzZDUW9JMXB1NzJ1Nm9HMkd1N2hNcTNMSDlKdHd6anJVQXZFSWpMZTFicDJ1UkNB0gFuQVVfeXFMUFVsVlpSU1BYVzJ6Yi1qZW1HSGx3ZHhQdmt5UWE4ZXlPUlFqdy1nRFFDQnl0Y2M4WVdSV1FhYUZfNkNRb0kxcHU3MnU2b0cyR3U3aE1xM0xIOUp0d3pqclVBdkVJakxlMWJwMnVSQ0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9ENUxlRXd3bkJKeTBveTlSUnFfUDNEbTZ2WkxFdjJ1NnloRDRIZUNHaTY3R0l5dFNPUWRDckNyQ0FJOU5WWU5sRmUzZHBHR1U2aEVzYVNwRGlIYzZGVEh1NEtBVzdBelpVRkl6Ynk5MHozdjJjT1hz0gF3QVVfeXFMT0Q1TGVFd3duQkp5MG95OVJScV9QM0RtNnZaTEV2MnU2eWhENEhlQ0dpNjdHSXl0U09RZENyQ3JDQUk5TlZZTmxGZTNkcEdHVTZoRXNhU3BEaUhjNkZUSHU0S0FXN0F6WlVGSXpieTkwejN2MmNPWHM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>The Nike Air Force 1 Low Odes To Team USA - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B44" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>First Look At The Air Jordan 1 “Baroque Brown” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C44" s="27" t="inlineStr">
@@ -2891,9 +2891,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>$100</t>
+      <c r="D44" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E44" s="17" t="inlineStr">
@@ -2901,31 +2901,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F44" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G44" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F44" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G44" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H44" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQcGVCSmxsMEVsRFJMU281VzVpa0ZJT01abGl1YldaVXZXQUxWRzVxblpnSnhVU3RXMGh4dXJxdEYzNTdWaWFwR2ZoLVdnUVJ3b2RkS0s2TWZQMUhIOUdQcEFVVTRLdEthSVVzYl8tSlZ1Vll1MTh2Rkh5SmhTRDZjUkh30gGCAUFVX3lxTFBwZUJKbGwwRWxEUkxTbzVXNWlrRklPTVpsaXViV1pVdldBTFZHNXFuWmdKeFVTdFcwaHh1cnF0RjM1N1ZpYXBHZmgtV2dRUndvZGRLSzZNZlAxSEg5R1BwQVVVNEt0S2FJVXNiXy1KVnVWWXUxOHZGSHlKaFNENmNSSHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPVnV4Y043SkZUTHJobW9NM1VYTjBMeGFfQU1rSjR1T3h0akpfV2o5bU5GaUxwWDBkYkNsTkJDdzZnYk5fRmpWYzJmeDE5WEtNMm5NZnNVck1CTE1TVUZBOVpsWlZEdmFkRDR1TDZIOHF5TGhicFlEWjVwdVdta3Bfd1dnRW1BazVxNnBnTWJjNmLSAZABQVVfeXFMT1Z1eGNON0pGVExyaG1vTTNVWE4wTHhhX0FNa0o0dU94dGpKX1dqOW1ORmlMcFgwZGJDbE5CQ3c2Z2JOX0ZqVmMyZngxOVhLTTJuTWZzVXJNQkxNU1VGQTlabFpWRHZhZEQ0dUw2SDhxeUxoYnBZRFo1cHVXbWtwX3dXZ0VtQWs1cTZwZ01iYzZi?oc=5</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>The Nike Air Tech Challenge II “Pixel Court” Returns August 30th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Nike Adds A Sequined Swoosh To This Denim Air Jordan 1 Low For Kids - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B45" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C45" s="22" t="inlineStr">
@@ -2933,9 +2933,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D45" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>$100</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -2943,26 +2943,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G45" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G45" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQRURBSi1KcWNMRTExQ3VwQ0wwTVNlWHhVWS10eDZrLWNGSHdMWEJlbXFWX2kzYXFuZWk2dE85cVFzZ2RFbWJSSTQzS295bl9vMGdneXFIcVJiV3AwcXh6bzRwWndWcWg1X3FpamtMNGlCdVZVZWJqZ3FyQnF5Z2doX0tnSmxZT1pvb0w0X2hR0gGOAUFVX3lxTFBFREFKLUpxY0xFMTFDdXBDTDBNU2VYeFVZLXR4NmstY0ZId0xYQmVtcVZfaTNhcW5laTZ0TzlxUXNnZEVtYlJJNDNLb3luX28wZ2d5cUhxUmJXcDBxeHpvNHBad1ZxaDVfcWlqa0w0aUJ1VlVlYmpncXJCcXlnZ2hfS2dKbFlPWm9vTDRfaFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQWUNSeGxJek81dUJlclpCNGdmbFhNSHcxcWVkeDgyYjJfVm9tZ1FVMkYyQkZ2U19QbTVvUmFRbWk2a3pVU2dRemswV0NMV2lXRXpScUlNUjhzbzljMTQ2NXRUTTd4eW9aYjdUYmM4NDBzc2tmbE94djhZeWQ5V2FlLVdnelhjTno4ZnF5Q3pRUdIBjwFBVV95cUxQWUNSeGxJek81dUJlclpCNGdmbFhNSHcxcWVkeDgyYjJfVm9tZ1FVMkYyQkZ2U19QbTVvUmFRbWk2a3pVU2dRemswV0NMV2lXRXpScUlNUjhzbzljMTQ2NXRUTTd4eW9aYjdUYmM4NDBzc2tmbE94djhZeWQ5V2FlLVdnelhjTno4ZnF5Q3pRUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>Off-White x Nike Air Force 1 Low “Sesame” Releasing Fall 2025 - Sneaker News</t>
+          <t>First Look At The Nike Kobe 8 Protro “Mambacurial” - Sneaker News</t>
         </is>
       </c>
       <c r="B46" s="35" t="inlineStr">
@@ -2975,9 +2975,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>$100</t>
+      <c r="D46" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E46" s="17" t="inlineStr">
@@ -2985,31 +2985,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F46" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G46" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F46" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G46" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H46" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxPYnhpMGpMMHBiQ1JoNTZ0RWdQQTUzVi16bi1mSnF6cEREMmpDNDQ3M1ZQWGVRRkF0NUNPdzU3RDdjb2E5RC1md3ltTlUxWUtKTFExRDhjNWQ5Rlgzb1Ixb0cxTG1Tem1kelo2SDJTenI4d1BvY05JRXc1WF9WNEpqQjZ6Y2RIdE1hSW9jTdIBjAFBVV95cUxPYnhpMGpMMHBiQ1JoNTZ0RWdQQTUzVi16bi1mSnF6cEREMmpDNDQ3M1ZQWGVRRkF0NUNPdzU3RDdjb2E5RC1md3ltTlUxWUtKTFExRDhjNWQ5Rlgzb1Ixb0cxTG1Tem1kelo2SDJTenI4d1BvY05JRXc1WF9WNEpqQjZ6Y2RIdE1hSW9jTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNeXlHVUdiNHhkRmVpZ1VscjREV0NoY2hwX2pScG0tSnJIWHZmWWtGQXctUUFVTVVrX29OanZIeHB6eHVjYldENk9nNVJQTHQySlQ2ZkRGSmNqQ0RKaXlPeFdvRXBwZWFJZnVOZndMV3pqS01YQkVHTDFnOExvYjJERkJtUjhrb0wzeG5OUnU4WDNlMllU0gGUAUFVX3lxTE15eUdVR2I0eGRGZWlnVWxyNERXQ2hjaHBfalJwbS1KckhYdmZZa0ZBdy1RQVVNVWtfb05qdkh4cHp4dWNiV0Q2T2c1UlBMdDJKVDZmREZKY2pDREppeU94V29FcHBlYUlmdU5md0xXempLTVhCRUdMMWc4TG9iMkRGQm1SOGtvTDN4bk5SdThYM2UyWVQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Devin Booker’s Nike Book 2 Is Officially Unveiled - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B47" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Jordan Brand Preps For Graduation Season With The Air Jordan 6 “Cap And Gown” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C47" s="22" t="inlineStr">
@@ -3017,9 +3017,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D47" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -3027,26 +3027,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F47" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G47" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G47" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE85bXdkeFBTekkxMWdnOUxPYTYtd0c0cHJJMUUycXJTZXJIbmRkN0pORm5EV0Q3ck52b3NsQzdodmVRYUM1dkMwak9aRXhrOF9uRFhZMkFmYnpCVDdPbHNmNC1WSHhhbDltdDBjUNIBbEFVX3lxTE85bXdkeFBTekkxMWdnOUxPYTYtd0c0cHJJMUUycXJTZXJIbmRkN0pORm5EV0Q3ck52b3NsQzdodmVRYUM1dkMwak9aRXhrOF9uRFhZMkFmYnpCVDdPbHNmNC1WSHhhbDltdDBjUA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBVbFZaUlNQWFcyemItamVtR0hsd2R4UHZreVFhOGV5T1JRanctZ0RRQ0J5dGNjOFlXUldRYWFGXzZDUW9JMXB1NzJ1Nm9HMkd1N2hNcTNMSDlKdHd6anJVQXZFSWpMZTFicDJ1UkNB0gFuQVVfeXFMUFVsVlpSU1BYVzJ6Yi1qZW1HSGx3ZHhQdmt5UWE4ZXlPUlFqdy1nRFFDQnl0Y2M4WVdSV1FhYUZfNkNRb0kxcHU3MnU2b0cyR3U3aE1xM0xIOUp0d3pqclVBdkVJakxlMWJwMnVSQ0E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>The Nike S.T. Charge Is Leaving Ballers Everywhere Jealous - Sneaker News</t>
+          <t>The Nike Air Force 1 Low Odes To Team USA - Sneaker News</t>
         </is>
       </c>
       <c r="B48" s="35" t="inlineStr">
@@ -3059,9 +3059,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D48" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>$100</t>
         </is>
       </c>
       <c r="E48" s="17" t="inlineStr">
@@ -3081,19 +3081,19 @@
       </c>
       <c r="H48" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE81Y0FjVnFXRlpMVTM4UGJ1X2phelVILWc1REN5Yk1DeW5kOWhhTExMZE5QaDlCemZVaG5Oam5GUEowNGpLcF9WWURoM05MVVB4OHFpYTNrRXR3U1NZc1ZF0gFfQVVfeXFMTzVjQWNWcVdGWkxVMzhQYnVfamF6VUgtZzVEQ3liTUN5bmQ5aGFMTExkTlBoOUJ6ZlVobk5qbkZQSjA0aktwX1ZZRGgzTkxVUHg4cWlhM2tFdHdTU1lzVkU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQcGVCSmxsMEVsRFJMU281VzVpa0ZJT01abGl1YldaVXZXQUxWRzVxblpnSnhVU3RXMGh4dXJxdEYzNTdWaWFwR2ZoLVdnUVJ3b2RkS0s2TWZQMUhIOUdQcEFVVTRLdEthSVVzYl8tSlZ1Vll1MTh2Rkh5SmhTRDZjUkh30gGCAUFVX3lxTFBwZUJKbGwwRWxEUkxTbzVXNWlrRklPTVpsaXViV1pVdldBTFZHNXFuWmdKeFVTdFcwaHh1cnF0RjM1N1ZpYXBHZmgtV2dRUndvZGRLSzZNZlAxSEg5R1BwQVVVNEt0S2FJVXNiXy1KVnVWWXUxOHZGSHlKaFNENmNSSHc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>First Look At The Teyana Taylor x Air Jordan 3 “Concrete Rose” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike Air Tech Challenge II “Pixel Court” Returns August 30th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C49" s="22" t="inlineStr">
@@ -3101,9 +3101,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D49" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -3111,26 +3111,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F49" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G49" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNcjFFdkRuaXo2c1h4cTVLWUIxSE5PVmQ2alNic1V0dnZDb1BGTDE0OUlldkRSVzFsb19TcGNFQmdyOVZ0X3NpaWNLNkp1aktZOEVJVVdDRTMtYUVsd0oxS0lxdjV0ODJsV1NDU2YtODRkMzlHRWRjZXNtZGlJRzIzbWt2dFF5QdIBhgFBVV95cUxNcjFFdkRuaXo2c1h4cTVLWUIxSE5PVmQ2alNic1V0dnZDb1BGTDE0OUlldkRSVzFsb19TcGNFQmdyOVZ0X3NpaWNLNkp1aktZOEVJVVdDRTMtYUVsd0oxS0lxdjV0ODJsV1NDU2YtODRkMzlHRWRjZXNtZGlJRzIzbWt2dFF5QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQRURBSi1KcWNMRTExQ3VwQ0wwTVNlWHhVWS10eDZrLWNGSHdMWEJlbXFWX2kzYXFuZWk2dE85cVFzZ2RFbWJSSTQzS295bl9vMGdneXFIcVJiV3AwcXh6bzRwWndWcWg1X3FpamtMNGlCdVZVZWJqZ3FyQnF5Z2doX0tnSmxZT1pvb0w0X2hR0gGOAUFVX3lxTFBFREFKLUpxY0xFMTFDdXBDTDBNU2VYeFVZLXR4NmstY0ZId0xYQmVtcVZfaTNhcW5laTZ0TzlxUXNnZEVtYlJJNDNLb3luX28wZ2d5cUhxUmJXcDBxeHpvNHBad1ZxaDVfcWlqa0w0aUJ1VlVlYmpncXJCcXlnZ2hfS2dKbFlPWm9vTDRfaFE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Official Images Of The Nike Air Max 95 “Green Apple/Photo Blue” - Sneaker News</t>
+          <t>Devin Booker’s Nike Book 2 Is Officially Unveiled - Sneaker News</t>
         </is>
       </c>
       <c r="B50" s="35" t="inlineStr">
@@ -3143,9 +3143,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
+      <c r="D50" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E50" s="17" t="inlineStr">
@@ -3165,19 +3165,19 @@
       </c>
       <c r="H50" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxON2JUaTRaWVhlVkVwVk50VDJMR2dOeTFxa1hnQ2JpLWRBM1hFYlo2SC1qTU5WWjR4RzNMaDlJeC00ZEczdXNITWR5VnZiYWU4MGItWS1SbkJjYlRMR2laZVJGUTZCRjhYN08yVW5YY0wtUExpZ2J1TkNMNnJOU1JoMk1SNmdhQ19fTmlMWDlR0gGOAUFVX3lxTE43YlRpNFpZWGVWRXBWTnRUMkxHZ055MXFrWGdDYmktZEEzWEViWjZILWpNTlZaNHhHM0xoOUl4LTRkRzN1c0hNZHlWdmJhZTgwYi1ZLVJuQmNiVExHaVplUkZRNkJGOFg3TzJVblhjTC1QTGlnYnVOQ0w2ck5TUmgyTVI2Z2FDX19OaUxYOVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE85bXdkeFBTekkxMWdnOUxPYTYtd0c0cHJJMUUycXJTZXJIbmRkN0pORm5EV0Q3ck52b3NsQzdodmVRYUM1dkMwak9aRXhrOF9uRFhZMkFmYnpCVDdPbHNmNC1WSHhhbDltdDBjUNIBbEFVX3lxTE85bXdkeFBTekkxMWdnOUxPYTYtd0c0cHJJMUUycXJTZXJIbmRkN0pORm5EV0Q3ck52b3NsQzdodmVRYUM1dkMwak9aRXhrOF9uRFhZMkFmYnpCVDdPbHNmNC1WSHhhbDltdDBjUA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>The 2026 Air Jordan 11 “Space Jam” Will Feature “23” Text On The Heel - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike S.T. Charge Is Leaving Ballers Everywhere Jealous - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C51" s="22" t="inlineStr">
@@ -3185,9 +3185,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>$220</t>
+      <c r="D51" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -3195,31 +3195,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F51" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G51" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H51" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBCUWdEV2FBTmJGZmpVUW11T0dUdUJhNWc0WGdPOTg5REVpYUo1b0JzN0dURkh5S2ppZExGSjJVWWdlUUJGX01MOXdiRGtmcHd1RE5kdU9PalBaai1GZEZEYWFyMElKVmZaaVhDdm9IaG01QdIBckFVX3lxTFBCUWdEV2FBTmJGZmpVUW11T0dUdUJhNWc0WGdPOTg5REVpYUo1b0JzN0dURkh5S2ppZExGSjJVWWdlUUJGX01MOXdiRGtmcHd1RE5kdU9PalBaai1GZEZEYWFyMElKVmZaaVhDdm9IaG01QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE81Y0FjVnFXRlpMVTM4UGJ1X2phelVILWc1REN5Yk1DeW5kOWhhTExMZE5QaDlCemZVaG5Oam5GUEowNGpLcF9WWURoM05MVVB4OHFpYTNrRXR3U1NZc1ZF0gFfQVVfeXFMTzVjQWNWcVdGWkxVMzhQYnVfamF6VUgtZzVEQ3liTUN5bmQ5aGFMTExkTlBoOUJ6ZlVobk5qbkZQSjA0aktwX1ZZRGgzTkxVUHg4cWlhM2tFdHdTU1lzVkU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>LaMelo Ball Shoes - 2025 Release Dates - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B52" s="32" t="inlineStr">
-        <is>
-          <t>Other</t>
+          <t>Official Images Of The Nike Air Max 95 “Green Apple/Photo Blue” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B52" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C52" s="27" t="inlineStr">
@@ -3227,9 +3227,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D52" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
         </is>
       </c>
       <c r="E52" s="17" t="inlineStr">
@@ -3237,31 +3237,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F52" s="16" t="inlineStr">
-        <is>
-          <t>★☆☆☆☆  1/5</t>
-        </is>
-      </c>
-      <c r="G52" s="43" t="inlineStr">
-        <is>
-          <t>⚪ General Release</t>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H52" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBrT0t4aENxYTdzcU82VS1fbEVHaXBCQi1DNFpMd2hSajJ5eU9oX05tZ3hLUlVVQU9qbEp0YmNJRGo2M0hUWVp5WllwcDJfVU01VUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxON2JUaTRaWVhlVkVwVk50VDJMR2dOeTFxa1hnQ2JpLWRBM1hFYlo2SC1qTU5WWjR4RzNMaDlJeC00ZEczdXNITWR5VnZiYWU4MGItWS1SbkJjYlRMR2laZVJGUTZCRjhYN08yVW5YY0wtUExpZ2J1TkNMNnJOU1JoMk1SNmdhQ19fTmlMWDlR0gGOAUFVX3lxTE43YlRpNFpZWGVWRXBWTnRUMkxHZ055MXFrWGdDYmktZEEzWEViWjZILWpNTlZaNHhHM0xoOUl4LTRkRzN1c0hNZHlWdmJhZTgwYi1ZLVJuQmNiVExHaVplUkZRNkJGOFg3TzJVblhjTC1QTGlnYnVOQ0w2ck5TUmgyTVI2Z2FDX19OaUxYOVE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>The Year Of The Vans Authentic Continues With A Haven Collab - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B53" s="23" t="inlineStr">
-        <is>
-          <t>Vans</t>
+          <t>The 2026 Air Jordan 11 “Space Jam” Will Feature “23” Text On The Heel - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C53" s="22" t="inlineStr">
@@ -3269,9 +3269,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D53" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>$220</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -3291,19 +3291,19 @@
       </c>
       <c r="H53" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNZUQ0d1JDRTAxMl84NEItRGM4cE0zbW9JMkFyTDdRbUtYX0RNMU1ZbURzdWV3S081ekdpbXoxT2V4TWVrWmhWSFE3Z0FZMlYyaG5nMjd2dXFNY0ptYmN3S2VJbXJaUHZqS3ByM2V3Z0ZJVVNoOExFYUlsdFM2Unp1YV9R0gGCAUFVX3lxTE1lRDR3UkNFMDEyXzg0Qi1EYzhwTTNtb0kyQXJMN1FtS1hfRE0xTVltRHN1ZXdLTzV6R2ltejFPZXhNZWtaaFZIUTdnQVkyVjJobmcyN3Z1cU1jSm1iY3dLZUltclpQdmpLcHIzZXdnRklVU2g4TEVhSWx0UzZSenVhX1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBCUWdEV2FBTmJGZmpVUW11T0dUdUJhNWc0WGdPOTg5REVpYUo1b0JzN0dURkh5S2ppZExGSjJVWWdlUUJGX01MOXdiRGtmcHd1RE5kdU9PalBaai1GZEZEYWFyMElKVmZaaVhDdm9IaG01QdIBckFVX3lxTFBCUWdEV2FBTmJGZmpVUW11T0dUdUJhNWc0WGdPOTg5REVpYUo1b0JzN0dURkh5S2ppZExGSjJVWWdlUUJGX01MOXdiRGtmcHd1RE5kdU9PalBaai1GZEZEYWFyMElKVmZaaVhDdm9IaG01QQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>The Nike Book 2 “Must Be The Denim” Releases On March 20th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B54" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>LaMelo Ball Shoes - 2025 Release Dates - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
       <c r="C54" s="27" t="inlineStr">
@@ -3321,31 +3321,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F54" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G54" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>★☆☆☆☆  1/5</t>
+        </is>
+      </c>
+      <c r="G54" s="43" t="inlineStr">
+        <is>
+          <t>⚪ General Release</t>
         </is>
       </c>
       <c r="H54" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNNHlCTkJ3TTFfUzZ2V1doeVlpYWpSLWR0Z3JXVEtiNmpJOVprbWxCRzBtVG9KSlozVzFiMy1lUk1YVDljUEx5R2JyaWN3RGdRMTQxRUlXMGJYU1EwTzlBSmFsd0tzRXF4TzhxTHNWVXFmX1B1alQ1cFZJNGc5T0lucHhGcVROWlltNkdSWHVtNm1uUUtQazRhTlhB0gGaAUFVX3lxTE00eUJOQndNMV9TNnZXV2h5WWlhalItZHRncldUS2I2akk5WmttbEJHMG1Ub0pKWjNXMWIzLWVSTVhUOWNQTHlHYnJpY3dEZ1ExNDFFSVcwYlhTUTBPOUFKYWx3S3NFcXhPOHFMc1ZVcWZfUHVqVDVwVkk0ZzlPSW5weEZxVE5aWW02R1JYdW02bW5RS1BrNGFOWEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBrT0t4aENxYTdzcU82VS1fbEVHaXBCQi1DNFpMd2hSajJ5eU9oX05tZ3hLUlVVQU9qbEp0YmNJRGo2M0hUWVp5WllwcDJfVU01VUE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>The Nike Ja 3 “Let Me Be Ja” Could Be Among The Last Drops Of The Model - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B55" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The Year Of The Vans Authentic Continues With A Haven Collab - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>Vans</t>
         </is>
       </c>
       <c r="C55" s="22" t="inlineStr">
@@ -3363,26 +3363,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F55" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G55" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H55" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQTTlVYVFkQTBHakRtSVMzMG9hTFA3ZldwbllMZnRXb0FHZXk3V1ZDbUJDM1ZqTEFOcldnQlMtMzR4T0lIX3FKN1NYOUN0S3NYU3hHSXJOcWw4QjBsRVhUWDNMZ1BreVN3ZWsxLVRsNEJjaWhiVkpMQ1NrMmo1czBlU2tYZUlEMTFRVWVWV0prV1JycE3SAZMBQVVfeXFMUE05VWFRZEEwR2pEbUlTMzBvYUxQN2ZXcG5ZTGZ0V29BR2V5N1dWQ21CQzNWakxBTnJXZ0JTLTM0eE9JSF9xSjdTWDlDdEtzWFN4R0lyTnFsOEIwbEVYVFgzTGdQa3lTd2VrMS1UbDRCY2loYlZKTENTazJqNXMwZVNrWGVJRDExUVVlVldKa1dScnBN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNZUQ0d1JDRTAxMl84NEItRGM4cE0zbW9JMkFyTDdRbUtYX0RNMU1ZbURzdWV3S081ekdpbXoxT2V4TWVrWmhWSFE3Z0FZMlYyaG5nMjd2dXFNY0ptYmN3S2VJbXJaUHZqS3ByM2V3Z0ZJVVNoOExFYUlsdFM2Unp1YV9R0gGCAUFVX3lxTE1lRDR3UkNFMDEyXzg0Qi1EYzhwTTNtb0kyQXJMN1FtS1hfRE0xTVltRHN1ZXdLTzV6R2ltejFPZXhNZWtaaFZIUTdnQVkyVjJobmcyN3Z1cU1jSm1iY3dLZUltclpQdmpLcHIzZXdnRklVU2g4TEVhSWx0UzZSenVhX1E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>Official Images Of The Nike Zoom GT Cut 4 “Think Pink” - Sneaker News</t>
+          <t>The Nike Book 2 “Must Be The Denim” Releases On March 20th - Sneaker News</t>
         </is>
       </c>
       <c r="B56" s="35" t="inlineStr">
@@ -3417,14 +3417,14 @@
       </c>
       <c r="H56" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOLURiYWxJZkZReGJ3d1pjNTVldUNqQ2xsaXltN3pNWURFajVhRTAtcHlkSVFhSjFHbUlCWUxfa0pIdlg1bkJGSUV0NElBczJQNFFTTmJnVHMtNjducFJDNnBFM0RjMDdYYXcyd1dXM1B3Y2psWWxDOXlJcEgtM0hlUnV4dHhiNVFjRGJsd9IBjAFBVV95cUxOLURiYWxJZkZReGJ3d1pjNTVldUNqQ2xsaXltN3pNWURFajVhRTAtcHlkSVFhSjFHbUlCWUxfa0pIdlg1bkJGSUV0NElBczJQNFFTTmJnVHMtNjducFJDNnBFM0RjMDdYYXcyd1dXM1B3Y2psWWxDOXlJcEgtM0hlUnV4dHhiNVFjRGJsdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNNHlCTkJ3TTFfUzZ2V1doeVlpYWpSLWR0Z3JXVEtiNmpJOVprbWxCRzBtVG9KSlozVzFiMy1lUk1YVDljUEx5R2JyaWN3RGdRMTQxRUlXMGJYU1EwTzlBSmFsd0tzRXF4TzhxTHNWVXFmX1B1alQ1cFZJNGc5T0lucHhGcVROWlltNkdSWHVtNm1uUUtQazRhTlhB0gGaAUFVX3lxTE00eUJOQndNMV9TNnZXV2h5WWlhalItZHRncldUS2I2akk5WmttbEJHMG1Ub0pKWjNXMWIzLWVSTVhUOWNQTHlHYnJpY3dEZ1ExNDFFSVcwYlhTUTBPOUFKYWx3S3NFcXhPOHFMc1ZVcWZfUHVqVDVwVkk0ZzlPSW5weEZxVE5aWW02R1JYdW02bW5RS1BrNGFOWEE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>The Air Jordan 40 “Bordeaux” Is Pure Class - Sneaker News</t>
+          <t>Fresh Look At The Air Jordan 11 “Gamma Blue” - Sneaker News</t>
         </is>
       </c>
       <c r="B57" s="21" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>$210</t>
+          <t>$220</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -3459,19 +3459,19 @@
       </c>
       <c r="H57" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFB5U3ZpMWhPS0RtcGtYZng4V19HWHZNZUh6ZGZaR2RDWnNfbF9xbDM0RDNKQXJzdkFuUm5hR3VGU21jVUpuU1V6NTBVUEUwb2ktWG1TZDR5Y0NTOXI1OHVHbUxfdjROVUxJNW9VaThsakFtNkpNd0t3ddIBeEFVX3lxTFB5U3ZpMWhPS0RtcGtYZng4V19HWHZNZUh6ZGZaR2RDWnNfbF9xbDM0RDNKQXJzdkFuUm5hR3VGU21jVUpuU1V6NTBVUEUwb2ktWG1TZDR5Y0NTOXI1OHVHbUxfdjROVUxJNW9VaThsakFtNkpNd0t3dQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBHWVJmOGU5Q3hiWHFrQ1NJZnNwSjU3TS16eFVtOUtBUmhMLVBiSWNDX3lrY194T0diWUo1VDBEZm01dFZJNDNuTWRZa0ozQlR4Y2lCMkpTb0E4VXQwdWNrdGd1Nkh1SWVnX19tRmFXbkhEVUXSAXNBVV95cUxQR1lSZjhlOUN4Ylhxa0NTSWZzcEo1N00tenhVbTlLQVJoTC1QYkljQ195a2NfeE9HYllKNVQwRGZtNXRWSTQzbk1kWWtKM0JUeGNpQjJKU29BOFV0MHVja3RndTZIdUllZ19fbUZhV25IRFVF?oc=5</t>
         </is>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>Where To Buy The Air Jordan 4 “Lakers” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B58" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike Vomero Premium Is Ready For Spring Miles In “Particle Pink” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B58" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C58" s="27" t="inlineStr">
@@ -3479,9 +3479,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>$210</t>
+      <c r="D58" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E58" s="17" t="inlineStr">
@@ -3501,14 +3501,14 @@
       </c>
       <c r="H58" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPRXE5SVRnWFFmWWNsakVJeGtndDNBUjNsRzRVM01CSVRDUkJ6OUloNVdranBFckZ5ZGlKcHJ3b3ZCNl9BdVktbzR4bmpTcGs3YUZ3TmowX2hhUF9JRl9YRGNIdkRBRFRHWGNlZEFVTzM1WF8wN3BnLWlwZWZHNk1JVNIBgAFBVV95cUxPRXE5SVRnWFFmWWNsakVJeGtndDNBUjNsRzRVM01CSVRDUkJ6OUloNVdranBFckZ5ZGlKcHJ3b3ZCNl9BdVktbzR4bmpTcGs3YUZ3TmowX2hhUF9JRl9YRGNIdkRBRFRHWGNlZEFVTzM1WF8wN3BnLWlwZWZHNk1JVA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOenNJd1ItWHZ5QkFhRzA0bkN0TXB6VlhFWWpkWDdGRjdvSUpsa2tlWWpCY1VKaGkzb1J0WkNnYUNKQnBSaVFsdDZhLVdFXzgyaDBkWGktUHc0Q2lqR3B5eUpwazV4b0ZxSHJQTlVnYkRVOEFHcE9fb01hVTFwRVRqZS0tam9wSk9tdzVocEZyODlZTWdKVll3Szl6ZVBfMk5oMlNoRjJjOEEzOUlkSUprMNIBsAFBVV95cUxOenNJd1ItWHZ5QkFhRzA0bkN0TXB6VlhFWWpkWDdGRjdvSUpsa2tlWWpCY1VKaGkzb1J0WkNnYUNKQnBSaVFsdDZhLVdFXzgyaDBkWGktUHc0Q2lqR3B5eUpwazV4b0ZxSHJQTlVnYkRVOEFHcE9fb01hVTFwRVRqZS0tam9wSk9tdzVocEZyODlZTWdKVll3Szl6ZVBfMk5oMlNoRjJjOEEzOUlkSUprMA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Carbon Fiber Swooshes Land On This Nike Air Force 1 Low - Sneaker News</t>
+          <t>Official Images Of The Nike Zoom GT Cut 4 “Think Pink” - Sneaker News</t>
         </is>
       </c>
       <c r="B59" s="30" t="inlineStr">
@@ -3521,9 +3521,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>$100</t>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
@@ -3543,19 +3543,19 @@
       </c>
       <c r="H59" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbXRDVlc4ZXVVeTJPVTFTS0VLN1ZCMGJHSlZKNE9GVnZlVHN5SmVsUHFwWGJWaEpjblNhdUJlSlpNZm1VemdyX1g0R2lJdXZhb1BkbFJOMXlPWUNkM1ZYc1ZuM0tpQTFsSm1HRFNzUFRVV2ZDcmhsdzF3UXBXUGxmODE5OUIyLW9DbTQ1WWFKM3PSAZABQVVfeXFMTW10Q1ZXOGV1VXkyT1UxU0tFSzdWQjBiR0pWSjRPRlZ2ZVRzeUplbFBxcFhiVmhKY25TYXVCZUpaTWZtVXpncl9YNEdpSXV2YW9QZGxSTjF5T1lDZDNWWHNWbjNLaUExbEptR0RTc1BUVVdmQ3JobHcxd1FwV1BsZjgxOTlCMi1vQ200NVlhSjNz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOLURiYWxJZkZReGJ3d1pjNTVldUNqQ2xsaXltN3pNWURFajVhRTAtcHlkSVFhSjFHbUlCWUxfa0pIdlg1bkJGSUV0NElBczJQNFFTTmJnVHMtNjducFJDNnBFM0RjMDdYYXcyd1dXM1B3Y2psWWxDOXlJcEgtM0hlUnV4dHhiNVFjRGJsd9IBjAFBVV95cUxOLURiYWxJZkZReGJ3d1pjNTVldUNqQ2xsaXltN3pNWURFajVhRTAtcHlkSVFhSjFHbUlCWUxfa0pIdlg1bkJGSUV0NElBczJQNFFTTmJnVHMtNjducFJDNnBFM0RjMDdYYXcyd1dXM1B3Y2psWWxDOXlJcEgtM0hlUnV4dHhiNVFjRGJsdw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>Fear Of God Just Dropped Its Last adidas Shoe - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>The Air Jordan 40 “Bordeaux” Is Pure Class - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C60" s="27" t="inlineStr">
@@ -3563,9 +3563,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D60" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>$210</t>
         </is>
       </c>
       <c r="E60" s="17" t="inlineStr">
@@ -3573,31 +3573,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F60" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G60" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F60" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G60" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H60" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNSFNCR2dpR215UEo5WFpxM1l3OTA3S3A5QklJWEg0RDNjeGlzNFZWNlAxN3VjS1JHREc1cC1SQVBScEUzT0YwcGRzNXVyRWdlMkc2Vjk2cXNyWjA3UnF1WndnQjY0aWRRMTMyVkxxcVlCRnFENUI3MXVLS2ZwXzU0etIBgAFBVV95cUxNSFNCR2dpR215UEo5WFpxM1l3OTA3S3A5QklJWEg0RDNjeGlzNFZWNlAxN3VjS1JHREc1cC1SQVBScEUzT0YwcGRzNXVyRWdlMkc2Vjk2cXNyWjA3UnF1WndnQjY0aWRRMTMyVkxxcVlCRnFENUI3MXVLS2ZwXzU0eg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFB5U3ZpMWhPS0RtcGtYZng4V19HWHZNZUh6ZGZaR2RDWnNfbF9xbDM0RDNKQXJzdkFuUm5hR3VGU21jVUpuU1V6NTBVUEUwb2ktWG1TZDR5Y0NTOXI1OHVHbUxfdjROVUxJNW9VaThsakFtNkpNd0t3ddIBeEFVX3lxTFB5U3ZpMWhPS0RtcGtYZng4V19HWHZNZUh6ZGZaR2RDWnNfbF9xbDM0RDNKQXJzdkFuUm5hR3VGU21jVUpuU1V6NTBVUEUwb2ktWG1TZDR5Y0NTOXI1OHVHbUxfdjROVUxJNW9VaThsakFtNkpNd0t3dQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>The Satoshi Nakamoto Influence Continues On The Vans Slip-On For Spring - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B61" s="23" t="inlineStr">
-        <is>
-          <t>Vans</t>
+          <t>Where To Buy The Air Jordan 4 “Lakers” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C61" s="22" t="inlineStr">
@@ -3605,9 +3605,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D61" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>$210</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
@@ -3615,31 +3615,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F61" s="41" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G61" s="42" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F61" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G61" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H61" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOV9IBeEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPRXE5SVRnWFFmWWNsakVJeGtndDNBUjNsRzRVM01CSVRDUkJ6OUloNVdranBFckZ5ZGlKcHJ3b3ZCNl9BdVktbzR4bmpTcGs3YUZ3TmowX2hhUF9JRl9YRGNIdkRBRFRHWGNlZEFVTzM1WF8wN3BnLWlwZWZHNk1JVNIBgAFBVV95cUxPRXE5SVRnWFFmWWNsakVJeGtndDNBUjNsRzRVM01CSVRDUkJ6OUloNVdranBFckZ5ZGlKcHJ3b3ZCNl9BdVktbzR4bmpTcGs3YUZ3TmowX2hhUF9JRl9YRGNIdkRBRFRHWGNlZEFVTzM1WF8wN3BnLWlwZWZHNk1JVA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>Quavo Spotted In The Upcoming Sinclair x PUMA Suede - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B62" s="44" t="inlineStr">
-        <is>
-          <t>Puma</t>
+          <t>Fear Of God Just Dropped Its Last adidas Shoe - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C62" s="27" t="inlineStr">
@@ -3647,9 +3647,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
-        <is>
-          <t>$75</t>
+      <c r="D62" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E62" s="17" t="inlineStr">
@@ -3657,31 +3657,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F62" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G62" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F62" s="36" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G62" s="37" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H62" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE13eWlSUXpENWV1UWhPdkY2SDVtVGhINXBNSUNRdDMzMDdtWVR3S1RwSndiLS1XVGxuZkJxV3FLQzRuZy1sSFNYZkx0M2g4Z04zTGNwZFQwQmphQ0VlaEdzVGdEcExKY2xocVY2R0xR0gFuQVVfeXFMTXd5aVJRekQ1ZXVRaE92RjZINW1UaEg1cE1JQ1F0MzMwN21ZVHdLVHBKd2ItLVdUbG5mQnFXcUtDNG5nLWxIU1hmTHQzaDhnTjNMY3BkVDBCamFDRWVoR3NUZ0RwTEpjbGhxVjZHTFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNSFNCR2dpR215UEo5WFpxM1l3OTA3S3A5QklJWEg0RDNjeGlzNFZWNlAxN3VjS1JHREc1cC1SQVBScEUzT0YwcGRzNXVyRWdlMkc2Vjk2cXNyWjA3UnF1WndnQjY0aWRRMTMyVkxxcVlCRnFENUI3MXVLS2ZwXzU0etIBgAFBVV95cUxNSFNCR2dpR215UEo5WFpxM1l3OTA3S3A5QklJWEg0RDNjeGlzNFZWNlAxN3VjS1JHREc1cC1SQVBScEUzT0YwcGRzNXVyRWdlMkc2Vjk2cXNyWjA3UnF1WndnQjY0aWRRMTMyVkxxcVlCRnFENUI3MXVLS2ZwXzU0eg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Elephant Print Finally Arrives On This Jordan Dad Shoe - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B63" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Satoshi Nakamoto Influence Continues On The Vans Slip-On For Spring - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>Vans</t>
         </is>
       </c>
       <c r="C63" s="22" t="inlineStr">
@@ -3699,31 +3699,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F63" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G63" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F63" s="41" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G63" s="42" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H63" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZ9IBhgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOV9IBeEFVX3lxTE92TGJYZnFYYkNyUjdQRVZnRUF0SWhMUmZzYXVZd3NFanFaU0hlZVRGVVhXWThldzYwMEJDek9Yb2x1T2JjTnZvNXliTVIxazB6RG1WZEhpU3JTQnZTN2FmRk9WOXp5Z1VRYmtOc1pRTDJBa0ZDbTNOVw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>adidas Delivers A Late “Chinese New Year” Tribute On The EVO SL Trainer - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B64" s="14" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Detailed Look At The Air Jordan 5 “Wolf Grey” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C64" s="27" t="inlineStr">
@@ -3731,9 +3731,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D64" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E64" s="17" t="inlineStr">
@@ -3741,26 +3741,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G64" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F64" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G64" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H64" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQdIBfkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTFAwQUZiQktBRDlWQmJSVlRpYjdVSVRZZUYycVFjZ053cG0tM2stODZRX0UtRHdnVW1EbHg1Z3lXejZfWU1RODkza190cGJLQmxtandjdFlBc2xZSGVpa3dIcjFoVUNLRTNWcHfSAWpBVV95cUxQMEFGYkJLQUQ5VkJiUlZUaWI3VUlUWWVGMnFRY2dOd3BtLTNrLTg2UV9FLUR3Z1VtRGx4NWd5V3o2X1lNUTg5M2tfdHBiS0JsbWp3Y3RZQXNsWUhlaWt3SHIxaFVDS0UzVnB3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>Nike Air Max 97 – History + Official Releases 2025 - Sneaker News</t>
+          <t>Carbon Fiber Swooshes Land On This Nike Air Force 1 Low - Sneaker News</t>
         </is>
       </c>
       <c r="B65" s="30" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>$175</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -3795,19 +3795,19 @@
       </c>
       <c r="H65" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE5mU01lTzVJUU5lZ1d5NmxPbEpiaWI5enZZNXJkdG5EVmlQYk13Y3RvcjJFS0ZiWG9iZjhMWVBISGZoNlZpdmd2SjUzMmFKeTB4X0JYZ2VDTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbXRDVlc4ZXVVeTJPVTFTS0VLN1ZCMGJHSlZKNE9GVnZlVHN5SmVsUHFwWGJWaEpjblNhdUJlSlpNZm1VemdyX1g0R2lJdXZhb1BkbFJOMXlPWUNkM1ZYc1ZuM0tpQTFsSm1HRFNzUFRVV2ZDcmhsdzF3UXBXUGxmODE5OUIyLW9DbTQ1WWFKM3PSAZABQVVfeXFMTW10Q1ZXOGV1VXkyT1UxU0tFSzdWQjBiR0pWSjRPRlZ2ZVRzeUplbFBxcFhiVmhKY25TYXVCZUpaTWZtVXpncl9YNEdpSXV2YW9QZGxSTjF5T1lDZDNWWHNWbjNLaUExbEptR0RTc1BUVVdmQ3JobHcxd1FwV1BsZjgxOTlCMi1vQ200NVlhSjNz?oc=5</t>
         </is>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>The Nike Air Max Plus Carries “Pink Foam” Echoes - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B66" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Quavo Spotted In The Upcoming Sinclair x PUMA Suede - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B66" s="44" t="inlineStr">
+        <is>
+          <t>Puma</t>
         </is>
       </c>
       <c r="C66" s="27" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$75</t>
         </is>
       </c>
       <c r="E66" s="17" t="inlineStr">
@@ -3825,26 +3825,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F66" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G66" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F66" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G66" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H66" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNRU1pWDF4alUtNjJGUVFLR0hya1h1Vm5RVFJnM1BvNGh1azNHdUFld19kZS15LUZIRXZ3aUFtbnlnYlpQWTZCTHAzd1FmZi1XY3A5OUFEZ3ZXRmR0MFpNU3BFX2ZDYUYzZG10Sl96OVlBd094OUVtQ1FiR0RrbTkyc2hBQzZlVml2MWdLQ0FUakpPY0pLRXfSAZYBQVVfeXFMTUVNaVgxeGpVLTYyRlFRS0dIcmtYdVZuUVRSZzNQbzRodWszR3VBZXdfZGUteS1GSEV2d2lBbW55Z2JaUFk2QkxwM3dRZmYtV2NwOTlBRGd2V0ZkdDBaTVNwRV9mQ2FGM2RtdEpfejlZQXdPeDlFbUNRYkdEa205MnNoQUM2ZVZpdjFnS0NBVGpKT2NKS0V3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE13eWlSUXpENWV1UWhPdkY2SDVtVGhINXBNSUNRdDMzMDdtWVR3S1RwSndiLS1XVGxuZkJxV3FLQzRuZy1sSFNYZkx0M2g4Z04zTGNwZFQwQmphQ0VlaEdzVGdEcExKY2xocVY2R0xR0gFuQVVfeXFMTXd5aVJRekQ1ZXVRaE92RjZINW1UaEg1cE1JQ1F0MzMwN21ZVHdLVHBKd2ItLVdUbG5mQnFXcUtDNG5nLWxIU1hmTHQzaDhnTjNMY3BkVDBCamFDRWVoR3NUZ0RwTEpjbGhxVjZHTFE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Kim Kardashian And NikeSkims Debut The Rift Mesh “Light Bone” - Sneaker News</t>
+          <t>The Nike ACG LDV Tells The Origin Story Of All-Conditions Gear - Sneaker News</t>
         </is>
       </c>
       <c r="B67" s="30" t="inlineStr">
@@ -3879,14 +3879,14 @@
       </c>
       <c r="H67" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPWVh4LUNfVjg0bFllenoxZFp1M1BxM1NQdDZCTmotbmt0MFRuVzUtanlJN1BiSkk1V240U2szLVlMVE1rZlBxbVhHRmV2MGcta0JBUnVSY3AwR0cyN05LWjVxYW9NNVUzUlZaR0V5cF9QWlBnTHVsTEg2THdka3NKTG82NkLSAYQBQVVfeXFMT1lYeC1DX1Y4NGxZZXp6MWRadTNQcTNTUHQ2Qk5qLW5rdDBUblc1LWp5STdQYkpJNVduNFNrMy1ZTFRNa2ZQcW1YR0ZldjBnLWtCQVJ1UmNwMEdHMjdOS1o1cWFvTTVVM1JWWkdFeXBfUFpQZ0x1bExINkx3ZGtzSkxvNjZC?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE5IdXF1aDZ3Q3gyOUJVb2FVeVZHWG4wcTVwYUk5cGU0cUFMZjhWeFBnZzhkR0ZXaVNhOXEzTU41cUx5VDcwTFB3T0o3a0ZqTzNmSXFxTERwS2YzZG81cEVyR3JXUl9BRUVza2tHRHFn0gFuQVVfeXFMTkh1cXVoNndDeDI5QlVvYVV5VkdYbjBxNXBhSTlwZTRxQUxmOFZ4UGdnOGRHRldpU2E5cTNNTjVxTHlUNzBMUHdPSjdrRmpPM2ZJcXFMRHBLZjNkbzVwRXJHcldSX0FFRXNra0dEcWc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Spring Is In The Air” Hits Before Easter Weekend - Sneaker News</t>
+          <t>Air Jordan 1 Low OG 2026 Release Dates + Colorways - Sneaker News</t>
         </is>
       </c>
       <c r="B68" s="26" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>$200</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="E68" s="17" t="inlineStr">
@@ -3921,19 +3921,19 @@
       </c>
       <c r="H68" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPRVJwUHFMZUx3NTVVZ0NsV3hCRUVQbTRQZDE2R3R1MWlURkF4ZHRYRE1PbVpNNzZwcUM4cHdiSXFCX3NBU2hCZUJtNFhKSU1lTEtYd1ZIQnVpcnNoOTNYOWk5N2E2Wkt1UmV0UHBzM0hmMWdsZVl4SnlHU1QtUHM0OERDSUhFc085bi1KWmh3amtCWF9OVnV5a9IBmAFBVV95cUxPRVJwUHFMZUx3NTVVZ0NsV3hCRUVQbTRQZDE2R3R1MWlURkF4ZHRYRE1PbVpNNzZwcUM4cHdiSXFCX3NBU2hCZUJtNFhKSU1lTEtYd1ZIQnVpcnNoOTNYOWk5N2E2Wkt1UmV0UHBzM0hmMWdsZVl4SnlHU1QtUHM0OERDSUhFc085bi1KWmh3amtCWF9OVnV5aw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5KWmg2T21vbk01YWswamtOYXBCeGxGdGRPaE1ZTkdWVlZtTDB3VFF1STFuUG9PbFZfUDF6M1ktaHA1b1JaUmVybVB4T0JhbWdnTTBOd01BQ1did1dR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>The Nike Mind 001 Dons “Team Red” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B69" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Elephant Print Finally Arrives On This Jordan Dad Shoe - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C69" s="22" t="inlineStr">
@@ -3951,31 +3951,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F69" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G69" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F69" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G69" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPdUhnbEZUUWhwTFVvR213Z3NsazZoT190ajJkNnRDOWxuUzJsLWY0UjFfUk5jSlV6OEVUOWl1ZmZGRmxmemlHMWI2NEotdnFPTmV1UUpCTUNwcGR0NXdDZll4Vks2aWhzSHI1T0I1clAtYzN5UlFFWm5ycHlXa2hiQVVVQkcxaUtUd25Gb2VSbkx1b2dKbWhOOXlQUFBmQnfSAZ8BQVVfeXFMT3VIZ2xGVFFocExVb0dtd2dzbGs2aE9fdGoyZDZ0QzlsblMybC1mNFIxX1JOY0pVejhFVDlpdWZmRkZsZnppRzFiNjRKLXZxT05ldVFKQk1DcHBkdDV3Q2ZZeFZLNmloc0hyNU9CNXJQLWMzeVJRRVpucnB5V2toYkFVVUJHMWlLVHduRm9lUm5MdW9nSm1oTjl5UFBQZkJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZ9IBhgFBVV95cUxQeWZPNjNva1VaeHFoRTBoeTFjdV9kWlVRUWdEcDR3bzZsdEJoZTZCTGJfV2dWQnozUEM5UjY3U1hfZ3pmVVg3emotaEsxZjA3Zk5td1NCVVdrWjZsQlRwRlgyVDZXM29DclhYM0hDY3ViN1J6MmtpSXlpLVVacWZwZkJrWUxDZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>Fragment Design Gives A Peek Into The Future Of The Nike Mind Series - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B70" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>adidas Delivers A Late “Chinese New Year” Tribute On The EVO SL Trainer - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C70" s="27" t="inlineStr">
@@ -3993,26 +3993,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F70" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G70" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G70" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H70" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQajFRX3BidzVza3RsNEpsYkF0UzlCVFJGbXZXNUsySGxWd3c2MUlHRmhhNDVybmgzYld3M202aWI0dEFhOXp2NXVMVk9TRWkzQ1l3SG9vYVZYNG9tcmQyRXFmQzMyVy1idkQ0MmhPZ01ST251SlZ0TF9fWktLaXY4NDNR0gGCAUFVX3lxTFBqMVFfcGJ3NXNrdGw0SmxiQXRTOUJUUkZtdlc1SzJIbFZ3dzYxSUdGaGE0NXJuaDNiV3czbTZpYjR0QWE5enY1dUxWT1NFaTNDWXdIb29hVlg0b21yZDJFcWZDMzJXLWJ2RDQyaE9nTVJPbnVKVnRMX19aS0tpdjg0M1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQdIBfkFVX3lxTE1VSVhKTWtMOE8tRTU4aUlNMkpZd3ZKMXlUWC1XelhUSkF4MjFhb0xhVGRpYVBYTE0tdUhnVWtZcU04VXpkMFVWTkdqRFRJQlN6QkNFRjhVRWtGcWZ1ZktPeVJjMkJLUTM4N3ZCX2RWSVo5WS0xa0xtTUtpRllFQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Nike Almost Put adidas And Reebok Logos On This LeBron Shirt - Sneaker News</t>
+          <t>Nike Air Max 97 – History + Official Releases 2025 - Sneaker News</t>
         </is>
       </c>
       <c r="B71" s="30" t="inlineStr">
@@ -4025,9 +4025,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D71" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>$175</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
@@ -4047,19 +4047,19 @@
       </c>
       <c r="H71" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRd9IBckFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE5mU01lTzVJUU5lZ1d5NmxPbEpiaWI5enZZNXJkdG5EVmlQYk13Y3RvcjJFS0ZiWG9iZjhMWVBISGZoNlZpdmd2SjUzMmFKeTB4X0JYZ2VDTQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>The Jordan MVP 92 Approaches A “Tour” Colorway - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B72" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Reebok Is Restocking The Angel Reese 1 “Receipts Ready” On February 6th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="inlineStr">
+        <is>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="C72" s="27" t="inlineStr">
@@ -4077,26 +4077,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F72" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G72" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F72" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G72" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H72" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPOXZZY2ozRUpkRVpXSzl6YWsxZ2hPaWlQajVWSUZPajVSVjRmX00wOXdlNEE2amtpcmtiRVZPQl9MTnQ4eWc3TXptakxKQmw3WVBuemVCQTdoTC1sSHZCT0VmYVlDWDA1dlAwRWVwNTBLQkxBeG1XZ0plNlllNzItX0lBMnN4Y1lGeWtXaTc5WkxzZzVIME930gGXAUFVX3lxTE85dlljajNFSmRFWldLOXphazFnaE9paVBqNVZJRk9qNVJWNGZfTTA5d2U0QTZqa2lya2JFVk9CX0xOdDh5ZzdNem1qTEpCbDdZUG56ZUJBN2hMLWxIdkJPRWZhWUNYMDV2UDBFZXA1MEtCTEF4bVdnSmU2WWU3Mi1fSUEyc3hjWUZ5a1dpNzlaTHNnNUgwT3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QdIBeEFVX3lxTFAyUERwV1laRVJfbGpzU3BaUWFJdTFqeDNkcFpMemVQSkcwNjdTNWlUM0ttMmNqWlpMa3hrZnpncTNqM242SWdBUEhnWVhDSE1SM3A0Q1NkcDlRV3F3QVJKZVB6dktwNHlRZjI4dzVYYU9oa3FrenJ4QQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>The Nike Air Max Plus Gathers A “Pencil Point” Gradient - Sneaker News</t>
+          <t>The Nike Air Max Plus Carries “Pink Foam” Echoes - Sneaker News</t>
         </is>
       </c>
       <c r="B73" s="30" t="inlineStr">
@@ -4131,19 +4131,19 @@
       </c>
       <c r="H73" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOenBOTEVoZjlEY0lFejN2bGFSaVpHekxuMWkzU1VUNHNHTmpvSjVMMDdFV3ltTlEyUjhvRURDNGlDMGVFUXYwVXhvNTE1M3VoeDdaQzgyTzMtR18tY2hrMS1JZlpLNlNhVHdVOE56eDJLZ0UtLU90SFFIWGxoQXhDVlkxcEdRR01JYW53OEkzSmcyTnl4Slg5Z2RlUlnSAZwBQVVfeXFMTnpwTkxFaGY5RGNJRXozdmxhUmlaR3pMbjFpM1NVVDRzR05qb0o1TDA3RVd5bU5RMlI4b0VEQzRpQzBlRVF2MFV4bzUxNTN1aHg3WkM4Mk8zLUdfLWNoazEtSWZaSzZTYVR3VThOengyS2dFLS1PdEhRSFhsaEF4Q1ZZMXBHUUdNSWFudzhJM0pnMk55eEpYOWdkZVJZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNRU1pWDF4alUtNjJGUVFLR0hya1h1Vm5RVFJnM1BvNGh1azNHdUFld19kZS15LUZIRXZ3aUFtbnlnYlpQWTZCTHAzd1FmZi1XY3A5OUFEZ3ZXRmR0MFpNU3BFX2ZDYUYzZG10Sl96OVlBd094OUVtQ1FiR0RrbTkyc2hBQzZlVml2MWdLQ0FUakpPY0pLRXfSAZYBQVVfeXFMTUVNaVgxeGpVLTYyRlFRS0dIcmtYdVZuUVRSZzNQbzRodWszR3VBZXdfZGUteS1GSEV2d2lBbW55Z2JaUFk2QkxwM3dRZmYtV2NwOTlBRGd2V0ZkdDBaTVNwRV9mQ2FGM2RtdEpfejlZQXdPeDlFbUNRYkdEa205MnNoQUM2ZVZpdjFnS0NBVGpKT2NKS0V3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>Official Images Of The Air Jordan 3 “El Vuelo” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B74" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Where To Buy The Nike Ja 3 “Light Show” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B74" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C74" s="27" t="inlineStr">
@@ -4151,9 +4151,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D74" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E74" s="17" t="inlineStr">
@@ -4161,26 +4161,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F74" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G74" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H74" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNMkxLNHFJenQ5VUc0OXg1M2hKWGwyeUpjN25QZHRKYllRSE5TU2xvcXBNSjNqQ0RzLXF4OVVfWDdaLTkweXZQZkZlWEplQmVqbm5BZlZibXBuWWgxeTFwSlZsVkpfSXlmaTM3Y0xTOFI3ZmFBLVRyRHpCUFc3WkRaVmJKeVFhSTNz0gGIAUFVX3lxTE0yTEs0cUl6dDlVRzQ5eDUzaEpYbDJ5SmM3blBkdEpiWVFITlNTbG9xcE1KM2pDRHMtcXg5VV9YN1otOTB5dlBmRmVYSmVCZWpubkFmVmJtcG5ZaDF5MXBKVmxWSl9JeWZpMzdjTFM4UjdmYUEtVHJEekJQVzdaRFpWYkp5UWFJM3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE13M1JfZjJrYmwzdUs0N0FiS1Q2NEJQbS01TnJLbEVpNzUwMUt1NFphVmtoWTBFeU90NmNqbVNwNnNlay1HZXBHcGtRTk1wRFR5WV92MnpxSTlQUmpmUGFkNXN5QnJJaUxfOFZLVmNaMnRnUWp3TGfSAXZBVV95cUxNdzNSX2Yya2JsM3VLNDdBYktUNjRCUG0tNU5yS2xFaTc1MDFLdTRaYVZraFkwRXlPdDZjam1TcDZzZWstR2VwR3BrUU5NcERUeVlfdjJ6cUk5UFJqZlBhZDVzeUJySWlMXzhWS1ZjWjJ0Z1Fqd0xn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Nike Basketball’s Unseen Hours Collection Inspired By Hustle And Grind - Sneaker News</t>
+          <t>Kim Kardashian And NikeSkims Debut The Rift Mesh “Light Bone” - Sneaker News</t>
         </is>
       </c>
       <c r="B75" s="30" t="inlineStr">
@@ -4215,14 +4215,14 @@
       </c>
       <c r="H75" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6b9IBgAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPWVh4LUNfVjg0bFllenoxZFp1M1BxM1NQdDZCTmotbmt0MFRuVzUtanlJN1BiSkk1V240U2szLVlMVE1rZlBxbVhHRmV2MGcta0JBUnVSY3AwR0cyN05LWjVxYW9NNVUzUlZaR0V5cF9QWlBnTHVsTEg2THdka3NKTG82NkLSAYQBQVVfeXFMT1lYeC1DX1Y4NGxZZXp6MWRadTNQcTNTUHQ2Qk5qLW5rdDBUblc1LWp5STdQYkpJNVduNFNrMy1ZTFRNa2ZQcW1YR0ZldjBnLWtCQVJ1UmNwMEdHMjdOS1o1cWFvTTVVM1JWWkdFeXBfUFpQZ0x1bExINkx3ZGtzSkxvNjZC?oc=5</t>
         </is>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>Giannis Antetokounmpo’s Nike Giannis Freak 7 Launches On July 29th - Sneaker News</t>
+          <t>The Nike Mind 001 Dons “Team Red” - Sneaker News</t>
         </is>
       </c>
       <c r="B76" s="35" t="inlineStr">
@@ -4257,19 +4257,19 @@
       </c>
       <c r="H76" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbtIBeEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPdUhnbEZUUWhwTFVvR213Z3NsazZoT190ajJkNnRDOWxuUzJsLWY0UjFfUk5jSlV6OEVUOWl1ZmZGRmxmemlHMWI2NEotdnFPTmV1UUpCTUNwcGR0NXdDZll4Vks2aWhzSHI1T0I1clAtYzN5UlFFWm5ycHlXa2hiQVVVQkcxaUtUd25Gb2VSbkx1b2dKbWhOOXlQUFBmQnfSAZ8BQVVfeXFMT3VIZ2xGVFFocExVb0dtd2dzbGs2aE9fdGoyZDZ0QzlsblMybC1mNFIxX1JOY0pVejhFVDlpdWZmRkZsZnppRzFiNjRKLXZxT05ldVFKQk1DcHBkdDV3Q2ZZeFZLNmloc0hyNU9CNXJQLWMzeVJRRVpucnB5V2toYkFVVUJHMWlLVHduRm9lUm5MdW9nSm1oTjl5UFBQZkJ3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Crocheted Swooshes Appear On This Air Jordan 1 Mid - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B77" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Fragment Design Gives A Peek Into The Future Of The Nike Mind Series - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C77" s="22" t="inlineStr">
@@ -4277,9 +4277,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D77" s="8" t="inlineStr">
-        <is>
-          <t>$115</t>
+      <c r="D77" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
@@ -4287,31 +4287,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F77" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G77" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F77" s="38" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G77" s="39" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H77" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNTkIyV2h4TlA5eTFFY1hCMmYtU1ctR2tSUVBsbkpsU3F2RHRDSEtpdlJOOVgwdjJzVzF3YllrUmxrY2hpN19BVXczVDRMeXNjQTI5ZXNKS1M2MVVmTnpkUzZxUWdEOHZLVmdoSVllZzlsdXp1SVFDM0hHOVAzNWRVbExhUExtQXJ4WnBtWEIxX0h2dXdJWkk4akxJa2FETml3VFFPeEk5UDFtRDZlVTVZ0gGvAUFVX3lxTE1OQjJXaHhOUDl5MUVjWEIyZi1TVy1Ha1JRUGxuSmxTcXZEdENIS2l2Uk45WDB2MnNXMXdiWWtSbGtjaGk3X0FVdzNUNEx5c2NBMjllc0pLUzYxVWZOemRTNnFRZ0Q4dktWZ2hJWWVnOWx1enVJUUMzSEc5UDM1ZFVsTGFQTG1BcnhacG1YQjFfSHZ1d0laSThqTElrYUROaXdUUU94STlQMW1ENmVVNVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQajFRX3BidzVza3RsNEpsYkF0UzlCVFJGbXZXNUsySGxWd3c2MUlHRmhhNDVybmgzYld3M202aWI0dEFhOXp2NXVMVk9TRWkzQ1l3SG9vYVZYNG9tcmQyRXFmQzMyVy1idkQ0MmhPZ01ST251SlZ0TF9fWktLaXY4NDNR0gGCAUFVX3lxTFBqMVFfcGJ3NXNrdGw0SmxiQXRTOUJUUkZtdlc1SzJIbFZ3dzYxSUdGaGE0NXJuaDNiV3czbTZpYjR0QWE5enY1dUxWT1NFaTNDWXdIb29hVlg0b21yZDJFcWZDMzJXLWJ2RDQyaE9nTVJPbnVKVnRMX19aS0tpdjg0M1E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>adidas Celebrates Atlanta’s 404 Day With The Superstar - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B78" s="14" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Nike Almost Put adidas And Reebok Logos On This LeBron Shirt - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B78" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C78" s="27" t="inlineStr">
@@ -4341,19 +4341,19 @@
       </c>
       <c r="H78" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZ9IBfkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRd9IBckFVX3lxTE9XRTNJOHphM2pvd1FQTW9XTktQTmtza2llbWxhTXBaUXNPU3F3Q2dHSWJDOVAybUVScWhsNHowQkw4MzZEVEhuN25VZlRMZHIyTUJkREZEQnRyT0JPb0haTHZlTXphcVF6ZDY3eG9RRjJRdw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>The New Balance P350 Basketball Shoe Debuts On February 11th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B79" s="40" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>The Jordan MVP 92 Approaches A “Tour” Colorway - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C79" s="22" t="inlineStr">
@@ -4371,31 +4371,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F79" s="41" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G79" s="42" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G79" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H79" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBPckdQYi1najdwS0ozUmVvZHJDajdRQTRzN2RsT09zbi1pZmtWWm9MRDNDUDlnblAzblNSemlsMlUtNVFOejdxYzZBdkdJWVBpUTVZZTFRSHJ4UVVSMHE0UFdQWm5wYmhMRUQ5YWY1RnJTYVHSAXNBVV95cUxQT3JHUGItZ2o3cEtKM1Jlb2RyQ2o3UUE0czdkbE9Pc24taWZrVlpvTEQzQ1A5Z25QM25TUnppbDJVLTVRTno3cWM2QXZHSVlQaVE1WWUxUUhyeFFVUjBxNFBXUFpucGJoTEVEOWFmNUZyU2FR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPOXZZY2ozRUpkRVpXSzl6YWsxZ2hPaWlQajVWSUZPajVSVjRmX00wOXdlNEE2amtpcmtiRVZPQl9MTnQ4eWc3TXptakxKQmw3WVBuemVCQTdoTC1sSHZCT0VmYVlDWDA1dlAwRWVwNTBLQkxBeG1XZ0plNlllNzItX0lBMnN4Y1lGeWtXaTc5WkxzZzVIME930gGXAUFVX3lxTE85dlljajNFSmRFWldLOXphazFnaE9paVBqNVZJRk9qNVJWNGZfTTA5d2U0QTZqa2lya2JFVk9CX0xOdDh5ZzdNem1qTEpCbDdZUG56ZUJBN2hMLWxIdkJPRWZhWUNYMDV2UDBFZXA1MEtCTEF4bVdnSmU2WWU3Mi1fSUEyc3hjWUZ5a1dpNzlaTHNnNUgwT3c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>The Nike Air Max 1 Low Poly “Donkey Kong” Releases On Air Max Day - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B80" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Official Images Of The Air Jordan 3 “El Vuelo” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B80" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C80" s="27" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>$110</t>
+          <t>$200</t>
         </is>
       </c>
       <c r="E80" s="17" t="inlineStr">
@@ -4413,31 +4413,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F80" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G80" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F80" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G80" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H80" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPQ2JjMWQ3RHItN0FBaDlWZ1Z4NlV2WWZsTkRtQjJldVNEaGhGRXhpMjNsUnpUY1dRM0tvZ1lQZEpacDVRd29vZnRlNVlNRU5DVWdjSzlWU0NMRFFZZWI5d3gzVTdGU3FBQzEyY1FUNEUtczZicm0xc1M5QXdYc0M4Rmp4c0JSaDhKMmfSAYoBQVVfeXFMT0NiYzFkN0RyLTdBQWg5VmdWeDZVdllmbE5EbUIyZXVTRGhoRkV4aTIzbFJ6VGNXUTNLb2dZUGRKWnA1UXdvb2Z0ZTVZTUVOQ1VnY0s5VlNDTERRWWViOXd4M1U3RlNxQUMxMmNRVDRFLXM2YnJtMXNTOUF3WHNDOEZqeHNCUmg4SjJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNMkxLNHFJenQ5VUc0OXg1M2hKWGwyeUpjN25QZHRKYllRSE5TU2xvcXBNSjNqQ0RzLXF4OVVfWDdaLTkweXZQZkZlWEplQmVqbm5BZlZibXBuWWgxeTFwSlZsVkpfSXlmaTM3Y0xTOFI3ZmFBLVRyRHpCUFc3WkRaVmJKeVFhSTNz0gGIAUFVX3lxTE0yTEs0cUl6dDlVRzQ5eDUzaEpYbDJ5SmM3blBkdEpiWVFITlNTbG9xcE1KM2pDRHMtcXg5VV9YN1otOTB5dlBmRmVYSmVCZWpubkFmVmJtcG5ZaDF5MXBKVmxWSl9JeWZpMzdjTFM4UjdmYUEtVHJEekJQVzdaRFpWYkp5UWFJM3M?oc=5</t>
         </is>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>The Nike Structure Plus Launches February 5th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B81" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Meet The Newest New Balance Basketball Shoe, The P400 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B81" s="40" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C81" s="22" t="inlineStr">
@@ -4455,26 +4455,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G81" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F81" s="41" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G81" s="42" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H81" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUdIBZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE13Q0d5X0VaTDlsSndTUDhUYUxLTjJMX1ZnQWFiRktEN1I4S3lEazc5R1BXYXJnSUd3QUpZeWpzMW5UQS1vWHNuQ2VFM19SWEhRVDhNSmRWWC1pVENGa0N3RkptRnhZVTN3bElHQkFoS3lPV3PSAXNBVV95cUxNd0NHeV9FWkw5bEp3U1A4VGFMS04yTF9WZ0FhYkZLRDdSOEt5RGs3OUdQV2FyZ0lHd0FKWXlqczFuVEEtb1hzbkNlRTNfUlhIUVQ4TUpkVlgtaVRDRmtDd0ZKbUZ4WVUzd2xJR0JBaEt5T1dz?oc=5</t>
         </is>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>The Nike First Sight Shadow Channels The Alpha Project Basketball Era - Sneaker News</t>
+          <t>July 1st’s Nike Book 1 “Night” Continues AZ Inspirations - Sneaker News</t>
         </is>
       </c>
       <c r="B82" s="35" t="inlineStr">
@@ -4509,19 +4509,19 @@
       </c>
       <c r="H82" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUdIBckFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNMXJlN3EtRjNWNE1iWDdFeVZ0WC0wWlVpNTZYZWNOck5zZGJKMHJ6M1VXbXQwdWJxN18xbUhEYzc3VUZZV2FoZkZDOWZycldKd29QX2lXREc5LTBPQXZfdUlxay11dkJmX0JlUFJhOGZ2XzBSNERSWjY5bUhtY04tTU1hamw3NFBRcDQ2cXFybTbSAZABQVVfeXFMTTFyZTdxLUYzVjRNYlg3RXlWdFgtMFpVaTU2WGVjTnJOc2RiSjByejNVV210MHVicTdfMW1IRGM3N1VGWVdhaGZGQzlmcnJXSndvUF9pV0RHOS0wT0F2X3VJcWstdXZCZl9CZVBSYThmdl8wUjREUlo2OW1IbWNOLU1NYWpsNzRQUXA0NnFxcm02?oc=5</t>
         </is>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Bad Bunny Is Dropping His Own adidas Clothing Line - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Nike Basketball’s Unseen Hours Collection Inspired By Hustle And Grind - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B83" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C83" s="22" t="inlineStr">
@@ -4551,19 +4551,19 @@
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBibmZGRldoVjVka21ONWNCUktDajBteGNKa3kzcGltZ0pFNjFzSEI2d0paNTlzM1NkeXBzamFKay1LNTAtbEMxU09PRW9wWnVPbzFZZmtHWDhYalB0WjVoOVpTNlNZbTk0aFVWREpRM2tIMjVFbVlqZ2Z30gF6QVVfeXFMUGJuZkZGV2hWNWRrbU41Y0JSS0NqMG14Y0preTNwaW1nSkU2MXNIQjZ3Slo1OXMzU2R5cHNqYUprLUs1MC1sQzFTT09Fb3BadU9vMVlma0dYOFhqUHRaNWg5WlM2U1ltOTRoVVZESlEza0gyNUVtWWpnZnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6b9IBgAFBVV95cUxQOXBhTzd2VmdyZ3pwdU15c0stcEpWYmVjN2VIS1kwS1B3MGxVWlplUk9qcW96dFRpaWtHQU5nOVp4aVprRXUyZlR0emEtdHN1bHpVU0p4UU5TZmhSeHB4bWJUNVVpR19mSlRTQlh2cEFpX19TRFZ1aG5wbkZaMVh6bw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>The adidas Anthony Edwards 2 “Bulldawgs” Releases Ahead Of March Madness - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>Adidas</t>
+          <t>Jordan Brand Officially Unveils The Jordan Heir Series 2 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B84" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C84" s="27" t="inlineStr">
@@ -4581,31 +4581,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F84" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G84" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F84" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G84" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H84" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCONIBgwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSdIBeEFVX3lxTE1hakFSQ0JtX1VFeURiZVhHWnVKMnN4dk9VWVNLTmd4alBZcG8tOVhieXVWaG9OUVJqcWpnSXU3QnhqYTJIMUplRGdIam5NUDNxRVM1Nnd0Qmg1ay1RNlQ1RUFPZHNCMVFYRlRkT2tIcE4yWkd3WlBHSQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>Cooper Flagg Is Finally Dropping His First New Balance Shoe - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B85" s="40" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>Giannis Antetokounmpo’s Nike Giannis Freak 7 Launches On July 29th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B85" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C85" s="22" t="inlineStr">
@@ -4623,31 +4623,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F85" s="41" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G85" s="42" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTzNpWjVHV2JLVHhnQllSeDZwbjYtZVU2c2dHVURTUWdCSVdyQU05Nzh2N0RfaDdKY1BqWW9fSVZ1US12OFI1YzNWemUwMDZEMVlRdlhfV2RuZEtmZDYwOC1sblhqSDFUdGRTZy1temN2QnA2SkdkWWpfQmNhblllN2FIZVFCcG1T0gGIAUFVX3lxTE5PM2laNUdXYktUeGdCWVJ4NnBuNi1lVTZzZ0dVRFNRZ0JJV3JBTTk3OHY3RF9oN0pjUGpZb19JVnVRLXY4UjVjM1Z6ZTAwNkQxWVF2WF9XZG5kS2ZkNjA4LWxuWGpIMVR0ZFNnLW16Y3ZCcDZKR2RZal9CY2FuWWU3YUhlUUJwbVM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbtIBeEFVX3lxTFBoRjkzb2U5M1NpVjBhMlRzTGQ4alRFWHFTWlphTHdZc0J1b1BQSHN5VVNScm1tYk1zWVk5QjllQjFiaEcxT05IR1Ryd0lxUjJMc3RwWDhmTmxoUFh3enFyY1lTTVFaV0FLd1VNYkF6Wm4wUkNFdThsbg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>Easter Comes Early On The New Balance 2000 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B86" s="31" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>Crocheted Swooshes Appear On This Air Jordan 1 Mid - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B86" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C86" s="27" t="inlineStr">
@@ -4655,9 +4655,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D86" s="32" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>$115</t>
         </is>
       </c>
       <c r="E86" s="17" t="inlineStr">
@@ -4665,31 +4665,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F86" s="33" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G86" s="34" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F86" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G86" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H86" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1EQTk4ZjFuSF8yUndRR3g4SnRBeDd1V2V0eEs5MGZ6VGhtVEhkSVBQMDdoZXZ5dlNob1V4aUZucUVUcmRtdTZGeTdwV1FBR2VwZFZKelNlY2M2MVlQU2NpUmZtSTh3RHZoMmYyVzdUSFZpMTJEMkZV0gF3QVVfeXFMTURBOThmMW5IXzJSd1FHeDhKdEF4N3VXZXR4SzkwZnpUaG1USGRJUFAwN2hldnl2U2hvVXhpRm5xRVRyZG11NkZ5N3BXUUFHZXBkVkp6U2VjYzYxWVBTY2lSZm1JOHdEdmgyZjJXN1RIVmkxMkQyRlU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNTkIyV2h4TlA5eTFFY1hCMmYtU1ctR2tSUVBsbkpsU3F2RHRDSEtpdlJOOVgwdjJzVzF3YllrUmxrY2hpN19BVXczVDRMeXNjQTI5ZXNKS1M2MVVmTnpkUzZxUWdEOHZLVmdoSVllZzlsdXp1SVFDM0hHOVAzNWRVbExhUExtQXJ4WnBtWEIxX0h2dXdJWkk4akxJa2FETml3VFFPeEk5UDFtRDZlVTVZ0gGvAUFVX3lxTE1OQjJXaHhOUDl5MUVjWEIyZi1TVy1Ha1JRUGxuSmxTcXZEdENIS2l2Uk45WDB2MnNXMXdiWWtSbGtjaGk3X0FVdzNUNEx5c2NBMjllc0pLUzYxVWZOemRTNnFRZ0Q4dktWZ2hJWWVnOWx1enVJUUMzSEc5UDM1ZFVsTGFQTG1BcnhacG1YQjFfSHZ1d0laSThqTElrYUROaXdUUU94STlQMW1ENmVVNVk?oc=5</t>
         </is>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>It’s “Melo World” And The PUMA MB.05 Is Just Living In it - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B87" s="45" t="inlineStr">
-        <is>
-          <t>Puma</t>
+          <t>adidas Celebrates Atlanta’s 404 Day With The Superstar - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C87" s="22" t="inlineStr">
@@ -4707,31 +4707,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F87" s="41" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G87" s="42" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H87" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9VdmVOd0FPN3hQNXh5NEN5dGpBektnbS1vSlJFS2lBNVJKMHQxYy0wT0JRTDZ6YS02eXNWV2RaSlNDN095b0JyTnFLdlRIeDZxY295R2JDa1Buc0tUSktleUFSd05jaTFJWG0yOGxDeFlzLVJReWfSAXZBVV95cUxPVXZlTndBTzd4UDV4eTRDeXRqQXpLZ20tb0pSRUtpQTVSSjB0MWMtME9CUUw2emEtNnlzVldkWkpTQzdPeW9Cck5xS3ZUSHg2cWNveUdiQ2tQbnNLVEpLZXlBUndOY2kxSVhtMjhsQ3hZcy1SUXln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZ9IBfkFVX3lxTE1Ndk9OMTgtWHZBcE1yUmR5WFVPQ2x3WVVMa0pERmlCVEx4cGVpRGZEeFktS1JJRzFIeURIR1NhN0dLeGt6c1lnWmdpUFdFSmdvQ0tWRk5TNTNIZHdHcVN0SGs1dnlWSzRrRTNxSUVva29QNENET2c0aWVhMVhIZw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2k4 “All-Star” Returning In 2026 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B88" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The New Balance P350 Basketball Shoe Debuts On February 11th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B88" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C88" s="27" t="inlineStr">
@@ -4749,31 +4749,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F88" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G88" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F88" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G88" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H88" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNMF9pQmlnZ0swQ2hxVk5NeXlfOUFnTGVwZllMWTZGQUw3TWE4TkR3c1VFc3A0R2NWdmMwNEVIUl9uLXd0SlNWbDVJOGlla1c2TXAwRmpQeVdVdGZvdTFTTHlnVjM1RGJhOE4tTFB3cHgyRE5naklVZmtwR09MQUZ3V05CbVrSAYQBQVVfeXFMTTBfaUJpZ2dLMENocVZOTXl5XzlBZ0xlcGZZTFk2RkFMN01hOE5Ed3NVRXNwNEdjVnZjMDRFSFJfbi13dEpTVmw1SThpZWtXNk1wMEZqUHlXVXRmb3UxU0x5Z1YzNURiYThOLUxQd3B4MkROZ2pJVWZrcEdPTEFGd1dOQm1a?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBPckdQYi1najdwS0ozUmVvZHJDajdRQTRzN2RsT09zbi1pZmtWWm9MRDNDUDlnblAzblNSemlsMlUtNVFOejdxYzZBdkdJWVBpUTVZZTFRSHJ4UVVSMHE0UFdQWm5wYmhMRUQ5YWY1RnJTYVHSAXNBVV95cUxQT3JHUGItZ2o3cEtKM1Jlb2RyQ2o3UUE0czdkbE9Pc24taWZrVlpvTEQzQ1A5Z25QM25TUnppbDJVLTVRTno3cWM2QXZHSVlQaVE1WWUxUUhyeFFVUjBxNFBXUFpucGJoTEVEOWFmNUZyU2FR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>The New Balance 9060Z Puts On Two Night Vision Colorways - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B89" s="40" t="inlineStr">
-        <is>
-          <t>New Balance</t>
+          <t>The Nike Air Max 1 Low Poly “Donkey Kong” Releases On Air Max Day - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B89" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C89" s="22" t="inlineStr">
@@ -4781,9 +4781,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D89" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>$110</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
@@ -4791,26 +4791,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F89" s="41" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="G89" s="42" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H89" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5uWGpZMVVSN3ZiTVVSbzdMWXF6am5EVEdZckUxSmtBeFhZY0daQXNrMjRvMjA1WGNWWEVZc1hlel9ZOG5PRUY0TWpFUXctVTNpS3lpaGJ4dWYwQXlHVTBPZ0NiZ0c0Q2FUS2RWX1lEemJrZVHSAXNBVV95cUxOblhqWTFVUjd2Yk1VUm83TFlxempuRFRHWXJFMUprQXhYWWNHWkFzazI0bzIwNVhjVlhFWXNYZXpfWThuT0VGNE1qRVF3LVUzaUt5aWhieHVmMEF5R1UwT2dDYmdHNENhVEtkVl9ZRHpia2VR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPQ2JjMWQ3RHItN0FBaDlWZ1Z4NlV2WWZsTkRtQjJldVNEaGhGRXhpMjNsUnpUY1dRM0tvZ1lQZEpacDVRd29vZnRlNVlNRU5DVWdjSzlWU0NMRFFZZWI5d3gzVTdGU3FBQzEyY1FUNEUtczZicm0xc1M5QXdYc0M4Rmp4c0JSaDhKMmfSAYoBQVVfeXFMT0NiYzFkN0RyLTdBQWg5VmdWeDZVdllmbE5EbUIyZXVTRGhoRkV4aTIzbFJ6VGNXUTNLb2dZUGRKWnA1UXdvb2Z0ZTVZTUVOQ1VnY0s5VlNDTERRWWViOXd4M1U3RlNxQUMxMmNRVDRFLXM2YnJtMXNTOUF3WHNDOEZqeHNCUmg4SjJn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>Official Images Of The Nike A’One “Indigo Girl” - Sneaker News</t>
+          <t>The Nike Structure Plus Launches February 5th - Sneaker News</t>
         </is>
       </c>
       <c r="B90" s="35" t="inlineStr">
@@ -4845,19 +4845,19 @@
       </c>
       <c r="H90" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1obUpQQWoxMExaOUl1N20tZllnMVdLbVJwX1FXcGprMmg1TjE1d2NkMzV3NW1wOHc4UWU1eHZtUDF2Z1V4MGFxUXF0WTJTZ0NoUnk1TW1sYmc1TElYSlJLcHNXcjZOWjVUMnFqZExGeHNNTlZ5c0HSAXZBVV95cUxNaG1KUEFqMTBMWjlJdTdtLWZZZzFXS21ScF9RV3BqazJoNU4xNXdjZDM1dzVtcDh3OFFlNXh2bVAxdmdVeDBhcVFxdFkyU2dDaFJ5NU1tbGJnNUxJWEpSS3BzV3I2Tlo1VDJxamRMRnhzTU5WeXNB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUdIBZkFVX3lxTE92c0ZPTWhWNzdCRldQcndBdlNQRDZLUlhnWTlJRTM3dHBiNXUwa2NZTk9jaEtuYkl5eThkV3JVOTV5TFFwRmZzVXowUEpaR1BrMXM0SENWNlFHaFRGSDd5LV9EUnBJUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>YOASOBI’s “Just A Little Step” Turns Into An ASICS Sneaker Collaboration - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B91" s="23" t="inlineStr">
-        <is>
-          <t>ASICS</t>
+          <t>Nike Air Foamposite One “Floral” Returns Holiday 2026 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B91" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C91" s="22" t="inlineStr">
@@ -4875,31 +4875,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F91" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G91" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB4Sm1iZVVLNE9LS1VTSkMwLWViNkE2R3gzZXhyWlVOeGFxdVhMY3pyZXl6enZjb0xYbk9nWkt5SXlKNGlNSVlubjB3NmwtU1h2M3gwZlN5dk42UVhPaDNXcmNJZVBoN3FzYUdlWmNZNlgzVTNiN2lz0gF3QVVfeXFMUHhKbWJlVUs0T0tLVVNKQzAtZWI2QTZHeDNleHJaVU54YXF1WExjenJleXp6dmNvTFhuT2daS3lJeUo0aU1JWW5uMHc2bC1TWHYzeDBmU3l2TjZRWE9oM1dyY0llUGg3cXNhR2VaY1k2WDNVM2I3aXM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPYnBkY0s4NDRsS1dua05XVmg0ZzZZMkZTenNwbDBKc2thRXRwSXVvQ1hMLVJ5UEpBem9oeXMwZFhKODVWaE5PN3hsOG90eGM4RnY2NFJ1akhKZ2k5M3lVSmlsSm5wTFpIRG1zMDZlWDhHTG13U0lMVUwyQ3UxY0Z0aWgwZkNSSXF2SFHSAYoBQVVfeXFMT2JwZGNLODQ0bEtXbmtOV1ZoNGc2WTJGU3pzcGwwSnNrYUV0cEl1b0NYTC1SeVBKQXpvaHlzMGRYSjg1VmhOTzd4bDhvdHhjOEZ2NjRSdWpISmdpOTN5VUppbEpucExaSERtczA2ZVg4R0xtd1NJTFVMMkN1MWNGdGloMGZDUklxdkhR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Wolf Grey” Postponed To February 28th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B92" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>The Nike First Sight Shadow Channels The Alpha Project Basketball Era - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B92" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C92" s="27" t="inlineStr">
@@ -4907,9 +4907,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D92" s="16" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D92" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E92" s="17" t="inlineStr">
@@ -4917,31 +4917,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F92" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G92" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G92" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H92" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1xZHFjb1Q4RmZpbXB4cTFoblVaZmJOUUFVZEtWWWttelpYSGN4czg2bGx4WVN2Z1hWTkQ2bnNvbVhHbFcybmdDLXlCd29fNVNRYU9GVXItdnc0MjV2TFhwamY1MWpFQlJTSmNlNmN0d1VzSUNEc0V2dFFYUnI3RTjSAX9BVV95cUxNcWRxY29UOEZmaW1weHExaG5VWmZiTlFBVWRLVllrbXpaWEhjeHM4NmxseFlTdmdYVk5ENm5zb21YR2xXMm5nQy15QndvXzVTUWFPRlVyLXZ3NDI1dkxYcGpmNTFqRUJSU0pjZTZjdHdVc0lDRHNFdnRRWFJyN0U4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUdIBckFVX3lxTFBPOWs4SnhtTHl0dXh2ZWZGQlNqX2dQMFcxZ05WVDZQcmRFN2IwUVJWd0hSTzhzdG9OLVB4cjhRV2RvbWdndEhveVZaUFBGNWpSY054Q193RXptTzZYM1dPUjRQWUVibGE0N2d5ZjU5d0ZUUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>The Nike Mind 002 “Black/Hyper Crimson” Releases On February 5th - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B93" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Bad Bunny Is Dropping His Own adidas Clothing Line - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C93" s="22" t="inlineStr">
@@ -4971,19 +4971,19 @@
       </c>
       <c r="H93" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOcTYtWWhHTGk4T09CbElTMFpzT3J3dUF0OGxrNEVtY3AxeHRYRjc2WDVfQXlxQllnQzM4UXlGVHd5Y3d0NHdCTHZHS2kzSHZ1VEFGWi03UFJEUS01cG5ySGl2UGVjWlZ0OGpwSE5rdHgzZ3B0TW5kZ3p2Z3piV3ltOHdPczVyZ3NneFduWm1nMnDSAZABQVVfeXFMTnE2LVloR0xpOE9PQmxJUzBac09yd3VBdDhsazRFbWNwMXh0WEY3Nlg1X0F5cUJZZ0MzOFF5RlR3eWN3dDR3Qkx2R0tpM0h2dVRBRlotN1BSRFEtNXBuckhpdlBlY1pWdDhqcEhOa3R4M2dwdE1uZGd6dmd6Yld5bTh3T3M1cmdzZ3hXblptZzJw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTFBibmZGRldoVjVka21ONWNCUktDajBteGNKa3kzcGltZ0pFNjFzSEI2d0paNTlzM1NkeXBzamFKay1LNTAtbEMxU09PRW9wWnVPbzFZZmtHWDhYalB0WjVoOVpTNlNZbTk0aFVWREpRM2tIMjVFbVlqZ2Z30gF6QVVfeXFMUGJuZkZGV2hWNWRrbU41Y0JSS0NqMG14Y0preTNwaW1nSkU2MXNIQjZ3Slo1OXMzU2R5cHNqYUprLUs1MC1sQzFTT09Fb3BadU9vMVlma0dYOFhqUHRaNWg5WlM2U1ltOTRoVVZESlEza0gyNUVtWWpnZnc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>Patta x Nike Air Max 1 “Hyper Crimson” Is Available Now - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B94" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>The adidas Anthony Edwards 2 “Bulldawgs” Releases Ahead Of March Madness - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="C94" s="27" t="inlineStr">
@@ -4991,9 +4991,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D94" s="16" t="inlineStr">
-        <is>
-          <t>$110</t>
+      <c r="D94" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E94" s="17" t="inlineStr">
@@ -5001,31 +5001,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F94" s="36" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G94" s="37" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G94" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H94" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQb2RIdkRFNmlXWWIybWQxWTRjOVdhUlVFUTJ2TXpyNHR4RlhyZ3FTQnQtS3FkekhwdGYwZ1RzLU1qcHV0V0thSDRJbVgtR3M1ZFJsb0p6Ny1Cbi1fZDRXajhldGZtN2xqNjhTazNORkpIYkhkZFdMVTk1U2FnUFNxMklyNWMxcnB4VVlB0gGLAUFVX3lxTFBvZEh2REU2aVdZYjJtZDFZNGM5V2FSVUVRMnZNenI0dHhGWHJncVNCdC1LcWR6SHB0ZjBnVHMtTWpwdXRXS2FINEltWC1HczVkUmxvSno3LUJuLV9kNFdqOGV0Zm03bGo2OFNrM05GSkhiSGRkV0xVOTVTYWdQU3EySXI1YzFycHhVWUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCONIBgwFBVV95cUxOdEgtV25rQ2NEUDJtcWNIMVdBbjRXcWRNdzd2amJ2SjJOV1F1MjJzZ0JnWkdObElaNzRNbDVxS1JjOTd4NGtGVTlxalBRd3l5QjlWTnhGU3lhUGl0NDRSMGZodHdKYjJ0bmNQZHZaZUxtbFF2a1dfZE16ZXVsS0k5S0JCOA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Kobe Bryant – Nike adidas Shoes + Career - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B95" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Cooper Flagg Is Finally Dropping His First New Balance Shoe - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B95" s="40" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C95" s="22" t="inlineStr">
@@ -5043,31 +5043,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F95" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G95" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F95" s="41" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G95" s="42" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H95" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE94aFo5aE9GdkpSMS04a2NnM29ZUDlRRkNZNzJ1amkxUXRvcHBKbW04VjdiTVdvVE5rTHZPUXZGWkwyMGl3cTl3alVHY0hTSHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTzNpWjVHV2JLVHhnQllSeDZwbjYtZVU2c2dHVURTUWdCSVdyQU05Nzh2N0RfaDdKY1BqWW9fSVZ1US12OFI1YzNWemUwMDZEMVlRdlhfV2RuZEtmZDYwOC1sblhqSDFUdGRTZy1temN2QnA2SkdkWWpfQmNhblllN2FIZVFCcG1T0gGIAUFVX3lxTE5PM2laNUdXYktUeGdCWVJ4NnBuNi1lVTZzZ0dVRFNRZ0JJV3JBTTk3OHY3RF9oN0pjUGpZb19JVnVRLXY4UjVjM1Z6ZTAwNkQxWVF2WF9XZG5kS2ZkNjA4LWxuWGpIMVR0ZFNnLW16Y3ZCcDZKR2RZal9CY2FuWWU3YUhlUUJwbVM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>Nike Is Releasing A Triple White Ja 2 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B96" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Easter Comes Early On The New Balance 2000 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B96" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C96" s="27" t="inlineStr">
@@ -5085,31 +5085,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F96" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G96" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F96" s="33" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G96" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H96" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBmUWxueWp2bV81VFRzTDd6SkpnNE4xbGx1RmRuNFF1blNWYlRWMDNYR1BtbU9WcEpzd3JnMEw2aWhTRk9zWWktOXJ0YnBiMEFudjR4MFVMdkhhb2FUdEJ1ZWVBbTFDQjFsZ0hpSG9tOEJNLU1Zc09R0gF3QVVfeXFMUGZRbG55anZtXzVUVHNMN3pKSmc0TjFsbHVGZG40UXVuU1ZiVFYwM1hHUG1tT1ZwSnN3cmcwTDZpaFNGT3NZaS05cnRicGIwQW52NHgwVUx2SGFvYVR0QnVlZUFtMUNCMWxnSGlIb204Qk0tTVlzT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1EQTk4ZjFuSF8yUndRR3g4SnRBeDd1V2V0eEs5MGZ6VGhtVEhkSVBQMDdoZXZ5dlNob1V4aUZucUVUcmRtdTZGeTdwV1FBR2VwZFZKelNlY2M2MVlQU2NpUmZtSTh3RHZoMmYyVzdUSFZpMTJEMkZV0gF3QVVfeXFMTURBOThmMW5IXzJSd1FHeDhKdEF4N3VXZXR4SzkwZnpUaG1USGRJUFAwN2hldnl2U2hvVXhpRm5xRVRyZG11NkZ5N3BXUUFHZXBkVkp6U2VjYzYxWVBTY2lSZm1JOHdEdmgyZjJXN1RIVmkxMkQyRlU?oc=5</t>
         </is>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Travis Scott Shoes, “Valentine” Jordan 3, And This Week’s Best Releases - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B97" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>It’s “Melo World” And The PUMA MB.05 Is Just Living In it - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B97" s="45" t="inlineStr">
+        <is>
+          <t>Puma</t>
         </is>
       </c>
       <c r="C97" s="22" t="inlineStr">
@@ -5127,26 +5127,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F97" s="38" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="G97" s="39" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
+      <c r="F97" s="41" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="G97" s="42" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
         </is>
       </c>
       <c r="H97" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUdIBhgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9VdmVOd0FPN3hQNXh5NEN5dGpBektnbS1vSlJFS2lBNVJKMHQxYy0wT0JRTDZ6YS02eXNWV2RaSlNDN095b0JyTnFLdlRIeDZxY295R2JDa1Buc0tUSktleUFSd05jaTFJWG0yOGxDeFlzLVJReWfSAXZBVV95cUxPVXZlTndBTzd4UDV4eTRDeXRqQXpLZ20tb0pSRUtpQTVSSjB0MWMtME9CUUw2emEtNnlzVldkWkpTQzdPeW9Cck5xS3ZUSHg2cWNveUdiQ2tQbnNLVEpLZXlBUndOY2kxSVhtMjhsQ3hZcy1SUXln?oc=5</t>
         </is>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>Nike Prepares For April Showers With A New Batch Of Air Force 1 Vibram Options - Sneaker News</t>
+          <t>Nike LeBron 23 Unveiled - Sneaker News</t>
         </is>
       </c>
       <c r="B98" s="35" t="inlineStr">
@@ -5181,19 +5181,19 @@
       </c>
       <c r="H98" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CN9IBgAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE9iaUkzUDRSbVRzUE5sTlczbGNtbEZjRVFwb0JsTkRjMW9lQXRnZ2FjVlZUOWhFeFZsSUxnLW1URnl1S0tTdldXYnVfNlVBOUNlWkpoVHItaUFLcnhiellj0gFfQVVfeXFMT2JpSTNQNFJtVHNQTmxOVzNsY21sRmNFUXBvQmxORGMxb2VBdGdnYWNWVlQ5aEV4VmxJTGctbVRGeXVLS1N2V1didV82VUE5Q2VaSmhUci1pQUtyeGJ6WWM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>Detailed Look At The Paris Saint-Germain x Air Jordan 6 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B99" s="21" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Zoom Huarache 2k4 “All-Star” Returning In 2026 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B99" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C99" s="22" t="inlineStr">
@@ -5201,9 +5201,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D99" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
@@ -5211,31 +5211,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F99" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G99" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE44ZFVoWFRjQTREMXVva2o4S1lQX004N09PbFZNN0RmSkhiRUNxQkJGYldTVEJuSEdLX1g2dHJidmNOV1hNNVQzVEFDUDBZYy0wTXU1dzd2dzN1Wm5LMVhIU0FUUnp5emlsa0FxYjhyZGfSAXBBVV95cUxOOGRVaFhUY0E0RDF1b2tqOEtZUF9NODdPT2xWTTdEZkpIYkVDcUJCRmJXU1RCbkhHS19YNnRyYnZjTldYTTVUM1RBQ1AwWWMtME11NXc3dnczdVpuSzFYSFNBVFJ6eXppbGtBcWI4cmRn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNMF9pQmlnZ0swQ2hxVk5NeXlfOUFnTGVwZllMWTZGQUw3TWE4TkR3c1VFc3A0R2NWdmMwNEVIUl9uLXd0SlNWbDVJOGlla1c2TXAwRmpQeVdVdGZvdTFTTHlnVjM1RGJhOE4tTFB3cHgyRE5naklVZmtwR09MQUZ3V05CbVrSAYQBQVVfeXFMTTBfaUJpZ2dLMENocVZOTXl5XzlBZ0xlcGZZTFk2RkFMN01hOE5Ed3NVRXNwNEdjVnZjMDRFSFJfbi13dEpTVmw1SThpZWtXNk1wMEZqUHlXVXRmb3UxU0x5Z1YzNURiYThOLUxQd3B4MkROZ2pJVWZrcEdPTEFGd1dOQm1a?oc=5</t>
         </is>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>The ASICS GEL-Kayano 14 Pounds The Pavement In “Concrete” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B100" s="32" t="inlineStr">
-        <is>
-          <t>ASICS</t>
+          <t>The New Balance 9060Z Puts On Two Night Vision Colorways - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B100" s="31" t="inlineStr">
+        <is>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="C100" s="27" t="inlineStr">
@@ -5265,19 +5265,19 @@
       </c>
       <c r="H100" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOaGpiQjhhMWd3ZVhQZVJ4N2ozM1JPeHNvYURaa1BGbzhseW9hdFlQNC1ZaWRST3RQTEhJaElqanpVRldWVzBVLVd5ZUo1RW0tcFliQXJWdVVkbi13NlVMRDJ2aUI3eGxGY2w1TlhVVTYtU0ZWekRSMEtVa1ZNbEhXV0tqMktlckZMaUNqLVh3WUU3Y2fSAZMBQVVfeXFMTmhqYkI4YTFnd2VYUGVSeDdqMzNST3hzb2FEWmtQRm84bHlvYXRZUDQtWWlkUk90UExISWhJamp6VUZXVlcwVS1XeWVKNUVtLXBZYkFyVnVVZG4tdzZVTEQydmlCN3hsRmNsNU5YVVU2LVNGVnpEUjBLVWtWTWxIV1dLajJLZXJGTGlDai1Yd1lFN2Nn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5uWGpZMVVSN3ZiTVVSbzdMWXF6am5EVEdZckUxSmtBeFhZY0daQXNrMjRvMjA1WGNWWEVZc1hlel9ZOG5PRUY0TWpFUXctVTNpS3lpaGJ4dWYwQXlHVTBPZ0NiZ0c0Q2FUS2RWX1lEemJrZVHSAXNBVV95cUxOblhqWTFVUjd2Yk1VUm83TFlxempuRFRHWXJFMUprQXhYWWNHWkFzazI0bzIwNVhjVlhFWXNYZXpfWThuT0VGNE1qRVF3LVUzaUt5aWhieHVmMEF5R1UwT2dDYmdHNENhVEtkVl9ZRHpia2VR?oc=5</t>
         </is>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>The Cult Classic Nike Air Max Plus VII Drips On “Blue Crystal” - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B101" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>YOASOBI’s “Just A Little Step” Turns Into An ASICS Sneaker Collaboration - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>ASICS</t>
         </is>
       </c>
       <c r="C101" s="22" t="inlineStr">
@@ -5285,9 +5285,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D101" s="8" t="inlineStr">
-        <is>
-          <t>$160</t>
+      <c r="D101" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
@@ -5295,31 +5295,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F101" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G101" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F101" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G101" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQeEpmWW9SS0I3TUtfNXpSaUx4ZTRuODBKeFR3eHBVZlo5bk9CbkdmRVJjd3dsOXRuNTlCX0tDXzhBUk1NZ0I3WUdQWUhiN2VzQkhETEtYbEdVWXAwWF9JRjRfV2NQeTFDbDIwMmxGOWdlQzBMck1iVWZPQWZRYUpfN1Y5NjdqRVBVQWhyZ1lIYjNOSFBFc3F1YWRUR1JIeUs1dk5XN2ZR0gGmAUFVX3lxTFB4SmZZb1JLQjdNS181elJpTHhlNG44MEp4VHd4cFVmWjluT0JuR2ZFUmN3d2w5dG41OUJfS0NfOEFSTU1nQjdZR1BZSGI3ZXNCSERMS1hsR1VZcDBYX0lGNF9XY1B5MUNsMjAybEY5Z2VDMExyTWJVZk9BZlFhSl83Vjk2N2pFUFVBaHJnWUhiM05IUEVzcXVhZFRHUkh5SzV2Tlc3ZlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB4Sm1iZVVLNE9LS1VTSkMwLWViNkE2R3gzZXhyWlVOeGFxdVhMY3pyZXl6enZjb0xYbk9nWkt5SXlKNGlNSVlubjB3NmwtU1h2M3gwZlN5dk42UVhPaDNXcmNJZVBoN3FzYUdlWmNZNlgzVTNiN2lz0gF3QVVfeXFMUHhKbWJlVUs0T0tLVVNKQzAtZWI2QTZHeDNleHJaVU54YXF1WExjenJleXp6dmNvTFhuT2daS3lJeUo0aU1JWW5uMHc2bC1TWHYzeDBmU3l2TjZRWE9oM1dyY0llUGg3cXNhR2VaY1k2WDNVM2I3aXM?oc=5</t>
         </is>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>Nike Air Max 270 MLB City Connect Pack Is Available Now - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B102" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Nike Mind 001 / 002, Jordan Luka 5, And This Week’s Best Releases - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B102" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C102" s="27" t="inlineStr">
@@ -5327,9 +5327,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D102" s="16" t="inlineStr">
-        <is>
-          <t>$150</t>
+      <c r="D102" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E102" s="17" t="inlineStr">
@@ -5337,31 +5337,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F102" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G102" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F102" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G102" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H102" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5FVUN2bXpiRDgteEQ3bWxaSlZEZ3dZR1VFWU9RN2JnYVBHb1JTR0EyZDhydVluczN2MnRUaml3S0luWEZmb2p4WmlLY2pMd3I2UmtZS2xZNFdZSmlQREhMRDRMOWtDWEhsUUhSTjdkOUppbkJHQ3lrZGZyejVoZUHSAX9BVV95cUxORVVDdm16YkQ4LXhEN21sWkpWRGd3WUdVRVlPUTdiZ2FQR29SU0dBMmQ4cnVZbnMzdjJ0VGppd0tJblhGZm9qeFppS2NqTHdyNlJrWUtsWTRXWUppUERITEQ0TDlrQ1hIbFFIUk43ZDlKaW5CR0N5a2Rmcno1aGVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOdnkwZWZXT0REVVhjQnBXZzBVaGFPT3JDZGxCck12dHhwbXE2aDFUWDNfTWdyTTJpNnJwMzFqR2w1RkNrbFpkZExyQXRWMDU2UGpiSnA5T0V2MVNBcDRuVFcxeFNEd2U4eC1mLVNreHh6ZWlPVHE0cGJGYlF5SDV0amRnSkvSAYQBQVVfeXFMTnZ5MGVmV09ERFVYY0JwV2cwVWhhT09yQ2RsQnJNdnR4cG1xNmgxVFgzX01nck0yaTZycDMxakdsNUZDa2xaZGRMckF0VjA1NlBqYkpwOU9FdjFTQXA0blRXMXhTRHdlOHgtZi1Ta3h4emVpT1RxNHBiRmJReUg1dGpkZ0pL?oc=5</t>
         </is>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Nike Reloads The Mesh-Backed Air Force 1 Low For Spring - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B103" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Air Jordan 5 “Wolf Grey” Postponed To February 28th - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B103" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C103" s="22" t="inlineStr">
@@ -5369,9 +5369,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D103" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
@@ -5379,26 +5379,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F103" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G103" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F103" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G103" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H103" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOVE1tb0YxejhwZFVEMW8zS0V5WkVvckZVT2FwVDNNTU5nRkU4SnZ4Yk12bElLdjRhUXhBaWN3eDdYVkJtV2wxNFJEdmtPN2FNTzZRblBrRTFORENkd1FEWTdvRTJTUDN2N3M2dGdzVExJelhVczM2ZzJTSjNpd2t5cEpDdjFhUXhteHduQktHcTTSAZABQVVfeXFMTlRNbW9GMXo4cGRVRDFvM0tFeVpFb3JGVU9hcFQzTU1OZ0ZFOEp2eGJNdmxJS3Y0YVF4QWljd3g3WFZCbVdsMTRSRHZrTzdhTU82UW5Qa0UxTkRDZHdRRFk3b0UyU1AzdjdzNnRnc1RMSXpYVXMzNmcyU0ozaXdreXBKQ3YxYVF4bXh3bkJLR3E0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1xZHFjb1Q4RmZpbXB4cTFoblVaZmJOUUFVZEtWWWttelpYSGN4czg2bGx4WVN2Z1hWTkQ2bnNvbVhHbFcybmdDLXlCd29fNVNRYU9GVXItdnc0MjV2TFhwamY1MWpFQlJTSmNlNmN0d1VzSUNEc0V2dFFYUnI3RTjSAX9BVV95cUxNcWRxY29UOEZmaW1weHExaG5VWmZiTlFBVWRLVllrbXpaWEhjeHM4NmxseFlTdmdYVk5ENm5zb21YR2xXMm5nQy15QndvXzVTUWFPRlVyLXZ3NDI1dkxYcGpmNTFqRUJSU0pjZTZjdHdVc0lDRHNFdnRRWFJyN0U4?oc=5</t>
         </is>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>The Nike KD 4 “Gold Medal” Is Back Thirteen Years Later - Sneaker News</t>
+          <t>The Nike Mind 002 “Black/Hyper Crimson” Releases On February 5th - Sneaker News</t>
         </is>
       </c>
       <c r="B104" s="35" t="inlineStr">
@@ -5433,14 +5433,14 @@
       </c>
       <c r="H104" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE95Y1JPVm5xQUIwWGk4UE84MzlwbW4zZUItSWsyWm01a0FISUVFN1RuVDJqOVBRX0szdkpFMmIxcGVIUWp0d3AxaUFxVl9iSFJkMzR1S2xqTnVTTExsUk5zU0hPcUxFc1pPT3AzcU5yeFVCR2E3NVHSAXZBVV95cUxPeWNST1ZucUFCMFhpOFBPODM5cG1uM2VCLUlrMlptNWtBSElFRTdUblQyajlQUV9LM3ZKRTJiMXBlSFFqdHdwMWlBcVZfYkhSZDM0dUtsak51U0xMbFJOc1NIT3FMRXNaT09wM3FOcnhVQkdhNzVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOcTYtWWhHTGk4T09CbElTMFpzT3J3dUF0OGxrNEVtY3AxeHRYRjc2WDVfQXlxQllnQzM4UXlGVHd5Y3d0NHdCTHZHS2kzSHZ1VEFGWi03UFJEUS01cG5ySGl2UGVjWlZ0OGpwSE5rdHgzZ3B0TW5kZ3p2Z3piV3ltOHdPczVyZ3NneFduWm1nMnDSAZABQVVfeXFMTnE2LVloR0xpOE9PQmxJUzBac09yd3VBdDhsazRFbWNwMXh0WEY3Nlg1X0F5cUJZZ0MzOFF5RlR3eWN3dDR3Qkx2R0tpM0h2dVRBRlotN1BSRFEtNXBuckhpdlBlY1pWdDhqcEhOa3R4M2dwdE1uZGd6dmd6Yld5bTh3T3M1cmdzZ3hXblptZzJw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Nike Zoom GT Cut 3 “Christmas” Has Pockets Of Snowy Glitter - Sneaker News</t>
+          <t>Patta x Nike Air Max 1 “Hyper Crimson” Is Available Now - Sneaker News</t>
         </is>
       </c>
       <c r="B105" s="30" t="inlineStr">
@@ -5453,9 +5453,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D105" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>$110</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
@@ -5463,31 +5463,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F105" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G105" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F105" s="38" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G105" s="39" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H105" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNMXNwZy1kLUJaQmhEVEFOdC1mZXhuaURoTUpwVjFzb0tpLTBuTXlvZVZ1QWYtSDBuMUkyZFZCYkpMZGlHN0c0WWc2dWJ4VXRxbjNNaWg4TjhMT19XQzdQQTk1QWFpaU9md1BOX2V2VFp6TkZwdWhzc3pnMnpKbVFtTdIBgAFBVV95cUxNMXNwZy1kLUJaQmhEVEFOdC1mZXhuaURoTUpwVjFzb0tpLTBuTXlvZVZ1QWYtSDBuMUkyZFZCYkpMZGlHN0c0WWc2dWJ4VXRxbjNNaWg4TjhMT19XQzdQQTk1QWFpaU9md1BOX2V2VFp6TkZwdWhzc3pnMnpKbVFtTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQb2RIdkRFNmlXWWIybWQxWTRjOVdhUlVFUTJ2TXpyNHR4RlhyZ3FTQnQtS3FkekhwdGYwZ1RzLU1qcHV0V0thSDRJbVgtR3M1ZFJsb0p6Ny1Cbi1fZDRXajhldGZtN2xqNjhTazNORkpIYkhkZFdMVTk1U2FnUFNxMklyNWMxcnB4VVlB0gGLAUFVX3lxTFBvZEh2REU2aVdZYjJtZDFZNGM5V2FSVUVRMnZNenI0dHhGWHJncVNCdC1LcWR6SHB0ZjBnVHMtTWpwdXRXS2FINEltWC1HczVkUmxvSno3LUJuLV9kNFdqOGV0Zm03bGo2OFNrM05GSkhiSGRkV0xVOTVTYWdQU3EySXI1YzFycHhVWUE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>The Air Jordan 3 Is Ready For Spring Flowers - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B106" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Is Releasing A Triple White Ja 2 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B106" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C106" s="27" t="inlineStr">
@@ -5495,9 +5495,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D106" s="16" t="inlineStr">
-        <is>
-          <t>$200</t>
+      <c r="D106" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E106" s="17" t="inlineStr">
@@ -5505,26 +5505,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F106" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G106" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F106" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G106" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H106" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBKNm5kUk1FRzlhaHI1T0MwTUJQNXd5eEdfX0ZGcXJsOTI3REpwRER2bXRJMVBlNk1Qa1lsNE4yTWhMcHhQUzlpTGdLeXVwZzFUc2lGWjM5R2R2ckdLMjZlMm9KZnlQRHV6bE5FenpBQ3k5ZjZ6QWFIaGZ5OGJyLTjSAX9BVV95cUxQSjZuZFJNRUc5YWhyNU9DME1CUDV3eXhHX19GRnFybDkyN0RKcEREdm10STFQZTZNUGtZbDROMk1oTHB4UFM5aUxnS3l1cGcxVHNpRlozOUdkdnJHSzI2ZTJvSmZ5UER1emxORXp6QUN5OWY2ekFhSGhmeThici04?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBmUWxueWp2bV81VFRzTDd6SkpnNE4xbGx1RmRuNFF1blNWYlRWMDNYR1BtbU9WcEpzd3JnMEw2aWhTRk9zWWktOXJ0YnBiMEFudjR4MFVMdkhhb2FUdEJ1ZWVBbTFDQjFsZ0hpSG9tOEJNLU1Zc09R0gF3QVVfeXFMUGZRbG55anZtXzVUVHNMN3pKSmc0TjFsbHVGZG40UXVuU1ZiVFYwM1hHUG1tT1ZwSnN3cmcwTDZpaFNGT3NZaS05cnRicGIwQW52NHgwVUx2SGFvYVR0QnVlZUFtMUNCMWxnSGlIb204Qk0tTVlzT1E?oc=5</t>
         </is>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>The Air Jordan 40 Does Its Best XX3 Impression With Perfect Detailing - Sneaker News</t>
+          <t>Travis Scott Shoes, “Valentine” Jordan 3, And This Week’s Best Releases - Sneaker News</t>
         </is>
       </c>
       <c r="B107" s="21" t="inlineStr">
@@ -5537,9 +5537,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D107" s="8" t="inlineStr">
-        <is>
-          <t>$210</t>
+      <c r="D107" s="23" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
@@ -5547,31 +5547,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F107" s="24" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G107" s="25" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F107" s="38" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="G107" s="39" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
         </is>
       </c>
       <c r="H107" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE1IeUNNTWFCckJ4Nk41dkYyRlZqYTRqSGpDRTB5NUlWRUlJRk5uTjRMSnNIUmpOSWJFa2hhd25SdGpxTFlDd1VrdU5zX1hUV2Y0OGs5UU5ZMnlRTGFCNmJhOUVjSnJRenNMVVI4YUFyQjnSAXBBVV95cUxNSHlDTU1hQnJCeDZONXZGMkZWamE0akhqQ0UweTVJVkVJSUZObk40TEpzSFJqTkliRWtoYXduUnRqcUxZQ3dVa3VOc19YVFdmNDhrOVFOWTJ5UUxhQjZiYTlFY0pyUXpzTFVSOGFBckI5?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUdIBhgFBVV95cUxQTnNXRUZZNTM3c0RNT1pPWUJtYVluYXRyaWVYUGZwLWFvWTBNZk9UU2Mxd1BNZkR3QTA4Z3BJbXlLaE55NTgxZ1d2SjdWUkRvQktoV0ZXX2gyZERRdVd2WjAyZ0VDaC1uUzk1dTVCdkFULUxWY2RvcDFwN29xQTVIN0pHWFdlUQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Taxi,” Air Jordan 11 “Rare Air,” And This Week’s Best Releases - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B108" s="26" t="inlineStr">
-        <is>
-          <t>Jordan</t>
+          <t>Nike Prepares For April Showers With A New Batch Of Air Force 1 Vibram Options - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B108" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C108" s="27" t="inlineStr">
@@ -5579,9 +5579,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D108" s="16" t="inlineStr">
-        <is>
-          <t>$220</t>
+      <c r="D108" s="32" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E108" s="17" t="inlineStr">
@@ -5589,31 +5589,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F108" s="28" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="G108" s="29" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
+      <c r="F108" s="18" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="G108" s="19" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
         </is>
       </c>
       <c r="H108" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5TVzdKTERaMGY0Mi1iRzhPMjBMbUQwaVhVTGUwR013bER2VGFRVXRxc2xYcXBjTjhkY2NnR1FER3ItNDJFeW9LQ3dkTF9wUTZySmozc2dXZ2pRSmoybnhIRzdkc193dHFGMTBXTlZtNHRlSmo4eXRjQWVzYXlEYkHSAX9BVV95cUxOU1c3SkxEWjBmNDItYkc4TzIwTG1EMGlYVUxlMEdNd2xEdlRhUVV0cXNsWHFwY044ZGNjZ0dRREdyLTQyRXlvS0N3ZExfcFE2ckpqM3NnV2dqUUpqMm54SEc3ZHNfd3RxRjEwV05WbTR0ZUpqOHl0Y0Flc2F5RGJB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CN9IBgAFBVV95cUxPWVdXdW1uR09vc1kyRC1MY1phNVB4WjVMV2JCMjRnaE41TndkWmZUbW5aVzVlWTd0ZGhCMURLazFVd1VNTHFJTTJPU3F6LVYySjZpU25kN2hQdnJuY3FySlJhazdMMHphVHh5a3hzWkdsQ1pWN0R5c2xDY2g1a25CNw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>Air Max 95 “Blue Spark,” Ja 3 “Light Show” And This Week’s Best Releases - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B109" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Detailed Look At The Paris Saint-Germain x Air Jordan 6 - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B109" s="21" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C109" s="22" t="inlineStr">
@@ -5621,9 +5621,9 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="D109" s="23" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="D109" s="8" t="inlineStr">
+        <is>
+          <t>$200</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
@@ -5631,31 +5631,31 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G109" s="11" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F109" s="24" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G109" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H109" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQRWY1bXUwM1Z4WmNnQlJIdmFnSXJ4T2NMdVZrbHc1WmdCYWN2WVJ0YlpOX1VVWTE5VlBYNEJuQ1Fnd1dUUXR0U0pMamVUQnJpLURQYkMtWnYzaUtzNWd3aWhScDBSbVpjTTljcFBhMURiQ0kzTzlmcy1PT3QtcFZpatIBgAFBVV95cUxQRWY1bXUwM1Z4WmNnQlJIdmFnSXJ4T2NMdVZrbHc1WmdCYWN2WVJ0YlpOX1VVWTE5VlBYNEJuQ1Fnd1dUUXR0U0pMamVUQnJpLURQYkMtWnYzaUtzNWd3aWhScDBSbVpjTTljcFBhMURiQ0kzTzlmcy1PT3QtcFZpag?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE44ZFVoWFRjQTREMXVva2o4S1lQX004N09PbFZNN0RmSkhiRUNxQkJGYldTVEJuSEdLX1g2dHJidmNOV1hNNVQzVEFDUDBZYy0wTXU1dzd2dzN1Wm5LMVhIU0FUUnp5emlsa0FxYjhyZGfSAXBBVV95cUxOOGRVaFhUY0E0RDF1b2tqOEtZUF9NODdPT2xWTTdEZkpIYkVDcUJCRmJXU1RCbkhHS19YNnRyYnZjTldYTTVUM1RBQ1AwWWMtME11NXc3dnczdVpuSzFYSFNBVFJ6eXppbGtBcWI4cmRn?oc=5</t>
         </is>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>Nike Unveils Neuroscience-Based Footwear In The Mind 001 &amp; 002 - Sneaker News</t>
-        </is>
-      </c>
-      <c r="B110" s="35" t="inlineStr">
-        <is>
-          <t>Nike</t>
+          <t>Where To Buy The Air Jordan 1 “All-Star” - Sneaker News</t>
+        </is>
+      </c>
+      <c r="B110" s="26" t="inlineStr">
+        <is>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C110" s="27" t="inlineStr">
@@ -5673,26 +5673,26 @@
           <t>Online, In-Store</t>
         </is>
       </c>
-      <c r="F110" s="18" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="G110" s="19" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
+      <c r="F110" s="28" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="G110" s="29" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
         </is>
       </c>
       <c r="H110" s="20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE9kREhtM1JIVmlkTXNvYzdjbjRnanVYUXloUDZ6U3dJUTdyRUNFenFJYTAwYzlMeG5ycDBMVG9FYldWWGJKU3J1MWFSZHFXRDBLYkVya0hUX2x6SGxoWWfSAV5BVV95cUxPZERIbTNSSFZpZE1zb2M3Y240Z2p1WFF5aFA2elN3SVE3ckVDRXpxSWEwMGM5THhucnAwTFRvRWJXVlhiSlNydTFhUmRxV0QwS2JFcmtIVF9sekhsaFln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1FLW1lUEs3dWMxX0MzZFJaMUF2Wmp1clV3bk92VDNqbDN4LXFHOE0xZkRJYl9VVlRiSzJKZE5RVnlYWVZZaU1xR2IzSDAtR3NycHI3VE02UmJGcHNDWWFkem1nSkRqSTlZQVpFQnZ6czQ0aFdOeG930gF3QVVfeXFMTUUtbWVQSzd1YzFfQzNkUloxQXZaanVyVXduT3ZUM2psM3gtcUc4TTFmREliX1VWVGJLMkpkTlFWeVhZVllpTXFHYjNIMC1Hc3JwcjdUTTZSYkZwc0NZYWR6bWdKRGpJOVlBWkVCdnpzNDRoV054b3c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>ASICS Goes Techy And Low-Profile With The Hypersync - Sneaker News</t>
+          <t>The ASICS GEL-Kayano 14 Pounds The Pavement In “Concrete” - Sneaker News</t>
         </is>
       </c>
       <c r="B111" s="23" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="H111" s="12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTFBwMzZCdVFBOVhyZDdpeWFrMGRKNkpmT0hfNF8xWVc1ektQSk5pNU5adnRVbTh1NEl1emJxdkVndTl0dGoxU3dXdUlaSEZ0TW9DZkxwSkREVXVkVXRBbjJGdU5waGFWblRKcVBIVG82MS1OZ2loWnpVdNIBeEFVX3lxTFBwMzZCdVFBOVhyZDdpeWFrMGRKNkpmT0hfNF8xWVc1ektQSk5pNU5adnRVbTh1NEl1emJxdkVndTl0dGoxU3dXdUlaSEZ0TW9DZkxwSkREVXVkVXRBbjJGdU5waGFWblRKcVBIVG82MS1OZ2loWnpVdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOaGpiQjhhMWd3ZVhQZVJ4N2ozM1JPeHNvYURaa1BGbzhseW9hdFlQNC1ZaWRST3RQTEhJaElqanpVRldWVzBVLVd5ZUo1RW0tcFliQXJWdVVkbi13NlVMRDJ2aUI3eGxGY2w1TlhVVTYtU0ZWekRSMEtVa1ZNbEhXV0tqMktlckZMaUNqLVh3WUU3Y2fSAZMBQVVfeXFMTmhqYkI4YTFnd2VYUGVSeDdqMzNST3hzb2FEWmtQRm84bHlvYXRZUDQtWWlkUk90UExISWhJamp6VUZXVlcwVS1XeWVKNUVtLXBZYkFyVnVVZG4tdzZVTEQydmlCN3hsRmNsNU5YVVU2LVNGVnpEUjBLVWtWTWxIV1dLajJLZXJGTGlDai1Yd1lFN2Nn?oc=5</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7073,7 +7073,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  07:09 AM</t>
+          <t>📊  SNEAKER TRACKER — SUMMARY   ·   March 15, 2026  07:12 AM</t>
         </is>
       </c>
     </row>
@@ -7114,11 +7114,11 @@
         <v>2</v>
       </c>
       <c r="C5" s="59" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5" s="60" t="inlineStr">
         <is>
-          <t>$161</t>
+          <t>$156</t>
         </is>
       </c>
     </row>
@@ -7158,7 +7158,7 @@
         </is>
       </c>
       <c r="B9" s="63" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
@@ -7167,7 +7167,7 @@
       </c>
       <c r="D9" s="46" t="inlineStr">
         <is>
-          <t>$134</t>
+          <t>$132</t>
         </is>
       </c>
     </row>
@@ -7178,7 +7178,7 @@
         </is>
       </c>
       <c r="B10" s="65" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
@@ -7187,7 +7187,7 @@
       </c>
       <c r="D10" s="43" t="inlineStr">
         <is>
-          <t>$186</t>
+          <t>$176</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7198,7 @@
         </is>
       </c>
       <c r="B11" s="63" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="46" t="inlineStr">
         <is>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="B13" s="63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
@@ -7274,15 +7274,15 @@
     <row r="15">
       <c r="A15" s="66" t="inlineStr">
         <is>
-          <t>ASICS</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="B15" s="63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>2.7 / 5</t>
+        <v>2</v>
+      </c>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>2.0 / 5</t>
         </is>
       </c>
       <c r="D15" s="67" t="inlineStr">
@@ -7311,251 +7311,271 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="55" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="66" t="inlineStr">
+        <is>
+          <t>ASICS</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>3.0 / 5</t>
+        </is>
+      </c>
+      <c r="D17" s="67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="55" t="inlineStr">
         <is>
           <t>🔥  HYPE DISTRIBUTION</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="61" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="61" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B19" s="61" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C19" s="61" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="D19" s="61" t="inlineStr">
+      <c r="D20" s="61" t="inlineStr">
         <is>
           <t>% of Total</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="46" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>★☆☆☆☆  1/5</t>
         </is>
       </c>
-      <c r="B20" s="73" t="inlineStr">
+      <c r="B21" s="73" t="inlineStr">
         <is>
           <t>⚪ General Release</t>
         </is>
       </c>
-      <c r="C20" s="63" t="n">
-        <v>13</v>
-      </c>
-      <c r="D20" s="67" t="inlineStr">
+      <c r="C21" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="D21" s="67" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>★★☆☆☆  2/5</t>
+        </is>
+      </c>
+      <c r="B22" s="74" t="inlineStr">
+        <is>
+          <t>🟡 Popular</t>
+        </is>
+      </c>
+      <c r="C22" s="65" t="n">
+        <v>15</v>
+      </c>
+      <c r="D22" s="71" t="inlineStr">
+        <is>
+          <t>11%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>★★★☆☆  3/5</t>
+        </is>
+      </c>
+      <c r="B23" s="75" t="inlineStr">
+        <is>
+          <t>🟠 Hyped</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="n">
+        <v>58</v>
+      </c>
+      <c r="D23" s="67" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>★★★★☆  4/5</t>
+        </is>
+      </c>
+      <c r="B24" s="76" t="inlineStr">
+        <is>
+          <t>🔴 Limited</t>
+        </is>
+      </c>
+      <c r="C24" s="65" t="n">
+        <v>38</v>
+      </c>
+      <c r="D24" s="71" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>★★★★★  5/5</t>
+        </is>
+      </c>
+      <c r="B25" s="77" t="inlineStr">
+        <is>
+          <t>🟣 Grail</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="67" t="inlineStr">
         <is>
           <t>9%</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="34" t="inlineStr">
-        <is>
-          <t>★★☆☆☆  2/5</t>
-        </is>
-      </c>
-      <c r="B21" s="74" t="inlineStr">
-        <is>
-          <t>🟡 Popular</t>
-        </is>
-      </c>
-      <c r="C21" s="65" t="n">
-        <v>13</v>
-      </c>
-      <c r="D21" s="71" t="inlineStr">
-        <is>
-          <t>9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>★★★☆☆  3/5</t>
-        </is>
-      </c>
-      <c r="B22" s="75" t="inlineStr">
-        <is>
-          <t>🟠 Hyped</t>
-        </is>
-      </c>
-      <c r="C22" s="63" t="n">
-        <v>64</v>
-      </c>
-      <c r="D22" s="67" t="inlineStr">
-        <is>
-          <t>47%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>★★★★☆  4/5</t>
-        </is>
-      </c>
-      <c r="B23" s="76" t="inlineStr">
-        <is>
-          <t>🔴 Limited</t>
-        </is>
-      </c>
-      <c r="C23" s="65" t="n">
-        <v>34</v>
-      </c>
-      <c r="D23" s="71" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="39" t="inlineStr">
-        <is>
-          <t>★★★★★  5/5</t>
-        </is>
-      </c>
-      <c r="B24" s="77" t="inlineStr">
-        <is>
-          <t>🟣 Grail</t>
-        </is>
-      </c>
-      <c r="C24" s="63" t="n">
-        <v>13</v>
-      </c>
-      <c r="D24" s="67" t="inlineStr">
-        <is>
-          <t>9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="55" t="inlineStr">
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="55" t="inlineStr">
         <is>
           <t>🌐  SOURCE BREAKDOWN</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="61" t="inlineStr">
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="61" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B27" s="61" t="inlineStr">
+      <c r="B28" s="61" t="inlineStr">
         <is>
           <t>Releases</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="78" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="78" t="inlineStr">
         <is>
           <t>SneakerNews</t>
         </is>
       </c>
-      <c r="B28" s="63" t="n">
+      <c r="B29" s="63" t="n">
         <v>107</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="79" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="79" t="inlineStr">
         <is>
           <t>KicksOnFire</t>
         </is>
       </c>
-      <c r="B29" s="65" t="n">
+      <c r="B30" s="65" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="78" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="78" t="inlineStr">
         <is>
           <t>SoleCollector</t>
         </is>
       </c>
-      <c r="B30" s="63" t="n">
+      <c r="B31" s="63" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="79" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="79" t="inlineStr">
         <is>
           <t>SneakerBarDetroit</t>
         </is>
       </c>
-      <c r="B31" s="65" t="n">
+      <c r="B32" s="65" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="55" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="55" t="inlineStr">
         <is>
           <t>🛍️  TOP SALE METHODS</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="61" t="inlineStr">
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="61" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B34" s="61" t="inlineStr">
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="80" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="80" t="inlineStr">
         <is>
           <t>Online</t>
         </is>
       </c>
-      <c r="B35" s="67" t="n">
+      <c r="B36" s="67" t="n">
         <v>136</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="81" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="81" t="inlineStr">
         <is>
           <t>In-Store</t>
         </is>
       </c>
-      <c r="B36" s="71" t="n">
+      <c r="B37" s="71" t="n">
         <v>135</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="80" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="80" t="inlineStr">
         <is>
           <t>Raffle</t>
         </is>
       </c>
-      <c r="B37" s="67" t="n">
+      <c r="B38" s="67" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-19 07:53 UTC]
</commit_message>
<xml_diff>
--- a/reports/sneaker_releases.xlsx
+++ b/reports/sneaker_releases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Releases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="All Releases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="High Hype Alerts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -686,7 +686,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-19 07:46 UTC</t>
+          <t>Generated: 2026-03-19 07:53 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-03-19 08:22 UTC]
</commit_message>
<xml_diff>
--- a/reports/sneaker_releases.xlsx
+++ b/reports/sneaker_releases.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$1:$J$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Releases'!$A$1:$K$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode=""/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -125,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -143,6 +149,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -172,6 +181,9 @@
     <xf numFmtId="167" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -187,12 +199,15 @@
     <xf numFmtId="167" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -560,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -573,6 +588,7 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -626,6 +642,11 @@
           <t>Hype Level</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -666,6 +687,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -706,6 +732,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -746,6 +777,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -786,6 +822,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -826,6 +867,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -866,6 +912,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -906,6 +957,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -946,6 +1002,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -986,6 +1047,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1026,6 +1092,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1066,6 +1137,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1106,6 +1182,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1138,12 +1219,17 @@
         <v>215</v>
       </c>
       <c r="H14" s="6" t="n"/>
-      <c r="I14" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I14" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1186,6 +1272,11 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1218,12 +1309,17 @@
         <v>250</v>
       </c>
       <c r="H16" s="6" t="n"/>
-      <c r="I16" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I16" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1258,12 +1354,17 @@
         <v>1005</v>
       </c>
       <c r="H17" s="6" t="n"/>
-      <c r="I17" s="9" t="n">
+      <c r="I17" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="J17" s="11" t="inlineStr">
         <is>
           <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1306,6 +1407,11 @@
           <t>LOW</t>
         </is>
       </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1338,12 +1444,17 @@
         <v>120</v>
       </c>
       <c r="H19" s="6" t="n"/>
-      <c r="I19" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I19" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1489,17 @@
         <v>200</v>
       </c>
       <c r="H20" s="6" t="n"/>
-      <c r="I20" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I20" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1418,12 +1534,17 @@
         <v>120</v>
       </c>
       <c r="H21" s="6" t="n"/>
-      <c r="I21" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I21" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -1458,12 +1579,17 @@
         <v>130</v>
       </c>
       <c r="H22" s="6" t="n"/>
-      <c r="I22" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I22" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1624,17 @@
         <v>200</v>
       </c>
       <c r="H23" s="6" t="n"/>
-      <c r="I23" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I23" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -1538,12 +1669,17 @@
         <v>210</v>
       </c>
       <c r="H24" s="6" t="n"/>
-      <c r="I24" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I24" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1586,6 +1722,11 @@
           <t>LOW</t>
         </is>
       </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1626,6 +1767,11 @@
           <t>LOW</t>
         </is>
       </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1666,6 +1812,11 @@
           <t>LOW</t>
         </is>
       </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1698,12 +1849,17 @@
         <v>200</v>
       </c>
       <c r="H28" s="6" t="n"/>
-      <c r="I28" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I28" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -1738,12 +1894,17 @@
         <v>150</v>
       </c>
       <c r="H29" s="6" t="n"/>
-      <c r="I29" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I29" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1939,17 @@
         <v>190</v>
       </c>
       <c r="H30" s="6" t="n"/>
-      <c r="I30" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I30" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -1826,1165 +1992,1422 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="12" t="n">
         <v>46108</v>
       </c>
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C32" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G32" s="14" t="n">
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="n">
         <v>240</v>
       </c>
-      <c r="H32" s="15" t="n"/>
-      <c r="I32" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n">
+      <c r="A33" s="12" t="n">
         <v>46108</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="n">
         <v>240</v>
       </c>
-      <c r="H33" s="15" t="n"/>
-      <c r="I33" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J33" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H33" s="16" t="n"/>
+      <c r="I33" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n">
+      <c r="A34" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="n">
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="n">
         <v>230</v>
       </c>
-      <c r="H34" s="15" t="n"/>
-      <c r="I34" s="9" t="n">
+      <c r="H34" s="16" t="n"/>
+      <c r="I34" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="J34" s="10" t="inlineStr">
+      <c r="J34" s="11" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
+      <c r="A35" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="n">
         <v>215</v>
       </c>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J35" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H35" s="16" t="n"/>
+      <c r="I35" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B36" s="12" t="n">
+      <c r="B36" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C36" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>Nike GT Future “Swooshman”</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="n">
         <v>190</v>
       </c>
-      <c r="H36" s="15" t="n"/>
-      <c r="I36" s="12" t="n">
+      <c r="H36" s="16" t="n"/>
+      <c r="I36" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="J36" s="13" t="inlineStr">
+      <c r="J36" s="14" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n">
+      <c r="A37" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B37" s="12" t="n">
+      <c r="B37" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C37" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G37" s="14" t="n">
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="n">
         <v>190</v>
       </c>
-      <c r="H37" s="15" t="n"/>
-      <c r="I37" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H37" s="16" t="n"/>
+      <c r="I37" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B38" s="12" t="n">
+      <c r="B38" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C38" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="15" t="n"/>
-      <c r="I38" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J38" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="n"/>
+      <c r="H38" s="16" t="n"/>
+      <c r="I38" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K38" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n">
+      <c r="A39" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B39" s="12" t="n">
+      <c r="B39" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C39" s="14" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>adidas BadBo 1.0 “Rise”</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="n">
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="n">
         <v>160</v>
       </c>
-      <c r="H39" s="15" t="n"/>
-      <c r="I39" s="12" t="n">
+      <c r="H39" s="16" t="n"/>
+      <c r="I39" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="J39" s="13" t="inlineStr">
+      <c r="J39" s="14" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
+      <c r="K39" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n">
+      <c r="A40" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B40" s="12" t="n">
+      <c r="B40" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G40" s="14" t="n">
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="n">
         <v>162</v>
       </c>
-      <c r="H40" s="15" t="n"/>
-      <c r="I40" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H40" s="16" t="n"/>
+      <c r="I40" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K40" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n">
+      <c r="A41" s="12" t="n">
         <v>46111</v>
       </c>
-      <c r="B41" s="12" t="n">
+      <c r="B41" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>Nike GT Future “Galaxy Aura”</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F41" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G41" s="14" t="n">
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="n">
         <v>210</v>
       </c>
-      <c r="H41" s="15" t="n"/>
-      <c r="I41" s="12" t="n">
+      <c r="H41" s="16" t="n"/>
+      <c r="I41" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="J41" s="13" t="inlineStr">
+      <c r="J41" s="14" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K41" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n">
+      <c r="A42" s="12" t="n">
         <v>46112</v>
       </c>
-      <c r="B42" s="12" t="n">
+      <c r="B42" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>Jordan Jumpman Pro “Black Concord”</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G42" s="14" t="n">
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="n">
         <v>145</v>
       </c>
-      <c r="H42" s="15" t="n"/>
-      <c r="I42" s="12" t="n">
+      <c r="H42" s="16" t="n"/>
+      <c r="I42" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="J42" s="13" t="inlineStr">
+      <c r="J42" s="14" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K42" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
+      <c r="A43" s="12" t="n">
         <v>46112</v>
       </c>
-      <c r="B43" s="12" t="n">
+      <c r="B43" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F43" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G43" s="14" t="n">
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="n">
         <v>130</v>
       </c>
-      <c r="H43" s="15" t="n"/>
-      <c r="I43" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J43" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H43" s="16" t="n"/>
+      <c r="I43" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K43" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n">
+      <c r="A44" s="12" t="n">
         <v>46113</v>
       </c>
-      <c r="B44" s="12" t="n">
+      <c r="B44" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>Nike Sabrina 3 “What The”</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G44" s="14" t="n">
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="n">
         <v>145</v>
       </c>
-      <c r="H44" s="15" t="n"/>
-      <c r="I44" s="12" t="n">
+      <c r="H44" s="16" t="n"/>
+      <c r="I44" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="J44" s="13" t="inlineStr">
+      <c r="J44" s="14" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K44" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n">
+      <c r="A45" s="12" t="n">
         <v>46114</v>
       </c>
-      <c r="B45" s="12" t="n">
+      <c r="B45" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Nike Mind 001 “Geode Teal”</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G45" s="14" t="n">
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="n">
         <v>95</v>
       </c>
-      <c r="H45" s="15" t="n"/>
-      <c r="I45" s="12" t="n">
+      <c r="H45" s="16" t="n"/>
+      <c r="I45" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="J45" s="13" t="inlineStr">
+      <c r="J45" s="14" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="K45" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="n">
+      <c r="A46" s="18" t="n">
         <v>46115</v>
       </c>
-      <c r="B46" s="17" t="n">
+      <c r="B46" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="C46" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
+        <is>
+          <t>Converse</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>Converse SHAI 001 “Camo”</t>
+        </is>
+      </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G46" s="21" t="n">
+        <v>130</v>
+      </c>
+      <c r="H46" s="22" t="n"/>
+      <c r="I46" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J46" s="20" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B47" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr">
         <is>
           <t>Fragment x Nike Air Liquid Max</t>
         </is>
       </c>
-      <c r="E46" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F46" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G46" s="19" t="n">
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F47" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G47" s="21" t="n">
         <v>225</v>
       </c>
-      <c r="H46" s="20" t="n"/>
-      <c r="I46" s="17" t="n">
+      <c r="H47" s="22" t="n"/>
+      <c r="I47" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="J46" s="18" t="inlineStr">
+      <c r="J47" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="16" t="n">
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="n">
         <v>46115</v>
       </c>
-      <c r="B47" s="17" t="n">
+      <c r="B48" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D47" s="18" t="inlineStr">
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F47" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G47" s="19" t="n">
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F48" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G48" s="21" t="n">
         <v>235</v>
       </c>
-      <c r="H47" s="20" t="n"/>
-      <c r="I47" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J47" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="n">
+      <c r="H48" s="22" t="n"/>
+      <c r="I48" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
         <v>46116</v>
       </c>
-      <c r="B48" s="17" t="n">
+      <c r="B49" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="C49" s="20" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D48" s="18" t="inlineStr">
+      <c r="D49" s="20" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
-      <c r="E48" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F48" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G48" s="19" t="n">
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F49" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G49" s="21" t="n">
         <v>205</v>
       </c>
-      <c r="H48" s="20" t="n"/>
-      <c r="I48" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J48" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="16" t="n">
+      <c r="H49" s="22" t="n"/>
+      <c r="I49" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K49" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="n">
         <v>46122</v>
       </c>
-      <c r="B49" s="17" t="n">
+      <c r="B50" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
         <is>
           <t>Nike Ja 3 “Jurassic Park”</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G49" s="19" t="n">
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F50" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G50" s="21" t="n">
         <v>135</v>
       </c>
-      <c r="H49" s="20" t="n"/>
-      <c r="I49" s="17" t="n">
+      <c r="H50" s="22" t="n"/>
+      <c r="I50" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J49" s="18" t="inlineStr">
+      <c r="J50" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="16" t="n">
+      <c r="K50" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="n">
         <v>46122</v>
       </c>
-      <c r="B50" s="17" t="n">
+      <c r="B51" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D50" s="18" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="inlineStr">
         <is>
           <t>Jurassic Park x Nike Ja 3 “Raptor”</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G50" s="19" t="n">
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F51" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G51" s="21" t="n">
         <v>135</v>
       </c>
-      <c r="H50" s="20" t="n"/>
-      <c r="I50" s="17" t="n">
+      <c r="H51" s="22" t="n"/>
+      <c r="I51" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J50" s="18" t="inlineStr">
+      <c r="J51" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="16" t="n">
+      <c r="K51" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="n">
         <v>46122</v>
       </c>
-      <c r="B51" s="17" t="n">
+      <c r="B52" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D51" s="18" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>Jurassic Park x Nike Ja 3 “Explorer”</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G51" s="19" t="n">
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F52" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G52" s="21" t="n">
         <v>135</v>
       </c>
-      <c r="H51" s="20" t="n"/>
-      <c r="I51" s="17" t="n">
+      <c r="H52" s="22" t="n"/>
+      <c r="I52" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J51" s="18" t="inlineStr">
+      <c r="J52" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="n">
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="n">
         <v>46123</v>
       </c>
-      <c r="B52" s="17" t="n">
+      <c r="B53" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
         <is>
           <t>Nike Air Max Uptempo 95 “Derek Fisher”</t>
         </is>
       </c>
-      <c r="E52" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G52" s="19" t="n">
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G53" s="21" t="n">
         <v>170</v>
       </c>
-      <c r="H52" s="20" t="n"/>
-      <c r="I52" s="17" t="n">
+      <c r="H53" s="22" t="n"/>
+      <c r="I53" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J52" s="18" t="inlineStr">
+      <c r="J53" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="n">
+      <c r="K53" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="n">
         <v>46123</v>
       </c>
-      <c r="B53" s="17" t="n">
+      <c r="B54" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="C53" s="18" t="inlineStr">
+      <c r="C54" s="20" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D53" s="18" t="inlineStr">
+      <c r="D54" s="20" t="inlineStr">
         <is>
           <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G53" s="19" t="n">
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F54" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G54" s="21" t="n">
         <v>185</v>
       </c>
-      <c r="H53" s="20" t="n"/>
-      <c r="I53" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J53" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="16" t="n">
+      <c r="H54" s="22" t="n"/>
+      <c r="I54" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K54" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="n">
         <v>46124</v>
       </c>
-      <c r="B54" s="17" t="n">
+      <c r="B55" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="C54" s="18" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="D54" s="18" t="inlineStr">
+      <c r="D55" s="20" t="inlineStr">
         <is>
           <t>adidas Anthony Edwards 2 “Lime Burst”</t>
         </is>
       </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F54" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G54" s="19" t="n">
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G55" s="21" t="n">
         <v>130</v>
       </c>
-      <c r="H54" s="20" t="n"/>
-      <c r="I54" s="17" t="n">
+      <c r="H55" s="22" t="n"/>
+      <c r="I55" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J54" s="18" t="inlineStr">
+      <c r="J55" s="20" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="n">
+      <c r="K55" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="n">
         <v>46125</v>
       </c>
-      <c r="B55" s="17" t="n">
+      <c r="B56" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D55" s="18" t="inlineStr">
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
         <is>
           <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F55" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G55" s="20" t="n"/>
-      <c r="H55" s="20" t="n"/>
-      <c r="I55" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J55" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="16" t="n">
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F56" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G56" s="22" t="n"/>
+      <c r="H56" s="22" t="n"/>
+      <c r="I56" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K56" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="n">
         <v>46125</v>
       </c>
-      <c r="B56" s="17" t="n">
+      <c r="B57" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
         <is>
           <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G56" s="19" t="n">
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="n">
         <v>220</v>
       </c>
-      <c r="H56" s="20" t="n"/>
-      <c r="I56" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J56" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="n">
+      <c r="H57" s="22" t="n"/>
+      <c r="I57" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K57" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="18" t="n">
         <v>46128</v>
       </c>
-      <c r="B57" s="17" t="n">
+      <c r="B58" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="C57" s="18" t="inlineStr">
+      <c r="C58" s="20" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="D57" s="18" t="inlineStr">
+      <c r="D58" s="20" t="inlineStr">
         <is>
           <t>adidas Harden Vol. 10 “Lucid Aquamarine”</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G57" s="19" t="n">
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F58" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G58" s="21" t="n">
         <v>160</v>
       </c>
-      <c r="H57" s="20" t="n"/>
-      <c r="I57" s="17" t="n">
+      <c r="H58" s="22" t="n"/>
+      <c r="I58" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J57" s="18" t="inlineStr">
+      <c r="J58" s="20" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="16" t="n">
+      <c r="K58" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="18" t="n">
         <v>46129</v>
       </c>
-      <c r="B58" s="17" t="n">
+      <c r="B59" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="C58" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
-      <c r="E58" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F58" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G58" s="19" t="n">
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G59" s="21" t="n">
         <v>240</v>
       </c>
-      <c r="H58" s="20" t="n"/>
-      <c r="I58" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J58" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="16" t="n">
+      <c r="H59" s="22" t="n"/>
+      <c r="I59" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K59" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="18" t="n">
         <v>46130</v>
       </c>
-      <c r="B59" s="17" t="n">
+      <c r="B60" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="C59" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
         <is>
           <t>Nike Cryoshot Mercurial Vapor R9 “Varsity Royal”</t>
         </is>
       </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F59" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G59" s="19" t="n">
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G60" s="21" t="n">
         <v>210</v>
       </c>
-      <c r="H59" s="20" t="n"/>
-      <c r="I59" s="17" t="n">
+      <c r="H60" s="22" t="n"/>
+      <c r="I60" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J59" s="18" t="inlineStr">
+      <c r="J60" s="20" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="16" t="n">
+      <c r="K60" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="18" t="n">
         <v>46130</v>
       </c>
-      <c r="B60" s="17" t="n">
+      <c r="B61" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="C60" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D60" s="18" t="inlineStr">
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G60" s="19" t="n">
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G61" s="21" t="n">
         <v>240</v>
       </c>
-      <c r="H60" s="20" t="n"/>
-      <c r="I60" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J60" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H61" s="22" t="n"/>
+      <c r="I61" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K61" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J60"/>
+  <autoFilter ref="A1:K61"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId60"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2995,7 +3418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3008,6 +3431,7 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3061,6 +3485,11 @@
           <t>Hype Level</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3093,12 +3522,17 @@
         <v>215</v>
       </c>
       <c r="H2" s="6" t="n"/>
-      <c r="I2" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J2" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I2" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3133,12 +3567,17 @@
         <v>250</v>
       </c>
       <c r="H3" s="6" t="n"/>
-      <c r="I3" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I3" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3173,12 +3612,17 @@
         <v>1005</v>
       </c>
       <c r="H4" s="6" t="n"/>
-      <c r="I4" s="9" t="n">
+      <c r="I4" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="10" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3213,12 +3657,17 @@
         <v>120</v>
       </c>
       <c r="H5" s="6" t="n"/>
-      <c r="I5" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I5" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3702,17 @@
         <v>200</v>
       </c>
       <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I6" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3747,17 @@
         <v>120</v>
       </c>
       <c r="H7" s="6" t="n"/>
-      <c r="I7" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I7" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -3333,12 +3792,17 @@
         <v>130</v>
       </c>
       <c r="H8" s="6" t="n"/>
-      <c r="I8" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -3373,12 +3837,17 @@
         <v>200</v>
       </c>
       <c r="H9" s="6" t="n"/>
-      <c r="I9" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I9" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -3413,12 +3882,17 @@
         <v>210</v>
       </c>
       <c r="H10" s="6" t="n"/>
-      <c r="I10" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I10" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3453,12 +3927,17 @@
         <v>200</v>
       </c>
       <c r="H11" s="6" t="n"/>
-      <c r="I11" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I11" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
@@ -3493,12 +3972,17 @@
         <v>150</v>
       </c>
       <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I12" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
@@ -3533,612 +4017,721 @@
         <v>190</v>
       </c>
       <c r="H13" s="6" t="n"/>
-      <c r="I13" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="I13" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="12" t="n">
         <v>46108</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue” 2026</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="n">
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="n">
         <v>240</v>
       </c>
-      <c r="H14" s="15" t="n"/>
-      <c r="I14" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H14" s="16" t="n"/>
+      <c r="I14" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K14" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="12" t="n">
         <v>46108</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “University Blue”</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="n">
         <v>240</v>
       </c>
-      <c r="H15" s="15" t="n"/>
-      <c r="I15" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H15" s="16" t="n"/>
+      <c r="I15" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Virgil Abloh Archive x Air Jordan 1 High OG “Alaska”</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="n">
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="n">
         <v>230</v>
       </c>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="9" t="n">
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Spring is in the Air”</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="n">
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="n">
         <v>215</v>
       </c>
-      <c r="H17" s="15" t="n"/>
-      <c r="I17" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Nike Air Max 95 “Pink Foam” 2026</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="n">
         <v>190</v>
       </c>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H18" s="16" t="n"/>
+      <c r="I18" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K18" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low “Brew &amp; Biscuits”</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F19" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="15" t="n"/>
-      <c r="I19" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K19" s="17" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="12" t="n">
         <v>46109</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>LEGO x Nike Air Max 95 (GS)</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G20" s="14" t="n">
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="n">
         <v>162</v>
       </c>
-      <c r="H20" s="15" t="n"/>
-      <c r="I20" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="12" t="n">
         <v>46112</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>NOTE Manchester x Nike SB Dunk Low</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="n">
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="n">
         <v>130</v>
       </c>
-      <c r="H21" s="15" t="n"/>
-      <c r="I21" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H21" s="16" t="n"/>
+      <c r="I21" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="n">
+      <c r="A22" s="18" t="n">
         <v>46115</v>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Nike LeBron 23 “Good Intentions”</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G22" s="19" t="n">
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="n">
         <v>235</v>
       </c>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H22" s="22" t="n"/>
+      <c r="I22" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="n">
+      <c r="A23" s="18" t="n">
         <v>46116</v>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Air Jordan 3 “Orange Citrus” 2026</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G23" s="19" t="n">
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" s="21" t="n">
         <v>205</v>
       </c>
-      <c r="H23" s="20" t="n"/>
-      <c r="I23" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H23" s="22" t="n"/>
+      <c r="I23" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K23" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="n">
+      <c r="A24" s="18" t="n">
         <v>46123</v>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>Air Jordan 1 High OG “Flight Club”</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="n">
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="n">
         <v>185</v>
       </c>
-      <c r="H24" s="20" t="n"/>
-      <c r="I24" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H24" s="22" t="n"/>
+      <c r="I24" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="n">
+      <c r="A25" s="18" t="n">
         <v>46125</v>
       </c>
-      <c r="B25" s="17" t="n">
+      <c r="B25" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>Nike Kobe 11 Elite Protro “Mamba Out”</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G25" s="20" t="n"/>
-      <c r="H25" s="20" t="n"/>
-      <c r="I25" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="22" t="n"/>
+      <c r="I25" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K25" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="n">
+      <c r="A26" s="18" t="n">
         <v>46125</v>
       </c>
-      <c r="B26" s="17" t="n">
+      <c r="B26" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Nike Kobe 11 EM Protro “Mamba Out”</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="n">
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="n">
         <v>220</v>
       </c>
-      <c r="H26" s="20" t="n"/>
-      <c r="I26" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H26" s="22" t="n"/>
+      <c r="I26" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>SneakerBarDetroit</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="n">
+      <c r="A27" s="18" t="n">
         <v>46129</v>
       </c>
-      <c r="B27" s="17" t="n">
+      <c r="B27" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Voltage”</t>
         </is>
       </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G27" s="19" t="n">
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" s="21" t="n">
         <v>240</v>
       </c>
-      <c r="H27" s="20" t="n"/>
-      <c r="I27" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H27" s="22" t="n"/>
+      <c r="I27" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="n">
+      <c r="A28" s="18" t="n">
         <v>46130</v>
       </c>
-      <c r="B28" s="17" t="n">
+      <c r="B28" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G28" s="19" t="n">
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G28" s="21" t="n">
         <v>240</v>
       </c>
-      <c r="H28" s="20" t="n"/>
-      <c r="I28" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="H28" s="22" t="n"/>
+      <c r="I28" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>SneakerFiles</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4149,7 +4742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4158,143 +4751,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>Sneaker Release Report Summary</t>
         </is>
       </c>
-      <c r="C1" s="22" t="inlineStr">
-        <is>
-          <t>Generated: 2026-03-19 08:16 UTC</t>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>Generated: 2026-03-19 08:22 UTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Total releases tracked: 59</t>
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Total releases tracked: 60</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Releases by Brand</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="n">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n">
         <v>44</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Adidas</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="25" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="B7" s="25" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Converse</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Releases by Urgency</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>URGENT (within 7 days)</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B11" s="27" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>UPCOMING (8-14 days)</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B12" s="28" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>LATER (15-30 days)</t>
         </is>
       </c>
-      <c r="B12" s="26" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="B13" s="29" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Releases by Hype Level</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>EXTREME</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B16" s="25" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="n">
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B18" s="25" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n">
-        <v>7</v>
+      <c r="B19" s="25" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>